<commit_message>
feat: add topological guard for 'I', clean blank dataset, and update docs (acc 87.08%)
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-10 16:24:31 | ตรวจทั้งหมด: 3 แผ่น | รวม 60 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-10 17:45:39 | ตรวจทั้งหมด: 3 แผ่น | รวม 60 ข้อ</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>85.75%</t>
+          <t>87.08%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>33 ข้อ</t>
+          <t>24 ข้อ</t>
         </is>
       </c>
     </row>
@@ -765,12 +765,12 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.991</t>
+          <t>0.993</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>6 ข้อ</t>
+          <t>3 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,17 +793,17 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>71.00%</t>
+          <t>74.75%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.960</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>17 ข้อ</t>
+          <t>15 ข้อ</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>92.25%</t>
+          <t>92.50%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.986</t>
+          <t>0.989</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>10 ข้อ</t>
+          <t>6 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -913,14 +913,14 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>THB-QUICK-BROWN-FGX-</t>
+          <t>THE-QGICK-BROWN-FMX-</t>
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.985</v>
+        <v>1</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.84</v>
+        <v>0.999</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -939,18 +939,18 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-PQM-</t>
+          <t>JUMPS-OVERSLAZY-CQML</t>
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.972</v>
+        <v>0.998</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.448</v>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.966</v>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -969,10 +969,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.998</v>
+        <v>0.991</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.959</v>
+        <v>0.85</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -991,14 +991,14 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DNZEN-LIQUOR-JV</t>
+          <t>FIVE-DNZEN-LIQUOR-ZH</t>
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.998</v>
+        <v>0.99</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.968</v>
+        <v>0.8139999999999999</v>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
@@ -1043,14 +1043,14 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VNW-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.991</v>
+        <v>0.996</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.823</v>
+        <v>0.915</v>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
@@ -1073,10 +1073,10 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
@@ -1121,18 +1121,18 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MACHJNE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.998</v>
+        <v>0.979</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.582</v>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1147,18 +1147,18 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NEJWORKM</t>
+          <t>DEEP-NDURAL-NETWORKM</t>
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.979</v>
+        <v>0.987</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.6830000000000001</v>
-      </c>
-      <c r="F11" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.822</v>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1173,18 +1173,18 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETECT-OA</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.988</v>
+        <v>0.995</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.769</v>
-      </c>
-      <c r="F12" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1199,18 +1199,18 @@
       </c>
       <c r="C13" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENCV-RQBOT-</t>
+          <t>PYTHON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.969</v>
+        <v>1</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.6840000000000001</v>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.999</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1251,14 +1251,14 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTINN-</t>
+          <t>ACCURATE-PREDICTIQN-</t>
         </is>
       </c>
       <c r="D15" s="19" t="n">
         <v>0.998</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.96</v>
+        <v>0.952</v>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
@@ -1277,18 +1277,18 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>ARTIFJCIAL-SYSTEM-OZ</t>
+          <t>ARTIFJCIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.984</v>
+        <v>0.979</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F16" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6860000000000001</v>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.992</v>
+        <v>1</v>
       </c>
       <c r="F17" s="16" t="inlineStr">
         <is>
@@ -1329,14 +1329,14 @@
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>KNNWLEDGE-IS-POWBR--</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.998</v>
+        <v>0.999</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.972</v>
+        <v>0.99</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
@@ -1359,14 +1359,14 @@
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.978</v>
+        <v>0.997</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.5620000000000001</v>
-      </c>
-      <c r="F19" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1381,14 +1381,14 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SJX-JEM</t>
+          <t>ZERO-ONE-TWO-SJX-GEM</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.989</v>
+        <v>0.959</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.796</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
@@ -1411,10 +1411,10 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.971</v>
+        <v>0.996</v>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
@@ -1433,14 +1433,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>THU-DUIGK-RAOWN-FCX-</t>
+          <t>THP-QUICK-RMOWN-FCX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.945</v>
+        <v>0.967</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.498</v>
+        <v>0.632</v>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
@@ -1459,18 +1459,18 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-CNA-</t>
+          <t>JUMPS-OVER-LAZY-FQG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.968</v>
+        <v>0.994</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="F23" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.919</v>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1485,14 +1485,14 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-COX-WLTH-TEA</t>
+          <t>PACK-MV-GOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.966</v>
+        <v>0.975</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.748</v>
+        <v>0.704</v>
       </c>
       <c r="F24" s="20" t="inlineStr">
         <is>
@@ -1511,18 +1511,18 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>BIVF-POZFNWLLOUQR-JV</t>
+          <t>FIVF-GOZFNWLIQUQR-JV</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.971</v>
+        <v>0.985</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.731</v>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1537,14 +1537,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHLNX-GF-BLACK-GFM-</t>
+          <t>SPHLNX-CF-RLACK-GFM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.968</v>
+        <v>0.953</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.6879999999999999</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
@@ -1563,14 +1563,14 @@
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-GY-VOW-QVICKUY</t>
+          <t>JUDGE-MY-VQW-QVICOLY</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.967</v>
+        <v>0.979</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.654</v>
       </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
@@ -1589,18 +1589,18 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BRJGHT-ZEPHYMS-BLOK-</t>
+          <t>BRLGHT-ZEPHYRS-BLOE-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.983</v>
+        <v>0.971</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.819</v>
-      </c>
-      <c r="F28" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.65</v>
+      </c>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1615,18 +1615,18 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VUGLOM-TEST</t>
+          <t>COMPUTER-VISION-TESC</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.969</v>
+        <v>0.99</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.6860000000000001</v>
-      </c>
-      <c r="F29" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F29" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1641,7 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHLNE-UEA-NJNG-AJ-</t>
+          <t>MACHINE-LEAMNJNG-AJ-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
@@ -1667,14 +1667,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>OFEP-NFUPAU-AFJWQRKX</t>
+          <t>DFEP-NFXBAU-AFTWORKO</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.975</v>
+        <v>0.967</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.715</v>
+        <v>0.555</v>
       </c>
       <c r="F31" s="20" t="inlineStr">
         <is>
@@ -1693,18 +1693,18 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGF-CATA-FEUFCT-CK</t>
+          <t>-MAGE-CATA-RELFCZ-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.955</v>
+        <v>0.993</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.602</v>
-      </c>
-      <c r="F32" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.878</v>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1719,18 +1719,18 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYTHON-OPFYCV-ROBCT-</t>
+          <t>DYTHON-OPFYCV-RORCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.986</v>
+        <v>0.945</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F33" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="F33" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1745,14 +1745,14 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SOART-CCRJBECOGWLZE-</t>
+          <t>SGARS-CCRJRECGGWIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.961</v>
+        <v>0.896</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.681</v>
+        <v>0.498</v>
       </c>
       <c r="F34" s="20" t="inlineStr">
         <is>
@@ -1771,14 +1771,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>QCCURATF--PEDJCOJFA-</t>
+          <t>ACCURATF--AEDJCZJRAK</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.924</v>
+        <v>0.91</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.5669999999999999</v>
+        <v>0.345</v>
       </c>
       <c r="F35" s="20" t="inlineStr">
         <is>
@@ -1797,14 +1797,14 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>XRTUFSCJAL-SYSGEM-GQ</t>
+          <t>XRTIFICJALYSYSTEM-CW</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.916</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.396</v>
+        <v>0.441</v>
       </c>
       <c r="F36" s="20" t="inlineStr">
         <is>
@@ -1823,14 +1823,14 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLG-WORUD-DDLOCME-</t>
+          <t>HELLC-WOPLR-VDLOCMDK</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.957</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.538</v>
       </c>
       <c r="F37" s="20" t="inlineStr">
         <is>
@@ -1849,18 +1849,18 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KWQWL-CCF-US-PNKER--</t>
+          <t>KUQWL-CCE-IS-PQLER-K</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.984</v>
+        <v>0.97</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F38" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.772</v>
+      </c>
+      <c r="F38" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1875,14 +1875,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>FOND-FXTRA-ELNP-GOLW</t>
+          <t>MIND-FXTRA-FINR-GDLO</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.958</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.552</v>
+        <v>0.504</v>
       </c>
       <c r="F39" s="20" t="inlineStr">
         <is>
@@ -1901,18 +1901,18 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZIRQ-NNE-TXG-SLX-TEK</t>
+          <t>ZIRQ-ONE-TXG-SIX-TAH</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.971</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.438</v>
-      </c>
-      <c r="F40" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.848</v>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1927,14 +1927,14 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFSH-JKLMNOEWM-J</t>
+          <t>ABCDEFGHIJKLMNCEWBLZ</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.954</v>
+        <v>0.956</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.786</v>
+        <v>0.622</v>
       </c>
       <c r="F41" s="20" t="inlineStr">
         <is>
@@ -1957,14 +1957,14 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.964</v>
+        <v>0.989</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F42" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F42" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1979,14 +1979,14 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>JUMPS-GVER-LAZY-DOGL</t>
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.965</v>
+        <v>0.957</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.512</v>
       </c>
       <c r="F43" s="20" t="inlineStr">
         <is>
@@ -2005,11 +2005,11 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>DACK-MY-ROX-WITH-TEW</t>
+          <t>PACK-MY-ROX-WITH-TEW</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.993</v>
+        <v>0.992</v>
       </c>
       <c r="E44" s="15" t="n">
         <v>0.85</v>
@@ -2031,14 +2031,14 @@
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>PIVE-DOZEN-LIQUOR-JV</t>
+          <t>FIVE-DOZEN-LIQUOR-JV</t>
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.974</v>
+        <v>0.985</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.681</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="F45" s="20" t="inlineStr">
         <is>
@@ -2057,18 +2057,18 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLGCK-GEM-</t>
+          <t>SPHINX-OF-BLNCK-GEMK</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.989</v>
+        <v>0.985</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.895</v>
-      </c>
-      <c r="F46" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.788</v>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2083,18 +2083,18 @@
       </c>
       <c r="C47" s="18" t="inlineStr">
         <is>
-          <t>JUPGE-MY-VOW-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.987</v>
+        <v>0.999</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.745</v>
-      </c>
-      <c r="F47" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.99</v>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2113,10 +2113,10 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="15" t="n">
         <v>0.999</v>
-      </c>
-      <c r="E48" s="15" t="n">
-        <v>0.991</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
@@ -2135,14 +2135,14 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>CDMPVTFR-VISION-TEST</t>
+          <t>COMPVTFR-VISION-TEST</t>
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.993</v>
+        <v>0.999</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.912</v>
+        <v>0.992</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2165,10 +2165,10 @@
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.921</v>
+        <v>0.997</v>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
@@ -2187,18 +2187,18 @@
       </c>
       <c r="C51" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKK</t>
+          <t>DEEP-NEURAL-NETWORKR</t>
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="F51" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.771</v>
+      </c>
+      <c r="F51" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2213,18 +2213,18 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETECT-OM</t>
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>0.999</v>
+        <v>0.985</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="F52" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.696</v>
+      </c>
+      <c r="F52" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2239,14 +2239,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>PYTHONPDPENWVAROZON-</t>
+          <t>PYTHONBDPENCVEROBON-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.975</v>
+        <v>0.963</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.518</v>
+        <v>0.553</v>
       </c>
       <c r="F53" s="20" t="inlineStr">
         <is>
@@ -2265,14 +2265,14 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>SMART-ORC-RECOGNIZE-</t>
+          <t>SMART-ORC-RECOGNIZEB</t>
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>1</v>
+        <v>0.996</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.999</v>
+        <v>0.93</v>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
@@ -2291,18 +2291,18 @@
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-DREDICGION-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.989</v>
+        <v>1</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.799</v>
-      </c>
-      <c r="F55" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>1</v>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2317,18 +2317,18 @@
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SVSTEM-OK</t>
+          <t>ARTIFICIAL-SVSTEM-OM</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.968</v>
+        <v>0.998</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.369</v>
-      </c>
-      <c r="F56" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.962</v>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2343,18 +2343,18 @@
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCGME-</t>
+          <t>HELLO-DORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.966</v>
+        <v>0.992</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.679</v>
-      </c>
-      <c r="F57" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F57" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2369,14 +2369,14 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-TS-POWER--</t>
+          <t>KNOWLKDGE-IS-POWER-W</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.997</v>
+        <v>0.977</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.947</v>
+        <v>0.863</v>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
@@ -2395,18 +2395,18 @@
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLP</t>
+          <t>FIND-EXTRA-FIND-GOLG</t>
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>0.984</v>
+        <v>0.993</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.752</v>
-      </c>
-      <c r="F59" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.854</v>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2421,14 +2421,14 @@
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TEW</t>
+          <t>ZERO-ONE-TWO-SIX-TEH</t>
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.999</v>
+        <v>0.994</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.981</v>
+        <v>0.909</v>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
@@ -2447,18 +2447,18 @@
       </c>
       <c r="C61" s="18" t="inlineStr">
         <is>
-          <t>ARCDEFGHIJKLMNOPQRSG</t>
+          <t>ARCDEFGHIJKLMNOPQDST</t>
         </is>
       </c>
       <c r="D61" s="19" t="n">
-        <v>0.974</v>
+        <v>0.986</v>
       </c>
       <c r="E61" s="19" t="n">
-        <v>0.787</v>
-      </c>
-      <c r="F61" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: boost accuracy to 92.08%, expand training data to 78 sheets, and organize docs
- Retrain MLP classifier on 78 sheets with 1,176-D hybrid features
- Implement topological rules (B vs R, E vs F, C vs O) and expand border guard
- Benchmark 6 test sheets (2,400 cells) achieving 92.08% overall accuracy
- Restructure project: consolidate slides/scripts into docs/ and clean up artifacts
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -618,10 +618,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="77" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-10 17:45:39 | ตรวจทั้งหมด: 3 แผ่น | รวม 60 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-14 17:27:57 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
         </is>
       </c>
     </row>
@@ -676,27 +676,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>3 แผ่น</t>
+          <t>6 แผ่น</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>60 ข้อ</t>
+          <t>120 ข้อ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>1,200 ตัว</t>
+          <t>2,400 ตัว</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>87.08%</t>
+          <t>92.08%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>24 ข้อ</t>
+          <t>42 ข้อ</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>94.00%</t>
+          <t>97.25%</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.993</t>
+          <t>0.995</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>3 ข้อ</t>
+          <t>4 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>74.75%</t>
+          <t>78.00%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.962</t>
+          <t>0.959</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -826,20 +826,119 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>92.50%</t>
+          <t>95.00%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.989</t>
+          <t>0.993</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>6 ข้อ</t>
+          <t>5 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>96.50%</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>0.995</t>
+        </is>
+      </c>
+      <c r="F14" s="9" t="inlineStr">
+        <is>
+          <t>4 ข้อ</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>92.75%</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>0.987</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>9 ข้อ</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>93.00%</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>0.991</t>
+        </is>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>5 ข้อ</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
         <is>
           <t>English &amp; Tech (ชุดที่ 1)</t>
         </is>
@@ -859,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -913,14 +1012,14 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>THE-QGICK-BROWN-FMX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D2" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.999</v>
+        <v>0.998</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -939,14 +1038,14 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVERSLAZY-CQML</t>
+          <t>JUMPS-OVERALAZY-COG-</t>
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.998</v>
+        <v>0.992</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.966</v>
+        <v>0.848</v>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
@@ -969,10 +1068,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.991</v>
+        <v>1</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -991,14 +1090,14 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DNZEN-LIQUOR-ZH</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.99</v>
+        <v>0.999</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.984</v>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
@@ -1021,10 +1120,10 @@
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.999</v>
+        <v>0.984</v>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
@@ -1043,18 +1142,18 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VOW-QUICKLY</t>
+          <t>JUDGE-MY-VGW-QUICKLY</t>
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.996</v>
+        <v>0.986</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.915</v>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.725</v>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1073,10 +1172,10 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>1</v>
+        <v>0.861</v>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
@@ -1095,18 +1194,18 @@
       </c>
       <c r="C9" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TESJ</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.658</v>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1125,14 +1224,14 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.979</v>
+        <v>0.995</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.908</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1147,14 +1246,14 @@
       </c>
       <c r="C11" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NDURAL-NETWORKM</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.987</v>
+        <v>0.998</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.822</v>
+        <v>0.97</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -1173,14 +1272,14 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OA</t>
+          <t>JMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.995</v>
+        <v>0.999</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.985</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
@@ -1206,7 +1305,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
@@ -1251,14 +1350,14 @@
       </c>
       <c r="C15" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTIQN-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.998</v>
+        <v>1</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.952</v>
+        <v>0.994</v>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
@@ -1281,10 +1380,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.979</v>
+        <v>0.985</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.708</v>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
@@ -1333,14 +1432,14 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.999</v>
+        <v>0.986</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.772</v>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1355,14 +1454,14 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLM</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.997</v>
+        <v>1</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.9399999999999999</v>
+        <v>1</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
@@ -1381,18 +1480,18 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SJX-GEM</t>
+          <t>ZERO-ONE-TWO-SJX-JEM</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.959</v>
+        <v>1</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.6929999999999999</v>
-      </c>
-      <c r="F20" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.997</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1407,14 +1506,14 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPDRSY</t>
+          <t>ABCDEFGHIJKLMNOPMRST</t>
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>1</v>
+        <v>0.994</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.996</v>
+        <v>0.885</v>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
@@ -1433,14 +1532,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>THP-QUICK-RMOWN-FCX-</t>
+          <t>THI-UUICK-PROWN-FCX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.967</v>
+        <v>0.975</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.632</v>
+        <v>0.793</v>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
@@ -1459,18 +1558,18 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-FQG-</t>
+          <t>JUGPS-OVER-LAZY-COG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.994</v>
+        <v>0.952</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.543</v>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1485,18 +1584,18 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MV-GOX-WITH-TEA</t>
+          <t>PACK-MV-COX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.975</v>
+        <v>0.988</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.704</v>
-      </c>
-      <c r="F24" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.908</v>
+      </c>
+      <c r="F24" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1511,18 +1610,18 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>FIVF-GOZFNWLIQUQR-JV</t>
+          <t>EIVF-EOZFNWLIQUQR-JD</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.985</v>
+        <v>0.923</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.531</v>
+      </c>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1537,14 +1636,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHLNX-CF-RLACK-GFM-</t>
+          <t>GPHLNX-CF-BLACK-GFM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.953</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="F26" s="20" t="inlineStr">
         <is>
@@ -1563,14 +1662,14 @@
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VQW-QVICOLY</t>
+          <t>JUDGE-MY-VCW-QVICKLY</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.654</v>
+        <v>0.701</v>
       </c>
       <c r="F27" s="20" t="inlineStr">
         <is>
@@ -1589,18 +1688,18 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BRLGHT-ZEPHYRS-BLOE-</t>
+          <t>BRJGHT-ZEPHYRS-BLOL-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.971</v>
+        <v>0.979</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="F28" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F28" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1615,11 +1714,11 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TESC</t>
+          <t>COMPUTER-VISION-TESE</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.99</v>
+        <v>0.982</v>
       </c>
       <c r="E29" s="19" t="n">
         <v>0.85</v>
@@ -1641,14 +1740,14 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEAMNJNG-AJ-</t>
+          <t>MACHINE-LEANN-NG-AJ-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.967</v>
+        <v>0.97</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.521</v>
+        <v>0.504</v>
       </c>
       <c r="F30" s="20" t="inlineStr">
         <is>
@@ -1667,14 +1766,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DFEP-NFXBAU-AFTWORKO</t>
+          <t>DFEP-NEUPAU-AFTVORKX</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.967</v>
+        <v>0.952</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.555</v>
+        <v>0.548</v>
       </c>
       <c r="F31" s="20" t="inlineStr">
         <is>
@@ -1693,18 +1792,18 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGE-CATA-RELFCZ-CK</t>
+          <t>-MAGF-OATA-EEZFCT-CU</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.993</v>
+        <v>0.95</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.878</v>
-      </c>
-      <c r="F32" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.467</v>
+      </c>
+      <c r="F32" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1719,14 +1818,14 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYTHON-OPFYCV-RORCT-</t>
+          <t>DYTHGN-OPFNCV-BOBCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.945</v>
+        <v>0.977</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="F33" s="20" t="inlineStr">
         <is>
@@ -1745,14 +1844,14 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SGARS-CCRJRECGGWIZE-</t>
+          <t>SFART-CCRXRECCGWIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.896</v>
+        <v>0.925</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.498</v>
+        <v>0.496</v>
       </c>
       <c r="F34" s="20" t="inlineStr">
         <is>
@@ -1771,14 +1870,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>ACCURATF--AEDJCZJRAK</t>
+          <t>ACCURAJF--REDJCZJRA-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.91</v>
+        <v>0.944</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.345</v>
+        <v>0.725</v>
       </c>
       <c r="F35" s="20" t="inlineStr">
         <is>
@@ -1797,14 +1896,14 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>XRTIFICJALYSYSTEM-CW</t>
+          <t>ARTIFICZALXSYSTEM-CV</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.892</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.441</v>
+        <v>0.31</v>
       </c>
       <c r="F36" s="20" t="inlineStr">
         <is>
@@ -1823,18 +1922,18 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLC-WOPLR-VDLOCMDK</t>
+          <t>HELLG-WOFLD-VFLOCME-</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.957</v>
+        <v>0.987</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.538</v>
-      </c>
-      <c r="F37" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.876</v>
+      </c>
+      <c r="F37" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1849,14 +1948,14 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KUQWL-CCE-IS-PQLER-K</t>
+          <t>KWOWL-CCE-IS-POKER--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.97</v>
+        <v>0.965</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.772</v>
+        <v>0.733</v>
       </c>
       <c r="F38" s="20" t="inlineStr">
         <is>
@@ -1875,14 +1974,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>MIND-FXTRA-FINR-GDLO</t>
+          <t>FIND-FXTRA-GINF-GDLC</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.967</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.504</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="F39" s="20" t="inlineStr">
         <is>
@@ -1901,18 +2000,18 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZIRQ-ONE-TXG-SIX-TAH</t>
+          <t>ZJRG-NNE-TXG-SIX-TEN</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.971</v>
+        <v>0.951</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.848</v>
-      </c>
-      <c r="F40" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.404</v>
+      </c>
+      <c r="F40" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1927,18 +2026,18 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNCEWBLZ</t>
+          <t>ABCDEFGHIJKLMNOPGEOT</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.956</v>
+        <v>0.99</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.622</v>
-      </c>
-      <c r="F41" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.907</v>
+      </c>
+      <c r="F41" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1953,14 +2052,14 @@
       </c>
       <c r="C42" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOK-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.989</v>
+        <v>0.997</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.85</v>
+        <v>0.951</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -1979,18 +2078,18 @@
       </c>
       <c r="C43" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-GVER-LAZY-DOGL</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.957</v>
+        <v>0.993</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.512</v>
-      </c>
-      <c r="F43" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2005,18 +2104,18 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-ROX-WITH-TEW</t>
+          <t>DACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.992</v>
+        <v>0.974</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F44" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.514</v>
+      </c>
+      <c r="F44" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2031,18 +2130,18 @@
       </c>
       <c r="C45" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOR-JV</t>
+          <t>EIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.985</v>
+        <v>0.992</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="F45" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F45" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2057,14 +2156,14 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLNCK-GEMK</t>
+          <t>SPHINX-OF-BKHCK-GEM-</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.985</v>
+        <v>0.98</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.788</v>
+        <v>0.604</v>
       </c>
       <c r="F46" s="20" t="inlineStr">
         <is>
@@ -2087,10 +2186,10 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.999</v>
+        <v>0.991</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.99</v>
+        <v>0.822</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
@@ -2135,14 +2234,14 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>COMPVTFR-VISION-TEST</t>
+          <t>COMPUTFR-VISION-TEST</t>
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.992</v>
+        <v>0.995</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2165,10 +2264,10 @@
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>1</v>
+        <v>0.997</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.997</v>
+        <v>0.95</v>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
@@ -2187,18 +2286,18 @@
       </c>
       <c r="C51" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKR</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>0.989</v>
+        <v>1</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.771</v>
-      </c>
-      <c r="F51" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>1</v>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2213,18 +2312,18 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OM</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>0.985</v>
+        <v>1</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>0.696</v>
-      </c>
-      <c r="F52" s="20" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>1</v>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2239,14 +2338,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>PYTHONBDPENCVEROBON-</t>
+          <t>SYTHONPDPENUVBROBOT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.963</v>
+        <v>0.977</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.553</v>
+        <v>0.583</v>
       </c>
       <c r="F53" s="20" t="inlineStr">
         <is>
@@ -2265,14 +2364,14 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>SMART-ORC-RECOGNIZEB</t>
+          <t>SMART-ORC-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>0.996</v>
+        <v>1</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
@@ -2295,14 +2394,14 @@
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6</v>
+      </c>
+      <c r="F55" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2317,14 +2416,14 @@
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SVSTEM-OM</t>
+          <t>ARTIFICIAL-SVSPEM-OM</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.998</v>
+        <v>0.993</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.962</v>
+        <v>0.862</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
@@ -2343,11 +2442,11 @@
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>HELLO-DORLD-WELCOME-</t>
+          <t>HELLO-EORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.992</v>
+        <v>0.989</v>
       </c>
       <c r="E57" s="19" t="n">
         <v>0.85</v>
@@ -2369,18 +2468,18 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLKDGE-IS-POWER-W</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.977</v>
+        <v>0.989</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.863</v>
-      </c>
-      <c r="F58" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.781</v>
+      </c>
+      <c r="F58" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2395,14 +2494,14 @@
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLG</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.854</v>
+        <v>1</v>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
@@ -2421,14 +2520,14 @@
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TEH</t>
+          <t>ZERO-ONF-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.994</v>
+        <v>1</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.909</v>
+        <v>1</v>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
@@ -2447,23 +2546,1583 @@
       </c>
       <c r="C61" s="18" t="inlineStr">
         <is>
-          <t>ARCDEFGHIJKLMNOPQDST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D61" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C62" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D62" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OUER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="E63" s="19" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C64" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOX-WITH-IEA</t>
+        </is>
+      </c>
+      <c r="D64" s="15" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="E64" s="15" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="F64" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C65" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-BLACK-GEM-</t>
+        </is>
+      </c>
+      <c r="D66" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="15" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-NY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D67" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E67" s="19" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B68" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C68" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D68" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C69" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="E69" s="19" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C70" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-LEARNING-AIA</t>
+        </is>
+      </c>
+      <c r="D70" s="15" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E70" s="15" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="F70" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B71" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C71" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKY</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="E71" s="19" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C72" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D72" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C73" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOTP</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="E73" s="19" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="20" customHeight="1">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C74" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZEP</t>
+        </is>
+      </c>
+      <c r="D74" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E74" s="15" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B75" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C75" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTIONP</t>
+        </is>
+      </c>
+      <c r="D75" s="19" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="E75" s="19" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B76" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C76" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-SYSTEMAGK</t>
+        </is>
+      </c>
+      <c r="D76" s="15" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="E76" s="15" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C77" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOMK-</t>
+        </is>
+      </c>
+      <c r="D77" s="19" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="E77" s="19" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="F77" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C78" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POWERP-</t>
+        </is>
+      </c>
+      <c r="D78" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E78" s="15" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B79" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C79" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FINO-GOLN</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="E79" s="19" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="F79" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="13" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B80" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D80" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>test4.jpg</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C81" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="E81" s="19" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="F81" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B82" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D82" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="15" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B83" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="E83" s="19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B84" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C84" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MYXBOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D84" s="15" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="E84" s="15" t="n">
+        <v>0.296</v>
+      </c>
+      <c r="F84" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B85" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C85" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E85" s="19" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="F85" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B86" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C86" s="14" t="inlineStr">
+        <is>
+          <t>SPHJNX-OF-RLACK-GEM-</t>
+        </is>
+      </c>
+      <c r="D86" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="E86" s="15" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B87" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C87" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="20" customHeight="1">
+      <c r="A88" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B88" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C88" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZNPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D88" s="15" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E88" s="15" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="F88" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B89" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C89" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VIJTON-IEOT</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="n">
+        <v>0.988</v>
+      </c>
+      <c r="E89" s="19" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="F89" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B90" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C90" s="14" t="inlineStr">
+        <is>
+          <t>MACHTNE-LFARNJNG-AI-</t>
+        </is>
+      </c>
+      <c r="D90" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E90" s="15" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B91" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C91" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKS</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="E91" s="19" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F91" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B92" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C92" s="14" t="inlineStr">
+        <is>
+          <t>IMAGF-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D92" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="F92" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B93" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C93" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCU-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E93" s="19" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B94" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C94" s="14" t="inlineStr">
+        <is>
+          <t>SMARI-OCR-RECOGNIZF-</t>
+        </is>
+      </c>
+      <c r="D94" s="15" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="E94" s="15" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="F94" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B95" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C95" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATF-PREPICTION-</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="E95" s="19" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="F95" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B96" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C96" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D96" s="15" t="n">
+        <v>0.978</v>
+      </c>
+      <c r="E96" s="15" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="F96" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B97" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C97" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLO-NELCOMF-</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="E97" s="19" t="n">
+        <v>0.577</v>
+      </c>
+      <c r="F97" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B98" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C98" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEOGE-IS-POUEF--</t>
+        </is>
+      </c>
+      <c r="D98" s="15" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E98" s="15" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="F98" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B99" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C99" s="18" t="inlineStr">
+        <is>
+          <t>P-ND-FYTRA-FIND-GOLD</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="E99" s="19" t="n">
+        <v>0.758</v>
+      </c>
+      <c r="F99" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B100" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C100" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D100" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="E100" s="15" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F100" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="17" t="inlineStr">
+        <is>
+          <t>test5.jpg</t>
+        </is>
+      </c>
+      <c r="B101" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C101" s="18" t="inlineStr">
+        <is>
+          <t>ABPDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="E101" s="19" t="n">
+        <v>0.6879999999999999</v>
+      </c>
+      <c r="F101" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="20" customHeight="1">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B102" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUTCK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D102" s="15" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E102" s="15" t="n">
+        <v>0.783</v>
+      </c>
+      <c r="F102" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B103" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OUER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="E103" s="19" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="20" customHeight="1">
+      <c r="A104" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B104" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C104" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D104" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="15" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="20" customHeight="1">
+      <c r="A105" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B105" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C105" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LIQUOF-JU</t>
+        </is>
+      </c>
+      <c r="D105" s="19" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="E105" s="19" t="n">
+        <v>0.911</v>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="20" customHeight="1">
+      <c r="A106" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B106" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C106" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-BUACK-GEN-</t>
+        </is>
+      </c>
+      <c r="D106" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E106" s="15" t="n">
         <v>0.986</v>
       </c>
-      <c r="E61" s="19" t="n">
+      <c r="F106" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="20" customHeight="1">
+      <c r="A107" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B107" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C107" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-AY-VOC-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D107" s="19" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="E107" s="19" t="n">
+        <v>0.839</v>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="20" customHeight="1">
+      <c r="A108" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B108" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C108" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHG-ZERHVRS-RLOW-</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="E108" s="15" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="F108" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="20" customHeight="1">
+      <c r="A109" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B109" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C109" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VICION-TEST</t>
+        </is>
+      </c>
+      <c r="D109" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E109" s="19" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="F109" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="20" customHeight="1">
+      <c r="A110" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B110" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C110" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D110" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="F110" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B111" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C111" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKS</t>
+        </is>
+      </c>
+      <c r="D111" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F111" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="20" customHeight="1">
+      <c r="A112" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B112" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C112" s="14" t="inlineStr">
+        <is>
+          <t>TMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D112" s="15" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="E112" s="15" t="n">
+        <v>0.898</v>
+      </c>
+      <c r="F112" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B113" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C113" s="18" t="inlineStr">
+        <is>
+          <t>PVTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D113" s="19" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="E113" s="19" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="F113" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="20" customHeight="1">
+      <c r="A114" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B114" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C114" s="14" t="inlineStr">
+        <is>
+          <t>SMRRT-OCP-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="n">
+        <v>0.993</v>
+      </c>
+      <c r="E114" s="15" t="n">
         <v>0.85</v>
       </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>NO</t>
+      <c r="F114" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="20" customHeight="1">
+      <c r="A115" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B115" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C115" s="18" t="inlineStr">
+        <is>
+          <t>ARCUBATE-PREDICTION-</t>
+        </is>
+      </c>
+      <c r="D115" s="19" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E115" s="19" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="F115" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="20" customHeight="1">
+      <c r="A116" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B116" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C116" s="14" t="inlineStr">
+        <is>
+          <t>ADTIFTCTAY-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E116" s="15" t="n">
+        <v>0.359</v>
+      </c>
+      <c r="F116" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="20" customHeight="1">
+      <c r="A117" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B117" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C117" s="18" t="inlineStr">
+        <is>
+          <t>RELLO-WORLD-WELCONE-</t>
+        </is>
+      </c>
+      <c r="D117" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E117" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F117" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="20" customHeight="1">
+      <c r="A118" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B118" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C118" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEOGE-IS-POWER--</t>
+        </is>
+      </c>
+      <c r="D118" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="20" customHeight="1">
+      <c r="A119" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B119" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C119" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FIND-GOLD</t>
+        </is>
+      </c>
+      <c r="D119" s="19" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="E119" s="19" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="F119" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="20" customHeight="1">
+      <c r="A120" s="13" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B120" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C120" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D120" s="15" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="E120" s="15" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="F120" s="16" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="20" customHeight="1">
+      <c r="A121" s="17" t="inlineStr">
+        <is>
+          <t>test6.jpg</t>
+        </is>
+      </c>
+      <c r="B121" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C121" s="18" t="inlineStr">
+        <is>
+          <t>ARCDEFGHIJKLMNOPORST</t>
+        </is>
+      </c>
+      <c r="D121" s="19" t="n">
+        <v>0.973</v>
+      </c>
+      <c r="E121" s="19" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="F121" s="20" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F61"/>
+  <autoFilter ref="A1:F121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: enhance topological disambiguation (D vs C, U vs V, O vs C), achieving 92.21% accuracy
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-14 17:27:57 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-14 18:32:08 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>92.08%</t>
+          <t>92.21%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>78.00%</t>
+          <t>78.75%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -1636,11 +1636,11 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>GPHLNX-CF-BLACK-GFM-</t>
+          <t>GPHLNX-CF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E26" s="15" t="n">
         <v>0.5580000000000001</v>
@@ -1662,11 +1662,11 @@
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VCW-QVICKLY</t>
+          <t>JUDGE-MY-VOW-QVICKLY</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.978</v>
+        <v>0.97</v>
       </c>
       <c r="E27" s="19" t="n">
         <v>0.701</v>
@@ -1818,11 +1818,11 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYTHGN-OPFNCV-BOBCT-</t>
+          <t>DYTHGN-OPENCV-BOBCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.977</v>
+        <v>0.97</v>
       </c>
       <c r="E33" s="19" t="n">
         <v>0.5580000000000001</v>
@@ -1896,11 +1896,11 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICZALXSYSTEM-CV</t>
+          <t>ARTIFICZALXSYSTEM-CU</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.892</v>
+        <v>0.903</v>
       </c>
       <c r="E36" s="15" t="n">
         <v>0.31</v>

</xml_diff>

<commit_message>
feat: implement Level 1 & 2 optimizations, achieving all-time record 93.58% (2246/2400) accuracy
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -103,13 +103,13 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00375623"/>
+      <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00C00000"/>
+      <color rgb="00375623"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -238,7 +238,7 @@
     <xf numFmtId="164" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -250,7 +250,7 @@
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-14 18:32:08 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-15 14:38:40 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>92.21%</t>
+          <t>93.58%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>42 ข้อ</t>
+          <t>73 ข้อ</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>97.25%</t>
+          <t>99.50%</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.995</t>
+          <t>0.990</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>4 ข้อ</t>
+          <t>8 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,17 +793,17 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>78.75%</t>
+          <t>80.50%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.959</t>
+          <t>0.917</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>15 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>95.00%</t>
+          <t>95.25%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.993</t>
+          <t>0.975</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>5 ข้อ</t>
+          <t>12 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>96.50%</t>
+          <t>99.00%</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.995</t>
+          <t>0.993</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -892,17 +892,17 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>92.75%</t>
+          <t>93.25%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>0.987</t>
+          <t>0.977</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>9 ข้อ</t>
+          <t>14 ข้อ</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -925,17 +925,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>93.00%</t>
+          <t>94.00%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>0.991</t>
+          <t>0.970</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>5 ข้อ</t>
+          <t>15 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1016,14 +1016,14 @@
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.998</v>
+        <v>0.777</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1038,16 +1038,16 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVERALAZY-COG-</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D3" s="19" t="n">
         <v>0.992</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.848</v>
-      </c>
-      <c r="F3" s="16" t="inlineStr">
+        <v>0.85</v>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1068,14 +1068,14 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>1</v>
+        <v>0.785</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1094,14 +1094,14 @@
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.999</v>
+        <v>0.976</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.984</v>
+        <v>0.521</v>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1123,9 +1123,9 @@
         <v>0.999</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.984</v>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
+        <v>0.99</v>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1142,16 +1142,16 @@
       </c>
       <c r="C7" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VGW-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.986</v>
+        <v>0.982</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.725</v>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
+        <v>0.638</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1172,12 +1172,12 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.993</v>
+        <v>0.997</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.861</v>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
+        <v>0.931</v>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1198,14 +1198,14 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>0.983</v>
+        <v>1</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.658</v>
+        <v>0.998</v>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1220,16 +1220,16 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>MACHJNE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.995</v>
+        <v>0.992</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.908</v>
-      </c>
-      <c r="F10" s="16" t="inlineStr">
+        <v>0.899</v>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1250,14 +1250,14 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.998</v>
+        <v>0.986</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.97</v>
+        <v>0.744</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1272,18 +1272,18 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>JMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.999</v>
+        <v>0.972</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.985</v>
+        <v>0.511</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
       <c r="E13" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1333,7 +1333,7 @@
       <c r="E14" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1354,12 +1354,12 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>1</v>
+        <v>0.999</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
+        <v>0.989</v>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1376,16 +1376,16 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>ARTIFJCIAL-SYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.985</v>
+        <v>0.967</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.708</v>
-      </c>
-      <c r="F16" s="20" t="inlineStr">
+        <v>0.657</v>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1409,9 +1409,9 @@
         <v>1</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
+        <v>0.992</v>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1432,14 +1432,14 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.986</v>
+        <v>0.985</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.772</v>
+        <v>0.83</v>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1458,14 +1458,14 @@
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>1</v>
+        <v>0.976</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>1</v>
+        <v>0.513</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1480,16 +1480,16 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SJX-JEM</t>
+          <t>ZERO-ONE-TWO-SIX-IEN</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>1</v>
+        <v>0.995</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.997</v>
-      </c>
-      <c r="F20" s="16" t="inlineStr">
+        <v>0.95</v>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1506,16 +1506,16 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPMRST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.994</v>
+        <v>1</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.885</v>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -1532,16 +1532,16 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>THI-UUICK-PROWN-FCX-</t>
+          <t>THI-QUICK-DROWN-FCX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.975</v>
+        <v>0.909</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.793</v>
-      </c>
-      <c r="F22" s="20" t="inlineStr">
+        <v>0.468</v>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1558,16 +1558,16 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUGPS-OVER-LAZY-COG-</t>
+          <t>JUMPS-OVER-LAZY-CQG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.952</v>
+        <v>0.901</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.543</v>
-      </c>
-      <c r="F23" s="20" t="inlineStr">
+        <v>0.455</v>
+      </c>
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1584,18 +1584,18 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MV-COX-WITH-TEA</t>
+          <t>PACK-MV-GOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.988</v>
+        <v>0.971</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.908</v>
+        <v>0.519</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1610,16 +1610,16 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>EIVF-EOZFNWLIQUQR-JD</t>
+          <t>EIVE-EOZFNWLIQUQR-JD</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.923</v>
+        <v>0.92</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.531</v>
-      </c>
-      <c r="F25" s="20" t="inlineStr">
+        <v>0.501</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1636,16 +1636,16 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>GPHLNX-CF-BLACK-GEM-</t>
+          <t>SPHLNX-CF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.946</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.5580000000000001</v>
-      </c>
-      <c r="F26" s="20" t="inlineStr">
+        <v>0.64</v>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1666,12 +1666,12 @@
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.97</v>
+        <v>0.931</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.701</v>
-      </c>
-      <c r="F27" s="20" t="inlineStr">
+        <v>0.44</v>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1688,18 +1688,18 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BRJGHT-ZEPHYRS-BLOL-</t>
+          <t>BRIGHT-ZEPHYRS-RLOL-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.979</v>
+        <v>0.95</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.85</v>
+        <v>0.499</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1714,18 +1714,18 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TESE</t>
+          <t>COMPUTER-VISION-TESN</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.982</v>
+        <v>0.96</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.85</v>
+        <v>0.46</v>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1740,16 +1740,16 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEANN-NG-AJ-</t>
+          <t>MACHINE-UEAMN-NG-AJ-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.97</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.504</v>
-      </c>
-      <c r="F30" s="20" t="inlineStr">
+        <v>0.446</v>
+      </c>
+      <c r="F30" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1766,16 +1766,16 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DFEP-NEUPAU-AFTVORKX</t>
+          <t>DEEP-NFUPAU-NFTWORKX</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.952</v>
+        <v>0.864</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.548</v>
-      </c>
-      <c r="F31" s="20" t="inlineStr">
+        <v>0.501</v>
+      </c>
+      <c r="F31" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1792,16 +1792,16 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGF-OATA-EEZFCT-CU</t>
+          <t>-MAGE-OATA-EEZFCT-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.95</v>
+        <v>0.902</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.467</v>
-      </c>
-      <c r="F32" s="20" t="inlineStr">
+        <v>0.501</v>
+      </c>
+      <c r="F32" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1818,16 +1818,16 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYTHGN-OPENCV-BOBCT-</t>
+          <t>DYTHQN-OPENCV-BOBCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.97</v>
+        <v>0.968</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.5580000000000001</v>
-      </c>
-      <c r="F33" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1848,12 +1848,12 @@
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.925</v>
+        <v>0.885</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.496</v>
-      </c>
-      <c r="F34" s="20" t="inlineStr">
+        <v>0.381</v>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1870,16 +1870,16 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>ACCURAJF--REDJCZJRA-</t>
+          <t>-CCURAIF--REDICZJZN-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.944</v>
+        <v>0.918</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.725</v>
-      </c>
-      <c r="F35" s="20" t="inlineStr">
+        <v>0.503</v>
+      </c>
+      <c r="F35" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1896,16 +1896,16 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICZALXSYSTEM-CU</t>
+          <t>-RTIFICXALYSYS-EM-CK</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.903</v>
+        <v>0.882</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="F36" s="20" t="inlineStr">
+        <v>0.267</v>
+      </c>
+      <c r="F36" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1922,18 +1922,18 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLG-WOFLD-VFLOCME-</t>
+          <t>HELLC-WOFLD-VELOCME-</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.987</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.876</v>
+        <v>0.483</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1948,16 +1948,16 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KWOWL-CCE-IS-POKER--</t>
+          <t>KWOWL-CCF-IS-PQKER--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.965</v>
+        <v>0.906</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="F38" s="20" t="inlineStr">
+        <v>0.472</v>
+      </c>
+      <c r="F38" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -1974,16 +1974,16 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>FIND-FXTRA-GINF-GDLC</t>
+          <t>FIND-FXTRA-EINE-GDLC</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.967</v>
+        <v>0.895</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.5590000000000001</v>
-      </c>
-      <c r="F39" s="20" t="inlineStr">
+        <v>0.493</v>
+      </c>
+      <c r="F39" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2000,16 +2000,16 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZJRG-NNE-TXG-SIX-TEN</t>
+          <t>ZJRQ-ONE-TXG-SIX-TEN</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.951</v>
+        <v>0.867</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="F40" s="20" t="inlineStr">
+        <v>0.499</v>
+      </c>
+      <c r="F40" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2026,18 +2026,18 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPGEOT</t>
+          <t>ABCDEFGHIJKLMNCPGROT</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.99</v>
+        <v>0.891</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.907</v>
+        <v>0.489</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2056,14 +2056,14 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.997</v>
+        <v>0.973</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.951</v>
+        <v>0.495</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2082,12 +2082,12 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.993</v>
+        <v>0.989</v>
       </c>
       <c r="E43" s="19" t="n">
         <v>0.85</v>
       </c>
-      <c r="F43" s="16" t="inlineStr">
+      <c r="F43" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2104,16 +2104,16 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>DACK-MY-ROX-WITH-TEA</t>
+          <t>EACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.974</v>
+        <v>0.968</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.514</v>
-      </c>
-      <c r="F44" s="20" t="inlineStr">
+        <v>0.518</v>
+      </c>
+      <c r="F44" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2134,14 +2134,14 @@
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.992</v>
+        <v>0.979</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.85</v>
+        <v>0.725</v>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2156,16 +2156,16 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BKHCK-GEM-</t>
+          <t>SPHINX-OF-BLHCK-GEM-</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.98</v>
+        <v>0.985</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.604</v>
-      </c>
-      <c r="F46" s="20" t="inlineStr">
+        <v>0.698</v>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2186,14 +2186,14 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.991</v>
+        <v>0.971</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.822</v>
+        <v>0.549</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2212,14 +2212,14 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>1</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.999</v>
+        <v>0.502</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2234,18 +2234,18 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>COMPUTFR-VISION-TEST</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>1</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.995</v>
+        <v>0.5</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2264,12 +2264,12 @@
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.997</v>
+        <v>0.999</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F50" s="16" t="inlineStr">
+        <v>0.972</v>
+      </c>
+      <c r="F50" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2290,12 +2290,12 @@
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>1</v>
+        <v>0.992</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F51" s="16" t="inlineStr">
+        <v>0.857</v>
+      </c>
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2321,7 +2321,7 @@
       <c r="E52" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F52" s="16" t="inlineStr">
+      <c r="F52" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2338,16 +2338,16 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>SYTHONPDPENUVBROBOT-</t>
+          <t>SYTHONPDPENUVAROBOT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.977</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.583</v>
-      </c>
-      <c r="F53" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F53" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2371,9 +2371,9 @@
         <v>1</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="16" t="inlineStr">
+        <v>0.996</v>
+      </c>
+      <c r="F54" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2394,12 +2394,12 @@
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.98</v>
+        <v>0.964</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F55" s="20" t="inlineStr">
+        <v>0.501</v>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2420,14 +2420,14 @@
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.993</v>
+        <v>0.969</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.862</v>
+        <v>0.5</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2442,18 +2442,18 @@
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>HELLO-EORLD-WELCOME-</t>
+          <t>HELLO-XOXLD-WELCOME-</t>
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.989</v>
+        <v>0.948</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.85</v>
+        <v>0.5</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2468,16 +2468,16 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWER--</t>
+          <t>KNOWLEDGE-IS-FOWER--</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.989</v>
+        <v>0.958</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.781</v>
-      </c>
-      <c r="F58" s="20" t="inlineStr">
+        <v>0.551</v>
+      </c>
+      <c r="F58" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2501,9 +2501,9 @@
         <v>1</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="16" t="inlineStr">
+        <v>0.993</v>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2520,16 +2520,16 @@
       </c>
       <c r="C60" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONF-TWO-SIX-TEN</t>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" s="16" t="inlineStr">
+        <v>0.85</v>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2555,7 +2555,7 @@
       <c r="E61" s="19" t="n">
         <v>0.999</v>
       </c>
-      <c r="F61" s="16" t="inlineStr">
+      <c r="F61" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2581,7 +2581,7 @@
       <c r="E62" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F62" s="16" t="inlineStr">
+      <c r="F62" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2602,12 +2602,12 @@
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.998</v>
+        <v>0.993</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.965</v>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
+        <v>0.85</v>
+      </c>
+      <c r="F63" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2624,18 +2624,18 @@
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOX-WITH-IEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>0.997</v>
+        <v>0.959</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.531</v>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2659,7 @@
       <c r="E65" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F65" s="16" t="inlineStr">
+      <c r="F65" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2683,9 +2683,9 @@
         <v>1</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="F66" s="16" t="inlineStr">
+        <v>0.997</v>
+      </c>
+      <c r="F66" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2706,12 +2706,12 @@
         </is>
       </c>
       <c r="D67" s="19" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>0.982</v>
-      </c>
-      <c r="F67" s="16" t="inlineStr">
+        <v>0.991</v>
+      </c>
+      <c r="F67" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2737,7 +2737,7 @@
       <c r="E68" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F68" s="16" t="inlineStr">
+      <c r="F68" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2758,12 +2758,12 @@
         </is>
       </c>
       <c r="D69" s="19" t="n">
-        <v>0.996</v>
+        <v>0.998</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>0.923</v>
-      </c>
-      <c r="F69" s="16" t="inlineStr">
+        <v>0.962</v>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2780,16 +2780,16 @@
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AIA</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.99</v>
+        <v>0.996</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>0.834</v>
-      </c>
-      <c r="F70" s="16" t="inlineStr">
+        <v>0.917</v>
+      </c>
+      <c r="F70" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2806,16 +2806,16 @@
       </c>
       <c r="C71" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKY</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D71" s="19" t="n">
-        <v>0.993</v>
+        <v>1</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>0.868</v>
-      </c>
-      <c r="F71" s="16" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="F71" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2841,7 +2841,7 @@
       <c r="E72" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F72" s="16" t="inlineStr">
+      <c r="F72" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2858,16 +2858,16 @@
       </c>
       <c r="C73" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENCV-ROBOTP</t>
+          <t>PYTHON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D73" s="19" t="n">
-        <v>0.997</v>
+        <v>0.999</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.9379999999999999</v>
-      </c>
-      <c r="F73" s="16" t="inlineStr">
+        <v>0.973</v>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2884,16 +2884,16 @@
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-RECOGNIZEP</t>
+          <t>SMART-OCR-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F74" s="16" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -2910,18 +2910,18 @@
       </c>
       <c r="C75" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTIONP</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>0.998</v>
+        <v>0.975</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>0.962</v>
+        <v>0.505</v>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2936,18 +2936,18 @@
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSTEMAGK</t>
+          <t>ARTIEICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.985</v>
+        <v>0.993</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>0.729</v>
+        <v>0.85</v>
       </c>
       <c r="F76" s="20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2962,16 +2962,16 @@
       </c>
       <c r="C77" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCOMK-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>0.989</v>
+        <v>0.975</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>0.786</v>
-      </c>
-      <c r="F77" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -2988,16 +2988,16 @@
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWERP-</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D78" s="15" t="n">
         <v>0.999</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>0.973</v>
-      </c>
-      <c r="F78" s="16" t="inlineStr">
+        <v>0.986</v>
+      </c>
+      <c r="F78" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3014,16 +3014,16 @@
       </c>
       <c r="C79" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FINO-GOLN</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>0.973</v>
+        <v>0.982</v>
       </c>
       <c r="E79" s="19" t="n">
-        <v>0.706</v>
-      </c>
-      <c r="F79" s="20" t="inlineStr">
+        <v>0.647</v>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3047,9 +3047,9 @@
         <v>1</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="F80" s="16" t="inlineStr">
+        <v>0.996</v>
+      </c>
+      <c r="F80" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3070,14 +3070,14 @@
         </is>
       </c>
       <c r="D81" s="19" t="n">
-        <v>0.989</v>
+        <v>0.993</v>
       </c>
       <c r="E81" s="19" t="n">
-        <v>0.786</v>
+        <v>0.85</v>
       </c>
       <c r="F81" s="20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3096,14 +3096,14 @@
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.997</v>
+        <v>0.771</v>
       </c>
       <c r="F82" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3122,12 +3122,12 @@
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>0.991</v>
+        <v>0.992</v>
       </c>
       <c r="E83" s="19" t="n">
         <v>0.85</v>
       </c>
-      <c r="F83" s="16" t="inlineStr">
+      <c r="F83" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3148,12 +3148,12 @@
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>0.954</v>
+        <v>0.956</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>0.296</v>
-      </c>
-      <c r="F84" s="20" t="inlineStr">
+        <v>0.221</v>
+      </c>
+      <c r="F84" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3174,14 +3174,14 @@
         </is>
       </c>
       <c r="D85" s="19" t="n">
-        <v>0.999</v>
+        <v>0.976</v>
       </c>
       <c r="E85" s="19" t="n">
-        <v>0.979</v>
+        <v>0.536</v>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3200,12 +3200,12 @@
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>0.993</v>
+        <v>0.992</v>
       </c>
       <c r="E86" s="15" t="n">
         <v>0.85</v>
       </c>
-      <c r="F86" s="16" t="inlineStr">
+      <c r="F86" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3231,7 +3231,7 @@
       <c r="E87" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F87" s="16" t="inlineStr">
+      <c r="F87" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3248,16 +3248,16 @@
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZNPHYRS-BLOW-</t>
+          <t>BRIGHT-ZYPHYRS-BLOW-</t>
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.976</v>
+        <v>0.979</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.511</v>
-      </c>
-      <c r="F88" s="20" t="inlineStr">
+        <v>0.57</v>
+      </c>
+      <c r="F88" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3274,18 +3274,18 @@
       </c>
       <c r="C89" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VIJTON-IEOT</t>
+          <t>COMPUTER-VIJTON-TEST</t>
         </is>
       </c>
       <c r="D89" s="19" t="n">
-        <v>0.988</v>
+        <v>0.954</v>
       </c>
       <c r="E89" s="19" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.499</v>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3304,12 +3304,12 @@
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>0.999</v>
+        <v>1</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="F90" s="16" t="inlineStr">
+        <v>0.995</v>
+      </c>
+      <c r="F90" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3330,12 +3330,12 @@
         </is>
       </c>
       <c r="D91" s="19" t="n">
-        <v>0.974</v>
+        <v>0.96</v>
       </c>
       <c r="E91" s="19" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="F91" s="20" t="inlineStr">
+        <v>0.503</v>
+      </c>
+      <c r="F91" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3359,9 +3359,9 @@
         <v>1</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="F92" s="16" t="inlineStr">
+        <v>0.996</v>
+      </c>
+      <c r="F92" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3385,9 +3385,9 @@
         <v>0.999</v>
       </c>
       <c r="E93" s="19" t="n">
-        <v>0.975</v>
-      </c>
-      <c r="F93" s="16" t="inlineStr">
+        <v>0.987</v>
+      </c>
+      <c r="F93" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3404,16 +3404,16 @@
       </c>
       <c r="C94" s="14" t="inlineStr">
         <is>
-          <t>SMARI-OCR-RECOGNIZF-</t>
+          <t>SMAR--OCR-RECOGNIZF-</t>
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>0.975</v>
+        <v>0.963</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>0.5620000000000001</v>
-      </c>
-      <c r="F94" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F94" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3434,14 +3434,14 @@
         </is>
       </c>
       <c r="D95" s="19" t="n">
-        <v>0.996</v>
+        <v>0.968</v>
       </c>
       <c r="E95" s="19" t="n">
-        <v>0.923</v>
+        <v>0.598</v>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3460,12 +3460,12 @@
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>0.978</v>
+        <v>0.966</v>
       </c>
       <c r="E96" s="15" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="F96" s="20" t="inlineStr">
+        <v>0.509</v>
+      </c>
+      <c r="F96" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3486,12 +3486,12 @@
         </is>
       </c>
       <c r="D97" s="19" t="n">
-        <v>0.971</v>
+        <v>0.976</v>
       </c>
       <c r="E97" s="19" t="n">
-        <v>0.577</v>
-      </c>
-      <c r="F97" s="20" t="inlineStr">
+        <v>0.679</v>
+      </c>
+      <c r="F97" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3512,12 +3512,12 @@
         </is>
       </c>
       <c r="D98" s="15" t="n">
-        <v>0.982</v>
+        <v>0.986</v>
       </c>
       <c r="E98" s="15" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="F98" s="20" t="inlineStr">
+        <v>0.712</v>
+      </c>
+      <c r="F98" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3538,12 +3538,12 @@
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.987</v>
+        <v>0.944</v>
       </c>
       <c r="E99" s="19" t="n">
-        <v>0.758</v>
-      </c>
-      <c r="F99" s="20" t="inlineStr">
+        <v>0.383</v>
+      </c>
+      <c r="F99" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3560,18 +3560,18 @@
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TEN</t>
+          <t>ZERO-ONE-TWO-SIX-TRN</t>
         </is>
       </c>
       <c r="D100" s="15" t="n">
-        <v>0.993</v>
+        <v>0.98</v>
       </c>
       <c r="E100" s="15" t="n">
-        <v>0.85</v>
+        <v>0.613</v>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3586,16 +3586,16 @@
       </c>
       <c r="C101" s="18" t="inlineStr">
         <is>
-          <t>ABPDEFGHIJKLMNOPQRST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D101" s="19" t="n">
-        <v>0.984</v>
+        <v>0.967</v>
       </c>
       <c r="E101" s="19" t="n">
-        <v>0.6879999999999999</v>
-      </c>
-      <c r="F101" s="20" t="inlineStr">
+        <v>0.501</v>
+      </c>
+      <c r="F101" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3616,12 +3616,12 @@
         </is>
       </c>
       <c r="D102" s="15" t="n">
-        <v>0.982</v>
+        <v>0.962</v>
       </c>
       <c r="E102" s="15" t="n">
-        <v>0.783</v>
-      </c>
-      <c r="F102" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F102" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3642,12 +3642,12 @@
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.997</v>
+        <v>0.992</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="F103" s="16" t="inlineStr">
+        <v>0.85</v>
+      </c>
+      <c r="F103" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3671,9 +3671,9 @@
         <v>1</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="F104" s="16" t="inlineStr">
+        <v>0.994</v>
+      </c>
+      <c r="F104" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -3690,18 +3690,18 @@
       </c>
       <c r="C105" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOF-JU</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D105" s="19" t="n">
-        <v>0.996</v>
+        <v>0.977</v>
       </c>
       <c r="E105" s="19" t="n">
-        <v>0.911</v>
+        <v>0.542</v>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3716,18 +3716,18 @@
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BUACK-GEN-</t>
+          <t>SPHINX-OF-BUACK-GEM-</t>
         </is>
       </c>
       <c r="D106" s="15" t="n">
-        <v>0.999</v>
+        <v>0.974</v>
       </c>
       <c r="E106" s="15" t="n">
-        <v>0.986</v>
+        <v>0.5</v>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3742,18 +3742,18 @@
       </c>
       <c r="C107" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-AY-VOC-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D107" s="19" t="n">
-        <v>0.989</v>
+        <v>0.95</v>
       </c>
       <c r="E107" s="19" t="n">
-        <v>0.839</v>
+        <v>0.5</v>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3768,16 +3768,16 @@
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>BRIGHG-ZERHVRS-RLOW-</t>
+          <t>BRIGHT-ZERHVRS-BLOW-</t>
         </is>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.966</v>
+        <v>0.918</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.695</v>
-      </c>
-      <c r="F108" s="20" t="inlineStr">
+        <v>0.524</v>
+      </c>
+      <c r="F108" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -3794,18 +3794,18 @@
       </c>
       <c r="C109" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VICION-TEST</t>
+          <t>COMPUTER-VICION-TECT</t>
         </is>
       </c>
       <c r="D109" s="19" t="n">
-        <v>0.999</v>
+        <v>0.925</v>
       </c>
       <c r="E109" s="19" t="n">
-        <v>0.971</v>
+        <v>0.5</v>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3824,14 +3824,14 @@
         </is>
       </c>
       <c r="D110" s="15" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.999</v>
+        <v>0.751</v>
       </c>
       <c r="F110" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3850,14 +3850,14 @@
         </is>
       </c>
       <c r="D111" s="19" t="n">
-        <v>1</v>
+        <v>0.976</v>
       </c>
       <c r="E111" s="19" t="n">
-        <v>1</v>
+        <v>0.52</v>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3872,18 +3872,18 @@
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>TMAGE-DATA-DETECT-OK</t>
+          <t>TMAG--DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.994</v>
+        <v>0.973</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.898</v>
+        <v>0.508</v>
       </c>
       <c r="F112" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3898,18 +3898,18 @@
       </c>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>PVTHON-OPENCV-ROBOT-</t>
+          <t>P-THON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D113" s="19" t="n">
-        <v>0.998</v>
+        <v>0.977</v>
       </c>
       <c r="E113" s="19" t="n">
-        <v>0.965</v>
+        <v>0.543</v>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3924,18 +3924,18 @@
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>SMRRT-OCP-RECOGNIZE-</t>
+          <t>SMPRT-OCP-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D114" s="15" t="n">
-        <v>0.993</v>
+        <v>0.973</v>
       </c>
       <c r="E114" s="15" t="n">
-        <v>0.85</v>
+        <v>0.479</v>
       </c>
       <c r="F114" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3950,18 +3950,18 @@
       </c>
       <c r="C115" s="18" t="inlineStr">
         <is>
-          <t>ARCUBATE-PREDICTION-</t>
+          <t>ARCUDATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D115" s="19" t="n">
-        <v>0.999</v>
+        <v>0.972</v>
       </c>
       <c r="E115" s="19" t="n">
-        <v>0.974</v>
+        <v>0.501</v>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3976,16 +3976,16 @@
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>ADTIFTCTAY-SYSTEM-OK</t>
+          <t>ADTIFTCTAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.95</v>
+        <v>0.958</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.359</v>
-      </c>
-      <c r="F116" s="20" t="inlineStr">
+        <v>0.503</v>
+      </c>
+      <c r="F116" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
@@ -4006,14 +4006,14 @@
         </is>
       </c>
       <c r="D117" s="19" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="E117" s="19" t="n">
-        <v>1</v>
+        <v>0.504</v>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       <c r="E118" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F118" s="16" t="inlineStr">
+      <c r="F118" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -4054,18 +4054,18 @@
       </c>
       <c r="C119" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D119" s="19" t="n">
-        <v>0.981</v>
+        <v>0.978</v>
       </c>
       <c r="E119" s="19" t="n">
-        <v>0.634</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="F119" s="20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4087,9 +4087,9 @@
         <v>0.999</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>0.981</v>
-      </c>
-      <c r="F120" s="16" t="inlineStr">
+        <v>0.99</v>
+      </c>
+      <c r="F120" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
@@ -4110,12 +4110,12 @@
         </is>
       </c>
       <c r="D121" s="19" t="n">
-        <v>0.973</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E121" s="19" t="n">
-        <v>0.611</v>
-      </c>
-      <c r="F121" s="20" t="inlineStr">
+        <v>0.5</v>
+      </c>
+      <c r="F121" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>

</xml_diff>

<commit_message>
feat: optimize accumulated stroke merging and surgical disambiguation, reaching new high 93.75% (2250/2400)
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-15 14:38:40 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-15 15:52:31 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>93.58%</t>
+          <t>93.75%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>73 ข้อ</t>
+          <t>75 ข้อ</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.917</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>99.00%</t>
+          <t>99.25%</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.993</t>
+          <t>0.992</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>4 ข้อ</t>
+          <t>5 ข้อ</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -892,7 +892,7 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>93.25%</t>
+          <t>93.75%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>94.00%</t>
+          <t>94.25%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>15 ข้อ</t>
+          <t>16 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -1688,11 +1688,11 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZEPHYRS-RLOL-</t>
+          <t>BRIGHT-ZEPHYRS-BLOL-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.95</v>
+        <v>0.954</v>
       </c>
       <c r="E28" s="15" t="n">
         <v>0.499</v>
@@ -1714,11 +1714,11 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TESN</t>
+          <t>COMPUTEB-VISION-TESN</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.96</v>
+        <v>0.968</v>
       </c>
       <c r="E29" s="19" t="n">
         <v>0.46</v>
@@ -1844,11 +1844,11 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SFART-CCRXRECCGWIZE-</t>
+          <t>SEABT-CCRXRECCGWIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.885</v>
+        <v>0.913</v>
       </c>
       <c r="E34" s="15" t="n">
         <v>0.381</v>
@@ -2026,11 +2026,11 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNCPGROT</t>
+          <t>ABCDEFGHIJKLMNOPGROT</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.891</v>
+        <v>0.908</v>
       </c>
       <c r="E41" s="19" t="n">
         <v>0.489</v>
@@ -2598,18 +2598,18 @@
       </c>
       <c r="C63" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OUER-LAZY-DOG-</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.993</v>
+        <v>0.976</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F63" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.517</v>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3196,14 +3196,14 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>SPHJNX-OF-RLACK-GEM-</t>
+          <t>SPHJNX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>0.992</v>
+        <v>1</v>
       </c>
       <c r="E86" s="15" t="n">
-        <v>0.85</v>
+        <v>0.997</v>
       </c>
       <c r="F86" s="20" t="inlineStr">
         <is>
@@ -3534,11 +3534,11 @@
       </c>
       <c r="C99" s="18" t="inlineStr">
         <is>
-          <t>P-ND-FYTRA-FIND-GOLD</t>
+          <t>P-ND-EYTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.944</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E99" s="19" t="n">
         <v>0.383</v>
@@ -3638,18 +3638,18 @@
       </c>
       <c r="C103" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OUER-LAZY-DOG-</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.992</v>
+        <v>0.976</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F103" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.53</v>
+      </c>
+      <c r="F103" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement Super-Ensemble and Custom 2D CNN with Focal Loss, boosting 9-sheet benchmark to 94.03% (3385/3600)
- Add Custom 2D CNN (CharCNN) trained with Focal Loss (gamma=2.0) and Random Stroke Erasing in train_cnn.py (Best Val Acc 95.52%).
- Implement SuperEnsembleClassifier (30% Dual-Ensemble MLP + 70% 2D CNN) in scan_and_predict.py, achieving new benchmark high 94.03% (3,385/3,600 cells).
- Breakthrough on faint pencil sheet test2.jpg: improved from 80.75% (323/400) to 83.50% (334/400) (+11 correct characters).
- Expand test suite to 9 student answer sheets (3,600 cells) with strict Master Key fidelity (zero dictionary hallucination).
- Upgrade batch_processor.py with multi-model CLI selector (--model super/cnn/ensemble) and regenerate all_results.xlsx.
- Add comparative benchmark script compare_cnn_vs_ensemble.py, presentation assets, and training logs.
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -618,10 +618,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="78" customWidth="1" min="1" max="1"/>
+    <col width="132" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-15 15:56:23 | ตรวจทั้งหมด: 6 แผ่น | รวม 120 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-20 13:29:05 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 9 แผ่น | รวม 180 ข้อ</t>
         </is>
       </c>
     </row>
@@ -676,27 +676,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>6 แผ่น</t>
+          <t>9 แผ่น</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>120 ข้อ</t>
+          <t>180 ข้อ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2,400 ตัว</t>
+          <t>3,600 ตัว</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>93.75%</t>
+          <t>94.03%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>75 ข้อ</t>
+          <t>128 ข้อ</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>99.50%</t>
+          <t>98.00%</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.990</t>
+          <t>0.968</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>8 ข้อ</t>
+          <t>11 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>80.50%</t>
+          <t>83.50%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.920</t>
+          <t>0.869</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>95.25%</t>
+          <t>95.50%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.975</t>
+          <t>0.946</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>12 ข้อ</t>
+          <t>17 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>99.25%</t>
+          <t>97.75%</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.992</t>
+          <t>0.970</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>5 ข้อ</t>
+          <t>10 ข้อ</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -892,17 +892,17 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>93.75%</t>
+          <t>94.50%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>0.977</t>
+          <t>0.947</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>14 ข้อ</t>
+          <t>16 ข้อ</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -925,20 +925,119 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>94.25%</t>
+          <t>95.25%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>0.970</t>
+          <t>0.957</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>16 ข้อ</t>
+          <t>12 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>95.75%</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>0.965</t>
+        </is>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>11 ข้อ</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>93.75%</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>0.925</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>18 ข้อ</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>92.25%</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>0.967</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>13 ข้อ</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
         <is>
           <t>English &amp; Tech (ชุดที่ 1)</t>
         </is>
@@ -958,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1012,14 +1111,14 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOX-</t>
+          <t>THE-QUICK-BROWN-EOX-</t>
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.988</v>
+        <v>0.961</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.777</v>
+        <v>0.747</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -1042,7 +1141,7 @@
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.992</v>
+        <v>0.982</v>
       </c>
       <c r="E3" s="19" t="n">
         <v>0.85</v>
@@ -1068,10 +1167,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.989</v>
+        <v>0.968</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.785</v>
+        <v>0.734</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -1090,18 +1189,18 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOR-JU</t>
+          <t>EIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.976</v>
+        <v>0.957</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.521</v>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1116,14 +1215,14 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLACK-GEM-</t>
+          <t>SPHINX-OE-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>0.999</v>
+        <v>0.983</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.99</v>
+        <v>0.85</v>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
@@ -1146,14 +1245,14 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.982</v>
+        <v>0.972</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.638</v>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.869</v>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1172,10 +1271,10 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.997</v>
+        <v>0.99</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.931</v>
+        <v>0.958</v>
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
@@ -1198,14 +1297,14 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.998</v>
-      </c>
-      <c r="F9" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.646</v>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1224,14 +1323,14 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.992</v>
+        <v>0.974</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.899</v>
-      </c>
-      <c r="F10" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1250,10 +1349,10 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.986</v>
+        <v>0.958</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.744</v>
+        <v>0.649</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -1276,10 +1375,10 @@
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.972</v>
+        <v>0.944</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.511</v>
+        <v>0.605</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
@@ -1302,10 +1401,10 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
@@ -1328,10 +1427,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>1</v>
+        <v>0.898</v>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
@@ -1354,14 +1453,14 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.999</v>
+        <v>0.966</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.989</v>
-      </c>
-      <c r="F15" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.792</v>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1376,14 +1475,14 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSTEM-OK</t>
+          <t>ARTIEICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.967</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.657</v>
+        <v>0.456</v>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
@@ -1406,14 +1505,14 @@
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>1</v>
+        <v>0.974</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.788</v>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1432,14 +1531,14 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.985</v>
+        <v>0.972</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="F18" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.711</v>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1454,18 +1553,18 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-EIND-GOLD</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.976</v>
+        <v>0.957</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.513</v>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.829</v>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1480,18 +1579,18 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-IEN</t>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.995</v>
+        <v>0.964</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F20" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1506,14 +1605,14 @@
       </c>
       <c r="C21" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPQRST</t>
+          <t>ABCDEEGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>1</v>
+        <v>0.977</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="F21" s="20" t="inlineStr">
         <is>
@@ -1532,14 +1631,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>THI-QUICK-DROWN-FCX-</t>
+          <t>TIL-QUICK-BROWN-FQX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.909</v>
+        <v>0.881</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.468</v>
+        <v>0.433</v>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
@@ -1558,14 +1657,14 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-CQG-</t>
+          <t>JUMMS-OVER-LAZY-CQG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.901</v>
+        <v>0.885</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.455</v>
+        <v>0.427</v>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
@@ -1584,14 +1683,14 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MV-GOX-WITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.971</v>
+        <v>0.961</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.519</v>
+        <v>0.745</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
@@ -1610,14 +1709,14 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>EIVE-EOZFNWLIQUQR-JD</t>
+          <t>EIVE-DOZEN-LIQUQR-JV</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.92</v>
+        <v>0.856</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.501</v>
+        <v>0.449</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -1636,14 +1735,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHLNX-CF-BLACK-GEM-</t>
+          <t>SPHUNX-OE-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.946</v>
+        <v>0.905</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.64</v>
+        <v>0.487</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -1666,10 +1765,10 @@
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.931</v>
+        <v>0.908</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.44</v>
+        <v>0.533</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -1688,14 +1787,14 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZEPHYRS-BLOL-</t>
+          <t>RR-GHI-LEPHYRS-ELOW-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.954</v>
+        <v>0.859</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.499</v>
+        <v>0.224</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
@@ -1714,14 +1813,14 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUTEB-VISION-TESN</t>
+          <t>COMPUIER-VISION-TESD</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.968</v>
+        <v>0.893</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.46</v>
+        <v>0.223</v>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
@@ -1740,14 +1839,14 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-UEAMN-NG-AJ-</t>
+          <t>MACHINEWLEARNING-AJ-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.908</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.446</v>
+        <v>0.282</v>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
@@ -1766,14 +1865,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NFUPAU-NFTWORKX</t>
+          <t>DEEP-NEURAU-NFTMQRKS</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.864</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.501</v>
+        <v>0.357</v>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
@@ -1792,14 +1891,14 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGE-OATA-EEZFCT-CK</t>
+          <t>-MAGE-DATA-DEZFCT-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.902</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.501</v>
+        <v>0.29</v>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
@@ -1818,14 +1917,14 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYTHQN-OPENCV-BOBCT-</t>
+          <t>DYIHON-OPENCV-BOBCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.968</v>
+        <v>0.906</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.5</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
@@ -1844,14 +1943,14 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SEABT-CCRXRECCGWIZE-</t>
+          <t>SMART-CCR-RECOGWIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.913</v>
+        <v>0.865</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.381</v>
+        <v>0.21</v>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
@@ -1870,14 +1969,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>-CCURAIF--REDICZJZN-</t>
+          <t>ACCUKATF--REDICTJBN-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.918</v>
+        <v>0.847</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.503</v>
+        <v>0.337</v>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
@@ -1896,14 +1995,14 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>-RTIFICXALYSYS-EM-CK</t>
+          <t>ARTIFICJAL-SYSTEM-CK</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.882</v>
+        <v>0.848</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.267</v>
+        <v>0.525</v>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
@@ -1922,14 +2021,14 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLC-WOFLD-VELOCME-</t>
+          <t>HELLC-WORLC-VELOCME-</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.877</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.483</v>
+        <v>0.412</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
@@ -1948,14 +2047,14 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KWOWL-CCF-IS-PQKER--</t>
+          <t>KNOWLUCCEDIS-PQWEB--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.906</v>
+        <v>0.826</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.472</v>
+        <v>0.14</v>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
@@ -1974,14 +2073,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>FIND-FXTRA-EINE-GDLC</t>
+          <t>EIND-FXTRA-EINE-GDLD</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.895</v>
+        <v>0.862</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.493</v>
+        <v>0.382</v>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
@@ -2000,14 +2099,14 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZJRQ-ONE-TXG-SIX-TEN</t>
+          <t>ZERQ-ONF--WG-SIX-TEN</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.867</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.499</v>
+        <v>0.355</v>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
@@ -2026,14 +2125,14 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPGROT</t>
+          <t>ABCDEFGHIJKL-NCHGRQT</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.908</v>
+        <v>0.856</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.489</v>
+        <v>0.215</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
@@ -2056,10 +2155,10 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.973</v>
+        <v>0.974</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.495</v>
+        <v>0.734</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -2082,14 +2181,14 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.989</v>
+        <v>0.957</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F43" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.582</v>
+      </c>
+      <c r="F43" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2104,14 +2203,14 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>EACK-MY-ROX-WITH-TEA</t>
+          <t>DACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.968</v>
+        <v>0.947</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.518</v>
+        <v>0.374</v>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
@@ -2134,10 +2233,10 @@
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.979</v>
+        <v>0.968</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.725</v>
+        <v>0.731</v>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
@@ -2160,14 +2259,14 @@
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.985</v>
+        <v>0.967</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.698</v>
-      </c>
-      <c r="F46" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.859</v>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2186,10 +2285,10 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.971</v>
+        <v>0.968</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.549</v>
+        <v>0.764</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
@@ -2212,10 +2311,10 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.946</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.502</v>
+        <v>0.536</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
@@ -2238,10 +2337,10 @@
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.5</v>
+        <v>0.66</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2260,18 +2359,18 @@
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MACHTNE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.999</v>
+        <v>0.956</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.972</v>
-      </c>
-      <c r="F50" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.551</v>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2290,14 +2389,14 @@
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>0.992</v>
+        <v>0.964</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.857</v>
-      </c>
-      <c r="F51" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.651</v>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2316,10 +2415,10 @@
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="F52" s="20" t="inlineStr">
         <is>
@@ -2338,14 +2437,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>SYTHONPDPENUVAROBOT-</t>
+          <t>SYTHONPDPENUVRROBDT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.835</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.5</v>
+        <v>0.26</v>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
@@ -2368,14 +2467,14 @@
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>1</v>
+        <v>0.954</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="F54" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.708</v>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2394,10 +2493,10 @@
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.964</v>
+        <v>0.917</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.501</v>
+        <v>0.625</v>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
@@ -2416,14 +2515,14 @@
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SVSPEM-OM</t>
+          <t>ARTIFICIAL-SVSTEM-OK</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.969</v>
+        <v>0.912</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.5</v>
+        <v>0.376</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
@@ -2442,14 +2541,14 @@
       </c>
       <c r="C57" s="18" t="inlineStr">
         <is>
-          <t>HELLO-XOXLD-WELCOME-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.948</v>
+        <v>0.909</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.5</v>
+        <v>0.256</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
@@ -2468,14 +2567,14 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-FOWER--</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.958</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.551</v>
+        <v>0.617</v>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
@@ -2494,18 +2593,18 @@
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-EIND-GOLD</t>
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>1</v>
+        <v>0.952</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="F59" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.646</v>
+      </c>
+      <c r="F59" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2524,14 +2623,14 @@
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.993</v>
+        <v>0.946</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F60" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.447</v>
+      </c>
+      <c r="F60" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2550,10 +2649,10 @@
         </is>
       </c>
       <c r="D61" s="19" t="n">
-        <v>1</v>
+        <v>0.977</v>
       </c>
       <c r="E61" s="19" t="n">
-        <v>0.999</v>
+        <v>0.889</v>
       </c>
       <c r="F61" s="20" t="inlineStr">
         <is>
@@ -2572,18 +2671,18 @@
       </c>
       <c r="C62" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOX-</t>
+          <t>THE-QUICK-BROWN-EOX-</t>
         </is>
       </c>
       <c r="D62" s="15" t="n">
-        <v>1</v>
+        <v>0.961</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="F62" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.586</v>
+      </c>
+      <c r="F62" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2602,10 +2701,10 @@
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.976</v>
+        <v>0.971</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.517</v>
+        <v>0.695</v>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
@@ -2628,10 +2727,10 @@
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>0.959</v>
+        <v>0.964</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.531</v>
+        <v>0.661</v>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
@@ -2650,14 +2749,14 @@
       </c>
       <c r="C65" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOR-JU</t>
+          <t>EIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D65" s="19" t="n">
-        <v>1</v>
+        <v>0.982</v>
       </c>
       <c r="E65" s="19" t="n">
-        <v>1</v>
+        <v>0.85</v>
       </c>
       <c r="F65" s="20" t="inlineStr">
         <is>
@@ -2676,14 +2775,14 @@
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLACK-GEM-</t>
+          <t>SPHINX-OE-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>1</v>
+        <v>0.985</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.997</v>
+        <v>0.85</v>
       </c>
       <c r="F66" s="20" t="inlineStr">
         <is>
@@ -2706,14 +2805,14 @@
         </is>
       </c>
       <c r="D67" s="19" t="n">
-        <v>1</v>
+        <v>0.951</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>0.991</v>
-      </c>
-      <c r="F67" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.518</v>
+      </c>
+      <c r="F67" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2732,10 +2831,10 @@
         </is>
       </c>
       <c r="D68" s="15" t="n">
-        <v>1</v>
+        <v>0.988</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
       <c r="F68" s="20" t="inlineStr">
         <is>
@@ -2758,10 +2857,10 @@
         </is>
       </c>
       <c r="D69" s="19" t="n">
-        <v>0.998</v>
+        <v>0.976</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>0.962</v>
+        <v>0.843</v>
       </c>
       <c r="F69" s="20" t="inlineStr">
         <is>
@@ -2784,10 +2883,10 @@
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.996</v>
+        <v>0.983</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>0.917</v>
+        <v>0.833</v>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
@@ -2806,18 +2905,18 @@
       </c>
       <c r="C71" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEEP-NEURAL-NETNORKS</t>
         </is>
       </c>
       <c r="D71" s="19" t="n">
-        <v>1</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.474</v>
+      </c>
+      <c r="F71" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2836,10 +2935,10 @@
         </is>
       </c>
       <c r="D72" s="15" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>1</v>
+        <v>0.886</v>
       </c>
       <c r="F72" s="20" t="inlineStr">
         <is>
@@ -2862,10 +2961,10 @@
         </is>
       </c>
       <c r="D73" s="19" t="n">
-        <v>0.999</v>
+        <v>0.975</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.973</v>
+        <v>0.834</v>
       </c>
       <c r="F73" s="20" t="inlineStr">
         <is>
@@ -2888,10 +2987,10 @@
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>1</v>
+        <v>0.987</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>1</v>
+        <v>0.961</v>
       </c>
       <c r="F74" s="20" t="inlineStr">
         <is>
@@ -2914,10 +3013,10 @@
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>0.975</v>
+        <v>0.951</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>0.505</v>
+        <v>0.793</v>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
@@ -2940,7 +3039,7 @@
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.993</v>
+        <v>0.977</v>
       </c>
       <c r="E76" s="15" t="n">
         <v>0.85</v>
@@ -2966,10 +3065,10 @@
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>0.975</v>
+        <v>0.969</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>0.5</v>
+        <v>0.657</v>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
@@ -2992,14 +3091,14 @@
         </is>
       </c>
       <c r="D78" s="15" t="n">
-        <v>0.999</v>
+        <v>0.974</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>0.986</v>
-      </c>
-      <c r="F78" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.746</v>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3014,14 +3113,14 @@
       </c>
       <c r="C79" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>0.982</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E79" s="19" t="n">
-        <v>0.647</v>
+        <v>0.493</v>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
@@ -3044,10 +3143,10 @@
         </is>
       </c>
       <c r="D80" s="15" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>0.996</v>
+        <v>0.919</v>
       </c>
       <c r="F80" s="20" t="inlineStr">
         <is>
@@ -3066,18 +3165,18 @@
       </c>
       <c r="C81" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPQRST</t>
+          <t>ABCDEEGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D81" s="19" t="n">
-        <v>0.993</v>
+        <v>0.953</v>
       </c>
       <c r="E81" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F81" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.502</v>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3092,18 +3191,18 @@
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOX-</t>
+          <t>THE-QUTCK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>0.989</v>
+        <v>0.968</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.771</v>
-      </c>
-      <c r="F82" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="F82" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3221,7 @@
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>0.992</v>
+        <v>0.979</v>
       </c>
       <c r="E83" s="19" t="n">
         <v>0.85</v>
@@ -3148,10 +3247,10 @@
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>0.956</v>
+        <v>0.921</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>0.221</v>
+        <v>0.082</v>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
@@ -3174,10 +3273,10 @@
         </is>
       </c>
       <c r="D85" s="19" t="n">
-        <v>0.976</v>
+        <v>0.969</v>
       </c>
       <c r="E85" s="19" t="n">
-        <v>0.536</v>
+        <v>0.774</v>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
@@ -3200,14 +3299,14 @@
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>1</v>
+        <v>0.972</v>
       </c>
       <c r="E86" s="15" t="n">
-        <v>0.997</v>
-      </c>
-      <c r="F86" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.701</v>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3226,10 +3325,10 @@
         </is>
       </c>
       <c r="D87" s="19" t="n">
-        <v>1</v>
+        <v>0.981</v>
       </c>
       <c r="E87" s="19" t="n">
-        <v>1</v>
+        <v>0.897</v>
       </c>
       <c r="F87" s="20" t="inlineStr">
         <is>
@@ -3248,14 +3347,14 @@
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZYPHYRS-BLOW-</t>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.979</v>
+        <v>0.967</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.57</v>
+        <v>0.724</v>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
@@ -3278,10 +3377,10 @@
         </is>
       </c>
       <c r="D89" s="19" t="n">
-        <v>0.954</v>
+        <v>0.912</v>
       </c>
       <c r="E89" s="19" t="n">
-        <v>0.499</v>
+        <v>0.469</v>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
@@ -3304,14 +3403,14 @@
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="F90" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.55</v>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3330,10 +3429,10 @@
         </is>
       </c>
       <c r="D91" s="19" t="n">
-        <v>0.96</v>
+        <v>0.944</v>
       </c>
       <c r="E91" s="19" t="n">
-        <v>0.503</v>
+        <v>0.538</v>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
@@ -3356,10 +3455,10 @@
         </is>
       </c>
       <c r="D92" s="15" t="n">
-        <v>1</v>
+        <v>0.968</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.996</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F92" s="20" t="inlineStr">
         <is>
@@ -3382,14 +3481,14 @@
         </is>
       </c>
       <c r="D93" s="19" t="n">
-        <v>0.999</v>
+        <v>0.965</v>
       </c>
       <c r="E93" s="19" t="n">
-        <v>0.987</v>
-      </c>
-      <c r="F93" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6840000000000001</v>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3408,10 +3507,10 @@
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>0.963</v>
+        <v>0.945</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>0.5</v>
+        <v>0.6860000000000001</v>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
@@ -3434,10 +3533,10 @@
         </is>
       </c>
       <c r="D95" s="19" t="n">
-        <v>0.968</v>
+        <v>0.947</v>
       </c>
       <c r="E95" s="19" t="n">
-        <v>0.598</v>
+        <v>0.628</v>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
@@ -3456,14 +3555,14 @@
       </c>
       <c r="C96" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSTEM-OK</t>
+          <t>ARTIFTCIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>0.966</v>
+        <v>0.919</v>
       </c>
       <c r="E96" s="15" t="n">
-        <v>0.509</v>
+        <v>0.579</v>
       </c>
       <c r="F96" s="16" t="inlineStr">
         <is>
@@ -3482,14 +3581,14 @@
       </c>
       <c r="C97" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLO-NELCOMF-</t>
+          <t>HELLO-WORLO-WELCOME-</t>
         </is>
       </c>
       <c r="D97" s="19" t="n">
-        <v>0.976</v>
+        <v>0.906</v>
       </c>
       <c r="E97" s="19" t="n">
-        <v>0.679</v>
+        <v>0.533</v>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
@@ -3508,14 +3607,14 @@
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEOGE-IS-POUEF--</t>
+          <t>KNOWLEOGE-IS-PONEE--</t>
         </is>
       </c>
       <c r="D98" s="15" t="n">
-        <v>0.986</v>
+        <v>0.952</v>
       </c>
       <c r="E98" s="15" t="n">
-        <v>0.712</v>
+        <v>0.673</v>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
@@ -3534,14 +3633,14 @@
       </c>
       <c r="C99" s="18" t="inlineStr">
         <is>
-          <t>P-ND-EYTRA-FIND-GOLD</t>
+          <t>F-ND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.896</v>
       </c>
       <c r="E99" s="19" t="n">
-        <v>0.383</v>
+        <v>0.534</v>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
@@ -3564,10 +3663,10 @@
         </is>
       </c>
       <c r="D100" s="15" t="n">
-        <v>0.98</v>
+        <v>0.945</v>
       </c>
       <c r="E100" s="15" t="n">
-        <v>0.613</v>
+        <v>0.35</v>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
@@ -3590,10 +3689,10 @@
         </is>
       </c>
       <c r="D101" s="19" t="n">
-        <v>0.967</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E101" s="19" t="n">
-        <v>0.501</v>
+        <v>0.543</v>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
@@ -3612,14 +3711,14 @@
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>THE-QUTCK-BROWN-FOX-</t>
+          <t>THE-QUTCK-BROWN-EOX-</t>
         </is>
       </c>
       <c r="D102" s="15" t="n">
-        <v>0.962</v>
+        <v>0.927</v>
       </c>
       <c r="E102" s="15" t="n">
-        <v>0.5</v>
+        <v>0.491</v>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
@@ -3642,10 +3741,10 @@
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.976</v>
+        <v>0.959</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.53</v>
+        <v>0.61</v>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
@@ -3668,14 +3767,14 @@
         </is>
       </c>
       <c r="D104" s="15" t="n">
-        <v>1</v>
+        <v>0.968</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="F104" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="F104" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3694,14 +3793,14 @@
         </is>
       </c>
       <c r="D105" s="19" t="n">
-        <v>0.977</v>
+        <v>0.962</v>
       </c>
       <c r="E105" s="19" t="n">
-        <v>0.542</v>
-      </c>
-      <c r="F105" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.821</v>
+      </c>
+      <c r="F105" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3720,10 +3819,10 @@
         </is>
       </c>
       <c r="D106" s="15" t="n">
-        <v>0.974</v>
+        <v>0.949</v>
       </c>
       <c r="E106" s="15" t="n">
-        <v>0.5</v>
+        <v>0.611</v>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
@@ -3746,14 +3845,14 @@
         </is>
       </c>
       <c r="D107" s="19" t="n">
-        <v>0.95</v>
+        <v>0.968</v>
       </c>
       <c r="E107" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F107" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.825</v>
+      </c>
+      <c r="F107" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3768,14 +3867,14 @@
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZERHVRS-BLOW-</t>
+          <t>BRIGHT-ZEPHVRS-BLOW-</t>
         </is>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.918</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.524</v>
+        <v>0.694</v>
       </c>
       <c r="F108" s="16" t="inlineStr">
         <is>
@@ -3794,14 +3893,14 @@
       </c>
       <c r="C109" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VICION-TECT</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D109" s="19" t="n">
-        <v>0.925</v>
+        <v>0.958</v>
       </c>
       <c r="E109" s="19" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
@@ -3824,14 +3923,14 @@
         </is>
       </c>
       <c r="D110" s="15" t="n">
-        <v>0.988</v>
+        <v>0.984</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.751</v>
-      </c>
-      <c r="F110" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.917</v>
+      </c>
+      <c r="F110" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3850,14 +3949,14 @@
         </is>
       </c>
       <c r="D111" s="19" t="n">
-        <v>0.976</v>
+        <v>0.98</v>
       </c>
       <c r="E111" s="19" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="F111" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.831</v>
+      </c>
+      <c r="F111" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3876,14 +3975,14 @@
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.973</v>
+        <v>0.98</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.508</v>
-      </c>
-      <c r="F112" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.827</v>
+      </c>
+      <c r="F112" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3902,10 +4001,10 @@
         </is>
       </c>
       <c r="D113" s="19" t="n">
-        <v>0.977</v>
+        <v>0.973</v>
       </c>
       <c r="E113" s="19" t="n">
-        <v>0.543</v>
+        <v>0.739</v>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
@@ -3924,14 +4023,14 @@
       </c>
       <c r="C114" s="14" t="inlineStr">
         <is>
-          <t>SMPRT-OCP-RECOGNIZE-</t>
+          <t>SMART-OCP-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D114" s="15" t="n">
-        <v>0.973</v>
+        <v>0.966</v>
       </c>
       <c r="E114" s="15" t="n">
-        <v>0.479</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F114" s="16" t="inlineStr">
         <is>
@@ -3950,14 +4049,14 @@
       </c>
       <c r="C115" s="18" t="inlineStr">
         <is>
-          <t>ARCUDATE-PREDICTION-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D115" s="19" t="n">
-        <v>0.972</v>
+        <v>0.929</v>
       </c>
       <c r="E115" s="19" t="n">
-        <v>0.501</v>
+        <v>0.41</v>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
@@ -3980,10 +4079,10 @@
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.958</v>
+        <v>0.926</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.503</v>
+        <v>0.453</v>
       </c>
       <c r="F116" s="16" t="inlineStr">
         <is>
@@ -4002,14 +4101,14 @@
       </c>
       <c r="C117" s="18" t="inlineStr">
         <is>
-          <t>RELLO-WORLD-WELCONE-</t>
+          <t>RELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D117" s="19" t="n">
-        <v>0.975</v>
+        <v>0.945</v>
       </c>
       <c r="E117" s="19" t="n">
-        <v>0.504</v>
+        <v>0.466</v>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
@@ -4032,10 +4131,10 @@
         </is>
       </c>
       <c r="D118" s="15" t="n">
-        <v>1</v>
+        <v>0.986</v>
       </c>
       <c r="E118" s="15" t="n">
-        <v>1</v>
+        <v>0.944</v>
       </c>
       <c r="F118" s="20" t="inlineStr">
         <is>
@@ -4054,14 +4153,14 @@
       </c>
       <c r="C119" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-EIND-GOLD</t>
         </is>
       </c>
       <c r="D119" s="19" t="n">
-        <v>0.978</v>
+        <v>0.959</v>
       </c>
       <c r="E119" s="19" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.85</v>
       </c>
       <c r="F119" s="20" t="inlineStr">
         <is>
@@ -4084,10 +4183,10 @@
         </is>
       </c>
       <c r="D120" s="15" t="n">
-        <v>0.999</v>
+        <v>0.984</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>0.99</v>
+        <v>0.91</v>
       </c>
       <c r="F120" s="20" t="inlineStr">
         <is>
@@ -4106,23 +4205,1583 @@
       </c>
       <c r="C121" s="18" t="inlineStr">
         <is>
-          <t>ARCDEFGHIJKLMNOPORST</t>
+          <t>ARCDEEGHIJKLMNOPORST</t>
         </is>
       </c>
       <c r="D121" s="19" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="E121" s="19" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F121" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="20" customHeight="1">
+      <c r="A122" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B122" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-EOX-</t>
+        </is>
+      </c>
+      <c r="D122" s="15" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E122" s="15" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="F122" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="20" customHeight="1">
+      <c r="A123" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B123" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D123" s="19" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="E123" s="19" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="F123" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="20" customHeight="1">
+      <c r="A124" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B124" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOXDWITH-TEA</t>
+        </is>
+      </c>
+      <c r="D124" s="15" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="E124" s="15" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F124" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="20" customHeight="1">
+      <c r="A125" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B125" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" s="18" t="inlineStr">
+        <is>
+          <t>EIVE-DOZEN-LIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D125" s="19" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E125" s="19" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="F125" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B126" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C126" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OE-BLACK-CEM-</t>
+        </is>
+      </c>
+      <c r="D126" s="15" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="E126" s="15" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F126" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="20" customHeight="1">
+      <c r="A127" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B127" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C127" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MYUVOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D127" s="19" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E127" s="19" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="F127" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="20" customHeight="1">
+      <c r="A128" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B128" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C128" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS------</t>
+        </is>
+      </c>
+      <c r="D128" s="15" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="E128" s="15" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="F128" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="20" customHeight="1">
+      <c r="A129" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B129" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C129" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D129" s="19" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="E129" s="19" t="n">
+        <v>0.656</v>
+      </c>
+      <c r="F129" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="20" customHeight="1">
+      <c r="A130" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B130" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C130" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-CEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D130" s="15" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="E130" s="15" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="F130" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="20" customHeight="1">
+      <c r="A131" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B131" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C131" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAC-NETWORKO</t>
+        </is>
+      </c>
+      <c r="D131" s="19" t="n">
+        <v>0.912</v>
+      </c>
+      <c r="E131" s="19" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="F131" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="20" customHeight="1">
+      <c r="A132" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B132" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C132" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D132" s="15" t="n">
+        <v>0.955</v>
+      </c>
+      <c r="E132" s="15" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="F132" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="20" customHeight="1">
+      <c r="A133" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B133" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C133" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D133" s="19" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="E133" s="19" t="n">
+        <v>0.774</v>
+      </c>
+      <c r="F133" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="20" customHeight="1">
+      <c r="A134" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B134" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C134" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D134" s="15" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="E134" s="15" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="F134" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="20" customHeight="1">
+      <c r="A135" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B135" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C135" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTION-</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="E135" s="19" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="F135" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="20" customHeight="1">
+      <c r="A136" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B136" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C136" s="14" t="inlineStr">
+        <is>
+          <t>ARTIEICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D136" s="15" t="n">
+        <v>0.966</v>
+      </c>
+      <c r="E136" s="15" t="n">
+        <v>0.754</v>
+      </c>
+      <c r="F136" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="20" customHeight="1">
+      <c r="A137" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B137" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C137" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D137" s="19" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="E137" s="19" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="F137" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="20" customHeight="1">
+      <c r="A138" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B138" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C138" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POWER--</t>
+        </is>
+      </c>
+      <c r="D138" s="15" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="E138" s="15" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="F138" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="20" customHeight="1">
+      <c r="A139" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B139" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C139" s="18" t="inlineStr">
+        <is>
+          <t>EIND-EXTRA-EIND-GOLD</t>
+        </is>
+      </c>
+      <c r="D139" s="19" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="E139" s="19" t="n">
+        <v>0.517</v>
+      </c>
+      <c r="F139" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="13" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B140" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C140" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D140" s="15" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="E140" s="15" t="n">
+        <v>0.833</v>
+      </c>
+      <c r="F140" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="20" customHeight="1">
+      <c r="A141" s="17" t="inlineStr">
+        <is>
+          <t>test7.jpg</t>
+        </is>
+      </c>
+      <c r="B141" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C141" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D141" s="19" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="E141" s="19" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="F141" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="20" customHeight="1">
+      <c r="A142" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B142" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BRAWN-EOX-</t>
+        </is>
+      </c>
+      <c r="D142" s="15" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E142" s="15" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="F142" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="20" customHeight="1">
+      <c r="A143" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B143" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D143" s="19" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="E143" s="19" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="F143" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="20" customHeight="1">
+      <c r="A144" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B144" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C144" s="14" t="inlineStr">
+        <is>
+          <t>YACK-MY-BCXXWITH-TEA</t>
+        </is>
+      </c>
+      <c r="D144" s="15" t="n">
+        <v>0.874</v>
+      </c>
+      <c r="E144" s="15" t="n">
+        <v>0.146</v>
+      </c>
+      <c r="F144" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="20" customHeight="1">
+      <c r="A145" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B145" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C145" s="18" t="inlineStr">
+        <is>
+          <t>EIVE-DOZEN-LIQUOR-IU</t>
+        </is>
+      </c>
+      <c r="D145" s="19" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="E145" s="19" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="F145" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="20" customHeight="1">
+      <c r="A146" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B146" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C146" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OR-BLACK-GEP-</t>
+        </is>
+      </c>
+      <c r="D146" s="15" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="E146" s="15" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="F146" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="20" customHeight="1">
+      <c r="A147" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B147" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C147" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOWKQUICKLY</t>
+        </is>
+      </c>
+      <c r="D147" s="19" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="E147" s="19" t="n">
+        <v>0.168</v>
+      </c>
+      <c r="F147" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="20" customHeight="1">
+      <c r="A148" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B148" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C148" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D148" s="15" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="E148" s="15" t="n">
+        <v>0.302</v>
+      </c>
+      <c r="F148" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="20" customHeight="1">
+      <c r="A149" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B149" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C149" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D149" s="19" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="E149" s="19" t="n">
+        <v>0.572</v>
+      </c>
+      <c r="F149" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="20" customHeight="1">
+      <c r="A150" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B150" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C150" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D150" s="15" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="E150" s="15" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="F150" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="20" customHeight="1">
+      <c r="A151" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B151" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C151" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAI-NITMORKS</t>
+        </is>
+      </c>
+      <c r="D151" s="19" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="E151" s="19" t="n">
+        <v>0.417</v>
+      </c>
+      <c r="F151" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="20" customHeight="1">
+      <c r="A152" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B152" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C152" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D152" s="15" t="n">
+        <v>0.946</v>
+      </c>
+      <c r="E152" s="15" t="n">
+        <v>0.6860000000000001</v>
+      </c>
+      <c r="F152" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="20" customHeight="1">
+      <c r="A153" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B153" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C153" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENOV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D153" s="19" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="E153" s="19" t="n">
+        <v>0.664</v>
+      </c>
+      <c r="F153" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="20" customHeight="1">
+      <c r="A154" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B154" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C154" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D154" s="15" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="E154" s="15" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="F154" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="20" customHeight="1">
+      <c r="A155" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B155" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C155" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREIICTJOD-</t>
+        </is>
+      </c>
+      <c r="D155" s="19" t="n">
+        <v>0.897</v>
+      </c>
+      <c r="E155" s="19" t="n">
+        <v>0.339</v>
+      </c>
+      <c r="F155" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="20" customHeight="1">
+      <c r="A156" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B156" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C156" s="14" t="inlineStr">
+        <is>
+          <t>ARTIEICIALESYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D156" s="15" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="E156" s="15" t="n">
+        <v>0.418</v>
+      </c>
+      <c r="F156" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1">
+      <c r="A157" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B157" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C157" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D157" s="19" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="E157" s="19" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F157" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="20" customHeight="1">
+      <c r="A158" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B158" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C158" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POWER--</t>
+        </is>
+      </c>
+      <c r="D158" s="15" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="E158" s="15" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="F158" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="20" customHeight="1">
+      <c r="A159" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B159" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C159" s="18" t="inlineStr">
+        <is>
+          <t>EIND-EXTRA-FIND-QOID</t>
+        </is>
+      </c>
+      <c r="D159" s="19" t="n">
+        <v>0.914</v>
+      </c>
+      <c r="E159" s="19" t="n">
+        <v>0.346</v>
+      </c>
+      <c r="F159" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="20" customHeight="1">
+      <c r="A160" s="13" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B160" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C160" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D160" s="15" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="E160" s="15" t="n">
+        <v>0.893</v>
+      </c>
+      <c r="F160" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="20" customHeight="1">
+      <c r="A161" s="17" t="inlineStr">
+        <is>
+          <t>test8.jpg</t>
+        </is>
+      </c>
+      <c r="B161" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C161" s="18" t="inlineStr">
+        <is>
+          <t>ABODEFGHIJXLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D161" s="19" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E161" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F161" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="20" customHeight="1">
+      <c r="A162" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B162" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C162" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUIOK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D162" s="15" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="E162" s="15" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F162" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="20" customHeight="1">
+      <c r="A163" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B163" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C163" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D163" s="19" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E163" s="19" t="n">
+        <v>0.729</v>
+      </c>
+      <c r="F163" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="20" customHeight="1">
+      <c r="A164" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B164" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C164" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D164" s="15" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="E164" s="15" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="F164" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="20" customHeight="1">
+      <c r="A165" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B165" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C165" s="18" t="inlineStr">
+        <is>
+          <t>EIVE-DOZEN-LTQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D165" s="19" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="E165" s="19" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="F165" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="20" customHeight="1">
+      <c r="A166" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B166" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C166" s="14" t="inlineStr">
+        <is>
+          <t>PHINX-OE-BLACK-GEM--</t>
+        </is>
+      </c>
+      <c r="D166" s="15" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="E166" s="15" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="F166" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="20" customHeight="1">
+      <c r="A167" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B167" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C167" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D167" s="19" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="E167" s="19" t="n">
+        <v>0.614</v>
+      </c>
+      <c r="F167" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="20" customHeight="1">
+      <c r="A168" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B168" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C168" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHTEZEPHYRS-BIOW-</t>
+        </is>
+      </c>
+      <c r="D168" s="15" t="n">
+        <v>0.9350000000000001</v>
+      </c>
+      <c r="E168" s="15" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F168" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="20" customHeight="1">
+      <c r="A169" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B169" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C169" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TESI</t>
+        </is>
+      </c>
+      <c r="D169" s="19" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E169" s="19" t="n">
+        <v>0.785</v>
+      </c>
+      <c r="F169" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="20" customHeight="1">
+      <c r="A170" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B170" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C170" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D170" s="15" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="E170" s="15" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="F170" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="20" customHeight="1">
+      <c r="A171" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B171" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C171" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETKORKS</t>
+        </is>
+      </c>
+      <c r="D171" s="19" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="E171" s="19" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F171" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="20" customHeight="1">
+      <c r="A172" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B172" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C172" s="14" t="inlineStr">
+        <is>
+          <t>TMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D172" s="15" t="n">
         <v>0.9389999999999999</v>
       </c>
-      <c r="E121" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F121" s="16" t="inlineStr">
+      <c r="E172" s="15" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="F172" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="20" customHeight="1">
+      <c r="A173" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B173" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C173" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D173" s="19" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="E173" s="19" t="n">
+        <v>0.886</v>
+      </c>
+      <c r="F173" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="20" customHeight="1">
+      <c r="A174" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B174" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C174" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D174" s="15" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="E174" s="15" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F174" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="20" customHeight="1">
+      <c r="A175" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B175" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C175" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTION-</t>
+        </is>
+      </c>
+      <c r="D175" s="19" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="E175" s="19" t="n">
+        <v>0.786</v>
+      </c>
+      <c r="F175" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="20" customHeight="1">
+      <c r="A176" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B176" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C176" s="14" t="inlineStr">
+        <is>
+          <t>ARTIEICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D176" s="15" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="E176" s="15" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="F176" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="20" customHeight="1">
+      <c r="A177" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B177" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C177" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D177" s="19" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E177" s="19" t="n">
+        <v>0.9360000000000001</v>
+      </c>
+      <c r="F177" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="20" customHeight="1">
+      <c r="A178" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B178" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C178" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POKER--</t>
+        </is>
+      </c>
+      <c r="D178" s="15" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="E178" s="15" t="n">
+        <v>0.596</v>
+      </c>
+      <c r="F178" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="20" customHeight="1">
+      <c r="A179" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B179" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C179" s="18" t="inlineStr">
+        <is>
+          <t>EIND-EXTRA-FIND-GOLD</t>
+        </is>
+      </c>
+      <c r="D179" s="19" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="E179" s="19" t="n">
+        <v>0.662</v>
+      </c>
+      <c r="F179" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="20" customHeight="1">
+      <c r="A180" s="13" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B180" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C180" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D180" s="15" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E180" s="15" t="n">
+        <v>0.847</v>
+      </c>
+      <c r="F180" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="20" customHeight="1">
+      <c r="A181" s="17" t="inlineStr">
+        <is>
+          <t>test9.jpg</t>
+        </is>
+      </c>
+      <c r="B181" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C181" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D181" s="19" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="E181" s="19" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="F181" s="16" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F121"/>
+  <autoFilter ref="A1:F181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: achieve record 94.70% benchmark (3788/4000) with Quad Geometry, Hard Mining, and Early Stopping
- Implement Quad Geometry Perspective Warp Refinement in scan_and_predict.py (test9 jumps from 63.25% to 93.75%)
- Add Edge Fragment Filter and strict hollow box defense to prevent false 'I' detections in blank cells
- Fine-tune topological disambiguation thresholds for E vs F
- Implement train_hard_mining.py pipeline with Focal Loss and 8x hard sample augmentation
- Add Early Stopping support (--auto-stop, --patience) to train_model.py and train_cnn.py
- Expand benchmark from 9 sheets (3,600 cells) to 10 sheets (4,000 cells) reaching 94.70% (3,788/4,000)
- Update README.md and howtodo.md documentation with full benchmark, methodology, and usage guides
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -618,10 +618,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="132" customWidth="1" min="1" max="1"/>
+    <col width="133" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-20 13:29:05 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 9 แผ่น | รวม 180 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-25 20:33:42 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 10 แผ่น | รวม 200 ข้อ</t>
         </is>
       </c>
     </row>
@@ -676,27 +676,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>9 แผ่น</t>
+          <t>10 แผ่น</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>180 ข้อ</t>
+          <t>200 ข้อ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>3,600 ตัว</t>
+          <t>4,000 ตัว</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>94.03%</t>
+          <t>94.70%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>128 ข้อ</t>
+          <t>190 ข้อ</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>98.00%</t>
+          <t>98.75%</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.968</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>11 ข้อ</t>
+          <t>19 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>83.50%</t>
+          <t>86.50%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.869</t>
+          <t>0.815</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>95.25%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.946</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>17 ข้อ</t>
+          <t>19 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.970</t>
+          <t>0.905</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>10 ข้อ</t>
+          <t>19 ข้อ</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -892,17 +892,17 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>94.50%</t>
+          <t>94.25%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>0.947</t>
+          <t>0.891</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>16 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -925,17 +925,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>95.25%</t>
+          <t>96.50%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>0.957</t>
+          <t>0.899</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>12 ข้อ</t>
+          <t>18 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>95.75%</t>
+          <t>97.25%</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>0.965</t>
+          <t>0.924</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>11 ข้อ</t>
+          <t>18 ข้อ</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -991,17 +991,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>93.75%</t>
+          <t>96.00%</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>0.925</t>
+          <t>0.898</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>18 ข้อ</t>
+          <t>17 ข้อ</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1024,20 +1024,53 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>92.25%</t>
+          <t>93.75%</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>0.967</t>
+          <t>0.872</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>13 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>91.00%</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>0.859</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>20 ข้อ</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
         <is>
           <t>English &amp; Tech (ชุดที่ 1)</t>
         </is>
@@ -1057,10 +1090,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F181"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -1111,14 +1144,14 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-EOX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.961</v>
+        <v>0.916</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.747</v>
+        <v>0.579</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -1141,14 +1174,14 @@
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.982</v>
+        <v>0.917</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.362</v>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1167,10 +1200,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.968</v>
+        <v>0.926</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.734</v>
+        <v>0.589</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -1189,18 +1222,18 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LIQUOR-JU</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.957</v>
+        <v>0.919</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.8139999999999999</v>
-      </c>
-      <c r="F5" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.751</v>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1219,14 +1252,14 @@
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>0.983</v>
+        <v>0.95</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F6" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.791</v>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1245,14 +1278,14 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.972</v>
+        <v>0.915</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.869</v>
-      </c>
-      <c r="F7" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.644</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1271,14 +1304,14 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.99</v>
+        <v>0.951</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="F8" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.764</v>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1297,10 +1330,10 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>0.96</v>
+        <v>0.895</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.646</v>
+        <v>0.552</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
@@ -1323,10 +1356,10 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.974</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.638</v>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
@@ -1349,10 +1382,10 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.958</v>
+        <v>0.911</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.649</v>
+        <v>0.518</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -1371,14 +1404,14 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DEIECT-OK</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.944</v>
+        <v>0.88</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.605</v>
+        <v>0.48</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
@@ -1401,14 +1434,14 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.989</v>
+        <v>0.944</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.9350000000000001</v>
-      </c>
-      <c r="F13" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.762</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1427,14 +1460,14 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>0.984</v>
+        <v>0.924</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>0.898</v>
-      </c>
-      <c r="F14" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.719</v>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1453,10 +1486,10 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.966</v>
+        <v>0.909</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.792</v>
+        <v>0.739</v>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
@@ -1475,14 +1508,14 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICIAL-SYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.882</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.456</v>
+        <v>0.61</v>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
@@ -1501,18 +1534,18 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCOME-</t>
+          <t>HELLO-WORLD-WELOOME-</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.974</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.788</v>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1531,10 +1564,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.972</v>
+        <v>0.954</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.711</v>
+        <v>0.791</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
@@ -1553,18 +1586,18 @@
       </c>
       <c r="C19" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-EIND-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.957</v>
+        <v>0.895</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.829</v>
-      </c>
-      <c r="F19" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1583,10 +1616,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.964</v>
+        <v>0.911</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.614</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
@@ -1609,14 +1642,14 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.977</v>
+        <v>0.924</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F21" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.668</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1631,14 +1664,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>TIL-QUICK-BROWN-FQX-</t>
+          <t>TIL-QUICK-RROWN-FQX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.881</v>
+        <v>0.878</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.433</v>
+        <v>0.491</v>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
@@ -1657,14 +1690,14 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMMS-OVER-LAZY-CQG-</t>
+          <t>JUMPS-OVER-LAZY-IOG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.885</v>
+        <v>0.884</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.427</v>
+        <v>0.307</v>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
@@ -1683,14 +1716,14 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOX-WITH-TEA</t>
+          <t>PACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.961</v>
+        <v>0.924</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.745</v>
+        <v>0.478</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
@@ -1709,14 +1742,14 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LIQUQR-JV</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.856</v>
+        <v>0.847</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.449</v>
+        <v>0.403</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -1735,14 +1768,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHUNX-OE-BLACK-GEM-</t>
+          <t>SPHUNX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.905</v>
+        <v>0.858</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.487</v>
+        <v>0.372</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -1761,14 +1794,14 @@
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VOW-QVICKLY</t>
+          <t>JUDSE-MY-VOW-QVICKLY</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.908</v>
+        <v>0.844</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.533</v>
+        <v>0.59</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -1787,14 +1820,14 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>RR-GHI-LEPHYRS-ELOW-</t>
+          <t>RR-GHI-ZEPHYRS-ILOW-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.859</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.224</v>
+        <v>0.312</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
@@ -1813,14 +1846,14 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUIER-VISION-TESD</t>
+          <t>COMPUIER-VISION-TESE</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.893</v>
+        <v>0.863</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.223</v>
+        <v>0.331</v>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
@@ -1839,14 +1872,14 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHINEWLEARNING-AJ-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.908</v>
+        <v>0.881</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.282</v>
+        <v>0.482</v>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
@@ -1865,14 +1898,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAU-NFTMQRKS</t>
+          <t>DEEP-NEURAL-NFTWORWS</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.775</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.357</v>
+        <v>0.402</v>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
@@ -1891,14 +1924,14 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGE-DATA-DEZFCT-CK</t>
+          <t>-MASE-DATA-DEUFOT-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.744</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.29</v>
+        <v>0.309</v>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
@@ -1917,14 +1950,14 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYIHON-OPENCV-BOBCT-</t>
+          <t>DYIHON-OPENCV-BORCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.906</v>
+        <v>0.758</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.37</v>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
@@ -1943,14 +1976,14 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SMART-CCR-RECOGWIZE-</t>
+          <t>SMART-OCR-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.865</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.21</v>
+        <v>0.475</v>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
@@ -1969,14 +2002,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>ACCUKATF--REDICTJBN-</t>
+          <t>AOCURATF--REDIOTJEQ-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.847</v>
+        <v>0.679</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.337</v>
+        <v>0.314</v>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
@@ -1995,14 +2028,14 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICJAL-SYSTEM-CK</t>
+          <t>ARTIFICIAL-SYSTEM-CK</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.848</v>
+        <v>0.786</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.525</v>
+        <v>0.426</v>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
@@ -2021,14 +2054,14 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLC-WORLC-VELOCME-</t>
+          <t>HELLO-WORLD-ZELOOME-</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.877</v>
+        <v>0.773</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.412</v>
+        <v>0.314</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
@@ -2047,14 +2080,14 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KNOWLUCCEDIS-PQWEB--</t>
+          <t>KNOWL-OCFCIS-PQWER--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.826</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.14</v>
+        <v>0.477</v>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
@@ -2073,14 +2106,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>EIND-FXTRA-EINE-GDLD</t>
+          <t>FIND-FXTRA-EIND-GDLD</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.862</v>
+        <v>0.819</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.382</v>
+        <v>0.388</v>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
@@ -2099,14 +2132,14 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZERQ-ONF--WG-SIX-TEN</t>
+          <t>ZFRO-ONF--WG-SIX-TEN</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.825</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.355</v>
+        <v>0.385</v>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
@@ -2125,14 +2158,14 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKL-NCHGRQT</t>
+          <t>ABCDEFGHIJKL-NCPQRST</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.856</v>
+        <v>0.723</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.215</v>
+        <v>0.255</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
@@ -2155,10 +2188,10 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.974</v>
+        <v>0.915</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.734</v>
+        <v>0.617</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -2181,10 +2214,10 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.957</v>
+        <v>0.9</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.582</v>
+        <v>0.584</v>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
@@ -2203,14 +2236,14 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>DACK-MY-ROX-WITH-TEA</t>
+          <t>EACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.947</v>
+        <v>0.912</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.374</v>
+        <v>0.413</v>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
@@ -2233,7 +2266,7 @@
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.968</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="E45" s="19" t="n">
         <v>0.731</v>
@@ -2255,18 +2288,18 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLHCK-GEM-</t>
+          <t>SPHINX-OF-BLADK-GEM-</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.967</v>
+        <v>0.918</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.859</v>
-      </c>
-      <c r="F46" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.493</v>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2285,10 +2318,10 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.968</v>
+        <v>0.915</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.764</v>
+        <v>0.596</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
@@ -2311,10 +2344,10 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>0.946</v>
+        <v>0.931</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.536</v>
+        <v>0.596</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
@@ -2333,14 +2366,14 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TEST</t>
+          <t>DOMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.901</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.66</v>
+        <v>0.527</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2359,14 +2392,14 @@
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>MACHTNE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.956</v>
+        <v>0.962</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.551</v>
+        <v>0.734</v>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
@@ -2389,10 +2422,10 @@
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>0.964</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.651</v>
+        <v>0.6909999999999999</v>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
@@ -2411,18 +2444,18 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETEDT-OK</t>
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>0.989</v>
+        <v>0.91</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F52" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.763</v>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2437,14 +2470,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>SYTHONPDPENUVRROBDT-</t>
+          <t>PYTHONRDPENUVNROBOT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.835</v>
+        <v>0.771</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
@@ -2463,14 +2496,14 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>SMART-ORC-RECOGNIZE-</t>
+          <t>SMART-ORD-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>0.954</v>
+        <v>0.927</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.708</v>
+        <v>0.676</v>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
@@ -2489,14 +2522,14 @@
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTION-</t>
+          <t>ADCURATE-PREDIDTION-</t>
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.917</v>
+        <v>0.859</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.625</v>
+        <v>0.577</v>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
@@ -2515,14 +2548,14 @@
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SVSTEM-OK</t>
+          <t>ARTIFIDIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.912</v>
+        <v>0.856</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.376</v>
+        <v>0.413</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
@@ -2545,10 +2578,10 @@
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.909</v>
+        <v>0.881</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.256</v>
+        <v>0.452</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
@@ -2567,14 +2600,14 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWER--</t>
+          <t>KNOWLEDGE-IS-FOWER--</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.878</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.617</v>
+        <v>0.417</v>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
@@ -2593,14 +2626,14 @@
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-EIND-GOLD</t>
+          <t>FINP-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>0.952</v>
+        <v>0.877</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.646</v>
+        <v>0.36</v>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
@@ -2623,10 +2656,10 @@
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.946</v>
+        <v>0.898</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.447</v>
+        <v>0.519</v>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
@@ -2649,10 +2682,10 @@
         </is>
       </c>
       <c r="D61" s="19" t="n">
-        <v>0.977</v>
+        <v>0.926</v>
       </c>
       <c r="E61" s="19" t="n">
-        <v>0.889</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F61" s="20" t="inlineStr">
         <is>
@@ -2671,14 +2704,14 @@
       </c>
       <c r="C62" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-EOX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D62" s="15" t="n">
-        <v>0.961</v>
+        <v>0.916</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>0.586</v>
+        <v>0.503</v>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
@@ -2701,10 +2734,10 @@
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.971</v>
+        <v>0.911</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.695</v>
+        <v>0.609</v>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
@@ -2723,14 +2756,14 @@
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOX-WITH-TEA</t>
+          <t>PAOK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>0.964</v>
+        <v>0.896</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.661</v>
+        <v>0.475</v>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
@@ -2749,18 +2782,18 @@
       </c>
       <c r="C65" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LIQUOR-JU</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D65" s="19" t="n">
-        <v>0.982</v>
+        <v>0.916</v>
       </c>
       <c r="E65" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F65" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.722</v>
+      </c>
+      <c r="F65" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2775,18 +2808,18 @@
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OE-BLACK-GEM-</t>
+          <t>SPHINX-OF-BLAOK-GEM-</t>
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>0.985</v>
+        <v>0.95</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F66" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.799</v>
+      </c>
+      <c r="F66" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2801,14 +2834,14 @@
       </c>
       <c r="C67" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-NY-VOW-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D67" s="19" t="n">
-        <v>0.951</v>
+        <v>0.873</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>0.518</v>
+        <v>0.602</v>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
@@ -2831,14 +2864,14 @@
         </is>
       </c>
       <c r="D68" s="15" t="n">
-        <v>0.988</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F68" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.696</v>
+      </c>
+      <c r="F68" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2857,14 +2890,14 @@
         </is>
       </c>
       <c r="D69" s="19" t="n">
-        <v>0.976</v>
+        <v>0.895</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>0.843</v>
-      </c>
-      <c r="F69" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.655</v>
+      </c>
+      <c r="F69" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2879,14 +2912,14 @@
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MAOHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.983</v>
+        <v>0.967</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>0.833</v>
+        <v>0.85</v>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
@@ -2905,14 +2938,14 @@
       </c>
       <c r="C71" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETNORKS</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D71" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.906</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>0.474</v>
+        <v>0.596</v>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
@@ -2931,18 +2964,18 @@
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETEOT-OK</t>
         </is>
       </c>
       <c r="D72" s="15" t="n">
-        <v>0.975</v>
+        <v>0.909</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>0.886</v>
-      </c>
-      <c r="F72" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.718</v>
+      </c>
+      <c r="F72" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2961,14 +2994,14 @@
         </is>
       </c>
       <c r="D73" s="19" t="n">
-        <v>0.975</v>
+        <v>0.878</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.834</v>
-      </c>
-      <c r="F73" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.589</v>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2983,18 +3016,18 @@
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-RECOGNIZE-</t>
+          <t>SMART-OCR-REOOGNIZE-</t>
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>0.987</v>
+        <v>0.895</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>0.961</v>
-      </c>
-      <c r="F74" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.528</v>
+      </c>
+      <c r="F74" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3009,14 +3042,14 @@
       </c>
       <c r="C75" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTION-</t>
+          <t>ACCURATE-PREDIDTION-</t>
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>0.951</v>
+        <v>0.851</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>0.793</v>
+        <v>0.506</v>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
@@ -3035,18 +3068,18 @@
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICIAL-SYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.977</v>
+        <v>0.891</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F76" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.473</v>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3061,14 +3094,14 @@
       </c>
       <c r="C77" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCOME-</t>
+          <t>HELLO-WORLD-WELOOME-</t>
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>0.969</v>
+        <v>0.914</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>0.657</v>
+        <v>0.609</v>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
@@ -3087,14 +3120,14 @@
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWER--</t>
+          <t>KNOWKEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D78" s="15" t="n">
-        <v>0.974</v>
+        <v>0.898</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>0.746</v>
+        <v>0.267</v>
       </c>
       <c r="F78" s="16" t="inlineStr">
         <is>
@@ -3113,14 +3146,14 @@
       </c>
       <c r="C79" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.892</v>
       </c>
       <c r="E79" s="19" t="n">
-        <v>0.493</v>
+        <v>0.661</v>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
@@ -3143,14 +3176,14 @@
         </is>
       </c>
       <c r="D80" s="15" t="n">
-        <v>0.983</v>
+        <v>0.928</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>0.919</v>
-      </c>
-      <c r="F80" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.677</v>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3165,14 +3198,14 @@
       </c>
       <c r="C81" s="18" t="inlineStr">
         <is>
-          <t>ABCDEEGHIJKLMNOPQRST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D81" s="19" t="n">
-        <v>0.953</v>
+        <v>0.875</v>
       </c>
       <c r="E81" s="19" t="n">
-        <v>0.502</v>
+        <v>0.521</v>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
@@ -3191,18 +3224,18 @@
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>THE-QUTCK-BROWN-FOX-</t>
+          <t>THE-QUTDK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>0.968</v>
+        <v>0.919</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.8149999999999999</v>
-      </c>
-      <c r="F82" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.44</v>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3221,14 +3254,14 @@
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>0.979</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E83" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F83" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.538</v>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3243,14 +3276,14 @@
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>PACK-MYXBOX-WITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>0.921</v>
+        <v>0.913</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>0.082</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
@@ -3273,10 +3306,10 @@
         </is>
       </c>
       <c r="D85" s="19" t="n">
-        <v>0.969</v>
+        <v>0.913</v>
       </c>
       <c r="E85" s="19" t="n">
-        <v>0.774</v>
+        <v>0.544</v>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
@@ -3295,14 +3328,14 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>SPHJNX-OF-BLACK-GEM-</t>
+          <t>SPHJNX-OF-RLACK-GEM-</t>
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>0.972</v>
+        <v>0.892</v>
       </c>
       <c r="E86" s="15" t="n">
-        <v>0.701</v>
+        <v>0.504</v>
       </c>
       <c r="F86" s="16" t="inlineStr">
         <is>
@@ -3325,14 +3358,14 @@
         </is>
       </c>
       <c r="D87" s="19" t="n">
-        <v>0.981</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E87" s="19" t="n">
-        <v>0.897</v>
-      </c>
-      <c r="F87" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.735</v>
+      </c>
+      <c r="F87" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3351,10 +3384,10 @@
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.967</v>
+        <v>0.887</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.724</v>
+        <v>0.296</v>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
@@ -3373,14 +3406,14 @@
       </c>
       <c r="C89" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VIJTON-TEST</t>
+          <t>COMPUTER-VISTON-TEST</t>
         </is>
       </c>
       <c r="D89" s="19" t="n">
-        <v>0.912</v>
+        <v>0.847</v>
       </c>
       <c r="E89" s="19" t="n">
-        <v>0.469</v>
+        <v>0.475</v>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
@@ -3403,10 +3436,10 @@
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.835</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>0.55</v>
+        <v>0.38</v>
       </c>
       <c r="F90" s="16" t="inlineStr">
         <is>
@@ -3429,10 +3462,10 @@
         </is>
       </c>
       <c r="D91" s="19" t="n">
-        <v>0.944</v>
+        <v>0.914</v>
       </c>
       <c r="E91" s="19" t="n">
-        <v>0.538</v>
+        <v>0.626</v>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
@@ -3455,14 +3488,14 @@
         </is>
       </c>
       <c r="D92" s="15" t="n">
-        <v>0.968</v>
+        <v>0.879</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="F92" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="F92" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3481,10 +3514,10 @@
         </is>
       </c>
       <c r="D93" s="19" t="n">
-        <v>0.965</v>
+        <v>0.905</v>
       </c>
       <c r="E93" s="19" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.578</v>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
@@ -3503,14 +3536,14 @@
       </c>
       <c r="C94" s="14" t="inlineStr">
         <is>
-          <t>SMAR--OCR-RECOGNIZF-</t>
+          <t>SMART-OCR-RECOGNIZF-</t>
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>0.945</v>
+        <v>0.926</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.792</v>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
@@ -3533,10 +3566,10 @@
         </is>
       </c>
       <c r="D95" s="19" t="n">
-        <v>0.947</v>
+        <v>0.851</v>
       </c>
       <c r="E95" s="19" t="n">
-        <v>0.628</v>
+        <v>0.485</v>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
@@ -3559,10 +3592,10 @@
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>0.919</v>
+        <v>0.854</v>
       </c>
       <c r="E96" s="15" t="n">
-        <v>0.579</v>
+        <v>0.368</v>
       </c>
       <c r="F96" s="16" t="inlineStr">
         <is>
@@ -3581,14 +3614,14 @@
       </c>
       <c r="C97" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLO-WELCOME-</t>
+          <t>HELIO-WORLO-WELCOMF-</t>
         </is>
       </c>
       <c r="D97" s="19" t="n">
-        <v>0.906</v>
+        <v>0.891</v>
       </c>
       <c r="E97" s="19" t="n">
-        <v>0.533</v>
+        <v>0.53</v>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
@@ -3607,14 +3640,14 @@
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEOGE-IS-PONEE--</t>
+          <t>KNOWLEOGE-IS-PONEF--</t>
         </is>
       </c>
       <c r="D98" s="15" t="n">
-        <v>0.952</v>
+        <v>0.898</v>
       </c>
       <c r="E98" s="15" t="n">
-        <v>0.673</v>
+        <v>0.424</v>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
@@ -3637,10 +3670,10 @@
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.896</v>
+        <v>0.832</v>
       </c>
       <c r="E99" s="19" t="n">
-        <v>0.534</v>
+        <v>0.415</v>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
@@ -3659,14 +3692,14 @@
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TRN</t>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D100" s="15" t="n">
-        <v>0.945</v>
+        <v>0.911</v>
       </c>
       <c r="E100" s="15" t="n">
-        <v>0.35</v>
+        <v>0.449</v>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
@@ -3685,14 +3718,14 @@
       </c>
       <c r="C101" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPQRST</t>
+          <t>ABNDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D101" s="19" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.873</v>
       </c>
       <c r="E101" s="19" t="n">
-        <v>0.543</v>
+        <v>0.268</v>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
@@ -3711,14 +3744,14 @@
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>THE-QUTCK-BROWN-EOX-</t>
+          <t>THE-QUTCK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D102" s="15" t="n">
-        <v>0.927</v>
+        <v>0.862</v>
       </c>
       <c r="E102" s="15" t="n">
-        <v>0.491</v>
+        <v>0.497</v>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
@@ -3741,10 +3774,10 @@
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.959</v>
+        <v>0.901</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.61</v>
+        <v>0.615</v>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
@@ -3767,10 +3800,10 @@
         </is>
       </c>
       <c r="D104" s="15" t="n">
-        <v>0.968</v>
+        <v>0.931</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.592</v>
       </c>
       <c r="F104" s="16" t="inlineStr">
         <is>
@@ -3793,14 +3826,14 @@
         </is>
       </c>
       <c r="D105" s="19" t="n">
-        <v>0.962</v>
+        <v>0.893</v>
       </c>
       <c r="E105" s="19" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="F105" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.578</v>
+      </c>
+      <c r="F105" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3815,14 +3848,14 @@
       </c>
       <c r="C106" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BUACK-GEM-</t>
+          <t>SPHINX-OF-BIACK-GEM-</t>
         </is>
       </c>
       <c r="D106" s="15" t="n">
-        <v>0.949</v>
+        <v>0.918</v>
       </c>
       <c r="E106" s="15" t="n">
-        <v>0.611</v>
+        <v>0.669</v>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
@@ -3845,14 +3878,14 @@
         </is>
       </c>
       <c r="D107" s="19" t="n">
-        <v>0.968</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E107" s="19" t="n">
-        <v>0.825</v>
-      </c>
-      <c r="F107" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.549</v>
+      </c>
+      <c r="F107" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3867,18 +3900,18 @@
       </c>
       <c r="C108" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZEPHVRS-BLOW-</t>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
         </is>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.694</v>
-      </c>
-      <c r="F108" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="F108" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3897,10 +3930,10 @@
         </is>
       </c>
       <c r="D109" s="19" t="n">
-        <v>0.958</v>
+        <v>0.918</v>
       </c>
       <c r="E109" s="19" t="n">
-        <v>0.75</v>
+        <v>0.662</v>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
@@ -3923,10 +3956,10 @@
         </is>
       </c>
       <c r="D110" s="15" t="n">
-        <v>0.984</v>
+        <v>0.972</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.917</v>
+        <v>0.834</v>
       </c>
       <c r="F110" s="20" t="inlineStr">
         <is>
@@ -3949,14 +3982,14 @@
         </is>
       </c>
       <c r="D111" s="19" t="n">
-        <v>0.98</v>
+        <v>0.949</v>
       </c>
       <c r="E111" s="19" t="n">
-        <v>0.831</v>
-      </c>
-      <c r="F111" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.72</v>
+      </c>
+      <c r="F111" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3971,18 +4004,18 @@
       </c>
       <c r="C112" s="14" t="inlineStr">
         <is>
-          <t>TMAG--DATA-DETECT-OK</t>
+          <t>TMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.98</v>
+        <v>0.884</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.827</v>
-      </c>
-      <c r="F112" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.55</v>
+      </c>
+      <c r="F112" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3997,14 +4030,14 @@
       </c>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>P-THON-OPENCV-ROBOT-</t>
+          <t>PYTHON-OPENDV-ROBOT-</t>
         </is>
       </c>
       <c r="D113" s="19" t="n">
-        <v>0.973</v>
+        <v>0.896</v>
       </c>
       <c r="E113" s="19" t="n">
-        <v>0.739</v>
+        <v>0.516</v>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
@@ -4027,10 +4060,10 @@
         </is>
       </c>
       <c r="D114" s="15" t="n">
-        <v>0.966</v>
+        <v>0.884</v>
       </c>
       <c r="E114" s="15" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.672</v>
       </c>
       <c r="F114" s="16" t="inlineStr">
         <is>
@@ -4049,14 +4082,14 @@
       </c>
       <c r="C115" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTION-</t>
+          <t>AOCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D115" s="19" t="n">
-        <v>0.929</v>
+        <v>0.847</v>
       </c>
       <c r="E115" s="19" t="n">
-        <v>0.41</v>
+        <v>0.454</v>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
@@ -4079,10 +4112,10 @@
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.926</v>
+        <v>0.805</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.453</v>
+        <v>0.377</v>
       </c>
       <c r="F116" s="16" t="inlineStr">
         <is>
@@ -4101,14 +4134,14 @@
       </c>
       <c r="C117" s="18" t="inlineStr">
         <is>
-          <t>RELLO-WORLD-WELCOME-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D117" s="19" t="n">
-        <v>0.945</v>
+        <v>0.885</v>
       </c>
       <c r="E117" s="19" t="n">
-        <v>0.466</v>
+        <v>0.576</v>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
@@ -4131,14 +4164,14 @@
         </is>
       </c>
       <c r="D118" s="15" t="n">
-        <v>0.986</v>
+        <v>0.911</v>
       </c>
       <c r="E118" s="15" t="n">
-        <v>0.944</v>
-      </c>
-      <c r="F118" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.58</v>
+      </c>
+      <c r="F118" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4153,18 +4186,18 @@
       </c>
       <c r="C119" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-EIND-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D119" s="19" t="n">
-        <v>0.959</v>
+        <v>0.886</v>
       </c>
       <c r="E119" s="19" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F119" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.632</v>
+      </c>
+      <c r="F119" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4183,14 +4216,14 @@
         </is>
       </c>
       <c r="D120" s="15" t="n">
-        <v>0.984</v>
+        <v>0.923</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="F120" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.627</v>
+      </c>
+      <c r="F120" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4205,14 +4238,14 @@
       </c>
       <c r="C121" s="18" t="inlineStr">
         <is>
-          <t>ARCDEEGHIJKLMNOPORST</t>
+          <t>ABDDEFGHIJKTMNOPORST</t>
         </is>
       </c>
       <c r="D121" s="19" t="n">
-        <v>0.901</v>
+        <v>0.832</v>
       </c>
       <c r="E121" s="19" t="n">
-        <v>0.42</v>
+        <v>0.347</v>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
@@ -4231,18 +4264,18 @@
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-EOX-</t>
+          <t>THE-QUIOK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D122" s="15" t="n">
-        <v>0.976</v>
+        <v>0.927</v>
       </c>
       <c r="E122" s="15" t="n">
-        <v>0.838</v>
-      </c>
-      <c r="F122" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.637</v>
+      </c>
+      <c r="F122" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4261,14 +4294,14 @@
         </is>
       </c>
       <c r="D123" s="19" t="n">
-        <v>0.984</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E123" s="19" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F123" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.548</v>
+      </c>
+      <c r="F123" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4283,18 +4316,18 @@
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOXDWITH-TEA</t>
+          <t>PAOK-MY-BOXNWITH-TEA</t>
         </is>
       </c>
       <c r="D124" s="15" t="n">
-        <v>0.986</v>
+        <v>0.919</v>
       </c>
       <c r="E124" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F124" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.233</v>
+      </c>
+      <c r="F124" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4309,18 +4342,18 @@
       </c>
       <c r="C125" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LIQUOR-JU</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D125" s="19" t="n">
-        <v>0.976</v>
+        <v>0.926</v>
       </c>
       <c r="E125" s="19" t="n">
-        <v>0.842</v>
-      </c>
-      <c r="F125" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.592</v>
+      </c>
+      <c r="F125" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4335,14 +4368,14 @@
       </c>
       <c r="C126" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OE-BLACK-CEM-</t>
+          <t>SPHINX-OF-BLACK-OEM-</t>
         </is>
       </c>
       <c r="D126" s="15" t="n">
-        <v>0.967</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E126" s="15" t="n">
-        <v>0.79</v>
+        <v>0.651</v>
       </c>
       <c r="F126" s="16" t="inlineStr">
         <is>
@@ -4365,14 +4398,14 @@
         </is>
       </c>
       <c r="D127" s="19" t="n">
-        <v>0.976</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E127" s="19" t="n">
-        <v>0.8070000000000001</v>
-      </c>
-      <c r="F127" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.74</v>
+      </c>
+      <c r="F127" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4391,10 +4424,10 @@
         </is>
       </c>
       <c r="D128" s="15" t="n">
-        <v>0.994</v>
+        <v>0.968</v>
       </c>
       <c r="E128" s="15" t="n">
-        <v>0.959</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="F128" s="20" t="inlineStr">
         <is>
@@ -4417,10 +4450,10 @@
         </is>
       </c>
       <c r="D129" s="19" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.907</v>
       </c>
       <c r="E129" s="19" t="n">
-        <v>0.656</v>
+        <v>0.674</v>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
@@ -4439,18 +4472,18 @@
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-CEARNING-AI-</t>
+          <t>MAOHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D130" s="15" t="n">
-        <v>0.947</v>
+        <v>0.96</v>
       </c>
       <c r="E130" s="15" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="F130" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.85</v>
+      </c>
+      <c r="F130" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4465,14 +4498,14 @@
       </c>
       <c r="C131" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAC-NETWORKO</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D131" s="19" t="n">
-        <v>0.912</v>
+        <v>0.885</v>
       </c>
       <c r="E131" s="19" t="n">
-        <v>0.333</v>
+        <v>0.361</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -4495,10 +4528,10 @@
         </is>
       </c>
       <c r="D132" s="15" t="n">
-        <v>0.955</v>
+        <v>0.893</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>0.451</v>
+        <v>0.607</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -4521,10 +4554,10 @@
         </is>
       </c>
       <c r="D133" s="19" t="n">
-        <v>0.966</v>
+        <v>0.912</v>
       </c>
       <c r="E133" s="19" t="n">
-        <v>0.774</v>
+        <v>0.696</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
@@ -4547,14 +4580,14 @@
         </is>
       </c>
       <c r="D134" s="15" t="n">
-        <v>0.986</v>
+        <v>0.946</v>
       </c>
       <c r="E134" s="15" t="n">
-        <v>0.913</v>
-      </c>
-      <c r="F134" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6830000000000001</v>
+      </c>
+      <c r="F134" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4573,14 +4606,14 @@
         </is>
       </c>
       <c r="D135" s="19" t="n">
-        <v>0.984</v>
+        <v>0.9320000000000001</v>
       </c>
       <c r="E135" s="19" t="n">
-        <v>0.865</v>
-      </c>
-      <c r="F135" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.71</v>
+      </c>
+      <c r="F135" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4595,14 +4628,14 @@
       </c>
       <c r="C136" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICIAL-SYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D136" s="15" t="n">
-        <v>0.966</v>
+        <v>0.889</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>0.754</v>
+        <v>0.484</v>
       </c>
       <c r="F136" s="16" t="inlineStr">
         <is>
@@ -4625,10 +4658,10 @@
         </is>
       </c>
       <c r="D137" s="19" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E137" s="19" t="n">
-        <v>0.516</v>
+        <v>0.748</v>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
@@ -4651,10 +4684,10 @@
         </is>
       </c>
       <c r="D138" s="15" t="n">
-        <v>0.957</v>
+        <v>0.921</v>
       </c>
       <c r="E138" s="15" t="n">
-        <v>0.616</v>
+        <v>0.414</v>
       </c>
       <c r="F138" s="16" t="inlineStr">
         <is>
@@ -4673,14 +4706,14 @@
       </c>
       <c r="C139" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-EIND-GOLD</t>
+          <t>FIND-EXTRA-FINP-GOLD</t>
         </is>
       </c>
       <c r="D139" s="19" t="n">
-        <v>0.949</v>
+        <v>0.892</v>
       </c>
       <c r="E139" s="19" t="n">
-        <v>0.517</v>
+        <v>0.374</v>
       </c>
       <c r="F139" s="16" t="inlineStr">
         <is>
@@ -4703,14 +4736,14 @@
         </is>
       </c>
       <c r="D140" s="15" t="n">
-        <v>0.981</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E140" s="15" t="n">
-        <v>0.833</v>
-      </c>
-      <c r="F140" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.712</v>
+      </c>
+      <c r="F140" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4729,10 +4762,10 @@
         </is>
       </c>
       <c r="D141" s="19" t="n">
-        <v>0.961</v>
+        <v>0.913</v>
       </c>
       <c r="E141" s="19" t="n">
-        <v>0.667</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="F141" s="16" t="inlineStr">
         <is>
@@ -4751,14 +4784,14 @@
       </c>
       <c r="C142" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BRAWN-EOX-</t>
+          <t>TPE-QUICK-BRAWN-FOX-</t>
         </is>
       </c>
       <c r="D142" s="15" t="n">
-        <v>0.882</v>
+        <v>0.844</v>
       </c>
       <c r="E142" s="15" t="n">
-        <v>0.386</v>
+        <v>0.236</v>
       </c>
       <c r="F142" s="16" t="inlineStr">
         <is>
@@ -4777,14 +4810,14 @@
       </c>
       <c r="C143" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>JUMPS-OVER-IAZY-DOG-</t>
         </is>
       </c>
       <c r="D143" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.886</v>
       </c>
       <c r="E143" s="19" t="n">
-        <v>0.575</v>
+        <v>0.413</v>
       </c>
       <c r="F143" s="16" t="inlineStr">
         <is>
@@ -4803,14 +4836,14 @@
       </c>
       <c r="C144" s="14" t="inlineStr">
         <is>
-          <t>YACK-MY-BCXXWITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D144" s="15" t="n">
-        <v>0.874</v>
+        <v>0.863</v>
       </c>
       <c r="E144" s="15" t="n">
-        <v>0.146</v>
+        <v>0.431</v>
       </c>
       <c r="F144" s="16" t="inlineStr">
         <is>
@@ -4829,14 +4862,14 @@
       </c>
       <c r="C145" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LIQUOR-IU</t>
+          <t>FIVE-DOZEN-LIQUOR-IU</t>
         </is>
       </c>
       <c r="D145" s="19" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.893</v>
       </c>
       <c r="E145" s="19" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.497</v>
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
@@ -4855,14 +4888,14 @@
       </c>
       <c r="C146" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OR-BLACK-GEP-</t>
+          <t>SPHINX-OR-BLAOK-GES-</t>
         </is>
       </c>
       <c r="D146" s="15" t="n">
-        <v>0.921</v>
+        <v>0.87</v>
       </c>
       <c r="E146" s="15" t="n">
-        <v>0.23</v>
+        <v>0.287</v>
       </c>
       <c r="F146" s="16" t="inlineStr">
         <is>
@@ -4881,14 +4914,14 @@
       </c>
       <c r="C147" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VOWKQUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D147" s="19" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E147" s="19" t="n">
-        <v>0.168</v>
+        <v>0.792</v>
       </c>
       <c r="F147" s="16" t="inlineStr">
         <is>
@@ -4911,10 +4944,10 @@
         </is>
       </c>
       <c r="D148" s="15" t="n">
-        <v>0.906</v>
+        <v>0.931</v>
       </c>
       <c r="E148" s="15" t="n">
-        <v>0.302</v>
+        <v>0.605</v>
       </c>
       <c r="F148" s="16" t="inlineStr">
         <is>
@@ -4937,10 +4970,10 @@
         </is>
       </c>
       <c r="D149" s="19" t="n">
-        <v>0.957</v>
+        <v>0.91</v>
       </c>
       <c r="E149" s="19" t="n">
-        <v>0.572</v>
+        <v>0.663</v>
       </c>
       <c r="F149" s="16" t="inlineStr">
         <is>
@@ -4959,18 +4992,18 @@
       </c>
       <c r="C150" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MAOHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D150" s="15" t="n">
-        <v>0.944</v>
+        <v>0.948</v>
       </c>
       <c r="E150" s="15" t="n">
-        <v>0.582</v>
-      </c>
-      <c r="F150" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="F150" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4985,14 +5018,14 @@
       </c>
       <c r="C151" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAI-NITMORKS</t>
+          <t>DEEP-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D151" s="19" t="n">
-        <v>0.871</v>
+        <v>0.882</v>
       </c>
       <c r="E151" s="19" t="n">
-        <v>0.417</v>
+        <v>0.592</v>
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
@@ -5015,10 +5048,10 @@
         </is>
       </c>
       <c r="D152" s="15" t="n">
-        <v>0.946</v>
+        <v>0.875</v>
       </c>
       <c r="E152" s="15" t="n">
-        <v>0.6860000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="F152" s="16" t="inlineStr">
         <is>
@@ -5037,14 +5070,14 @@
       </c>
       <c r="C153" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENOV-ROBOT-</t>
+          <t>PYTHON-OPENDV-ROBOT-</t>
         </is>
       </c>
       <c r="D153" s="19" t="n">
-        <v>0.944</v>
+        <v>0.911</v>
       </c>
       <c r="E153" s="19" t="n">
-        <v>0.664</v>
+        <v>0.539</v>
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
@@ -5063,14 +5096,14 @@
       </c>
       <c r="C154" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-RECOGNIZE-</t>
+          <t>SMART-OCR-REOOGNIZE-</t>
         </is>
       </c>
       <c r="D154" s="15" t="n">
-        <v>0.975</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E154" s="15" t="n">
-        <v>0.862</v>
+        <v>0.821</v>
       </c>
       <c r="F154" s="20" t="inlineStr">
         <is>
@@ -5089,14 +5122,14 @@
       </c>
       <c r="C155" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREIICTJOD-</t>
+          <t>ACCURATE-PREDIOTJON-</t>
         </is>
       </c>
       <c r="D155" s="19" t="n">
-        <v>0.897</v>
+        <v>0.854</v>
       </c>
       <c r="E155" s="19" t="n">
-        <v>0.339</v>
+        <v>0.368</v>
       </c>
       <c r="F155" s="16" t="inlineStr">
         <is>
@@ -5115,14 +5148,14 @@
       </c>
       <c r="C156" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICIALESYSTEM-OK</t>
+          <t>ARTIFICIALESYSTEM-OK</t>
         </is>
       </c>
       <c r="D156" s="15" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.912</v>
       </c>
       <c r="E156" s="15" t="n">
-        <v>0.418</v>
+        <v>0.46</v>
       </c>
       <c r="F156" s="16" t="inlineStr">
         <is>
@@ -5145,10 +5178,10 @@
         </is>
       </c>
       <c r="D157" s="19" t="n">
-        <v>0.928</v>
+        <v>0.905</v>
       </c>
       <c r="E157" s="19" t="n">
-        <v>0.58</v>
+        <v>0.595</v>
       </c>
       <c r="F157" s="16" t="inlineStr">
         <is>
@@ -5171,10 +5204,10 @@
         </is>
       </c>
       <c r="D158" s="15" t="n">
-        <v>0.931</v>
+        <v>0.923</v>
       </c>
       <c r="E158" s="15" t="n">
-        <v>0.522</v>
+        <v>0.704</v>
       </c>
       <c r="F158" s="16" t="inlineStr">
         <is>
@@ -5193,14 +5226,14 @@
       </c>
       <c r="C159" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-QOID</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D159" s="19" t="n">
-        <v>0.914</v>
+        <v>0.867</v>
       </c>
       <c r="E159" s="19" t="n">
-        <v>0.346</v>
+        <v>0.5</v>
       </c>
       <c r="F159" s="16" t="inlineStr">
         <is>
@@ -5223,10 +5256,10 @@
         </is>
       </c>
       <c r="D160" s="15" t="n">
-        <v>0.984</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E160" s="15" t="n">
-        <v>0.893</v>
+        <v>0.837</v>
       </c>
       <c r="F160" s="20" t="inlineStr">
         <is>
@@ -5245,14 +5278,14 @@
       </c>
       <c r="C161" s="18" t="inlineStr">
         <is>
-          <t>ABODEFGHIJXLMNOPQRST</t>
+          <t>ABODEFQHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D161" s="19" t="n">
-        <v>0.882</v>
+        <v>0.853</v>
       </c>
       <c r="E161" s="19" t="n">
-        <v>0.5</v>
+        <v>0.425</v>
       </c>
       <c r="F161" s="16" t="inlineStr">
         <is>
@@ -5271,18 +5304,18 @@
       </c>
       <c r="C162" s="14" t="inlineStr">
         <is>
-          <t>THE-QUIOK-BROWN-FOX-</t>
+          <t>IHE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D162" s="15" t="n">
-        <v>0.979</v>
+        <v>0.898</v>
       </c>
       <c r="E162" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F162" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.5659999999999999</v>
+      </c>
+      <c r="F162" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5297,14 +5330,14 @@
       </c>
       <c r="C163" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>IUMPS-OVER-LAZY-OOG-</t>
         </is>
       </c>
       <c r="D163" s="19" t="n">
-        <v>0.976</v>
+        <v>0.911</v>
       </c>
       <c r="E163" s="19" t="n">
-        <v>0.729</v>
+        <v>0.486</v>
       </c>
       <c r="F163" s="16" t="inlineStr">
         <is>
@@ -5327,14 +5360,14 @@
         </is>
       </c>
       <c r="D164" s="15" t="n">
-        <v>0.987</v>
+        <v>0.926</v>
       </c>
       <c r="E164" s="15" t="n">
-        <v>0.922</v>
-      </c>
-      <c r="F164" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.661</v>
+      </c>
+      <c r="F164" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5349,14 +5382,14 @@
       </c>
       <c r="C165" s="18" t="inlineStr">
         <is>
-          <t>EIVE-DOZEN-LTQUOR-JU</t>
+          <t>FJVE-DOZEN-LIQUOR-IU</t>
         </is>
       </c>
       <c r="D165" s="19" t="n">
-        <v>0.961</v>
+        <v>0.871</v>
       </c>
       <c r="E165" s="19" t="n">
-        <v>0.627</v>
+        <v>0.536</v>
       </c>
       <c r="F165" s="16" t="inlineStr">
         <is>
@@ -5375,14 +5408,14 @@
       </c>
       <c r="C166" s="14" t="inlineStr">
         <is>
-          <t>PHINX-OE-BLACK-GEM--</t>
+          <t>SPHINX-OT-RLACK-GEM-</t>
         </is>
       </c>
       <c r="D166" s="15" t="n">
-        <v>0.972</v>
+        <v>0.88</v>
       </c>
       <c r="E166" s="15" t="n">
-        <v>0.718</v>
+        <v>0.351</v>
       </c>
       <c r="F166" s="16" t="inlineStr">
         <is>
@@ -5401,14 +5434,14 @@
       </c>
       <c r="C167" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VOW-QUICKLY</t>
+          <t>IUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D167" s="19" t="n">
-        <v>0.961</v>
+        <v>0.853</v>
       </c>
       <c r="E167" s="19" t="n">
-        <v>0.614</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="F167" s="16" t="inlineStr">
         <is>
@@ -5427,14 +5460,14 @@
       </c>
       <c r="C168" s="14" t="inlineStr">
         <is>
-          <t>BRIGHTEZEPHYRS-BIOW-</t>
+          <t>BRZGHT-ZFPHYRS-RLOW-</t>
         </is>
       </c>
       <c r="D168" s="15" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.839</v>
       </c>
       <c r="E168" s="15" t="n">
-        <v>0.31</v>
+        <v>0.43</v>
       </c>
       <c r="F168" s="16" t="inlineStr">
         <is>
@@ -5453,14 +5486,14 @@
       </c>
       <c r="C169" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TESI</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D169" s="19" t="n">
-        <v>0.97</v>
+        <v>0.868</v>
       </c>
       <c r="E169" s="19" t="n">
-        <v>0.785</v>
+        <v>0.599</v>
       </c>
       <c r="F169" s="16" t="inlineStr">
         <is>
@@ -5483,10 +5516,10 @@
         </is>
       </c>
       <c r="D170" s="15" t="n">
-        <v>0.971</v>
+        <v>0.924</v>
       </c>
       <c r="E170" s="15" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.601</v>
       </c>
       <c r="F170" s="16" t="inlineStr">
         <is>
@@ -5505,18 +5538,18 @@
       </c>
       <c r="C171" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETKORKS</t>
+          <t>DEER-NQURAL-NETWORXS</t>
         </is>
       </c>
       <c r="D171" s="19" t="n">
-        <v>0.969</v>
+        <v>0.851</v>
       </c>
       <c r="E171" s="19" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="F171" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.278</v>
+      </c>
+      <c r="F171" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5531,14 +5564,14 @@
       </c>
       <c r="C172" s="14" t="inlineStr">
         <is>
-          <t>TMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D172" s="15" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.838</v>
       </c>
       <c r="E172" s="15" t="n">
-        <v>0.533</v>
+        <v>0.463</v>
       </c>
       <c r="F172" s="16" t="inlineStr">
         <is>
@@ -5557,18 +5590,18 @@
       </c>
       <c r="C173" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENCV-ROBOT-</t>
+          <t>PYTHON-OPENCV-ROROT-</t>
         </is>
       </c>
       <c r="D173" s="19" t="n">
-        <v>0.981</v>
+        <v>0.884</v>
       </c>
       <c r="E173" s="19" t="n">
-        <v>0.886</v>
-      </c>
-      <c r="F173" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.385</v>
+      </c>
+      <c r="F173" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5587,14 +5620,14 @@
         </is>
       </c>
       <c r="D174" s="15" t="n">
-        <v>0.989</v>
+        <v>0.831</v>
       </c>
       <c r="E174" s="15" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F174" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.401</v>
+      </c>
+      <c r="F174" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5613,10 +5646,10 @@
         </is>
       </c>
       <c r="D175" s="19" t="n">
-        <v>0.971</v>
+        <v>0.886</v>
       </c>
       <c r="E175" s="19" t="n">
-        <v>0.786</v>
+        <v>0.637</v>
       </c>
       <c r="F175" s="16" t="inlineStr">
         <is>
@@ -5635,14 +5668,14 @@
       </c>
       <c r="C176" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICIAL-SYSTEM-OK</t>
+          <t>ARTIEICJAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D176" s="15" t="n">
-        <v>0.954</v>
+        <v>0.84</v>
       </c>
       <c r="E176" s="15" t="n">
-        <v>0.64</v>
+        <v>0.539</v>
       </c>
       <c r="F176" s="16" t="inlineStr">
         <is>
@@ -5661,18 +5694,18 @@
       </c>
       <c r="C177" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCOME-</t>
+          <t>HEDLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D177" s="19" t="n">
-        <v>0.98</v>
+        <v>0.852</v>
       </c>
       <c r="E177" s="19" t="n">
-        <v>0.9360000000000001</v>
-      </c>
-      <c r="F177" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.306</v>
+      </c>
+      <c r="F177" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5687,14 +5720,14 @@
       </c>
       <c r="C178" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POKER--</t>
+          <t>KNOWLEPGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D178" s="15" t="n">
-        <v>0.96</v>
+        <v>0.918</v>
       </c>
       <c r="E178" s="15" t="n">
-        <v>0.596</v>
+        <v>0.418</v>
       </c>
       <c r="F178" s="16" t="inlineStr">
         <is>
@@ -5713,14 +5746,14 @@
       </c>
       <c r="C179" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-GOLD</t>
+          <t>EIND-EXTRA-FIND-OOLD</t>
         </is>
       </c>
       <c r="D179" s="19" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.868</v>
       </c>
       <c r="E179" s="19" t="n">
-        <v>0.662</v>
+        <v>0.454</v>
       </c>
       <c r="F179" s="16" t="inlineStr">
         <is>
@@ -5739,18 +5772,18 @@
       </c>
       <c r="C180" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TEN</t>
+          <t>ZERGNONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D180" s="15" t="n">
-        <v>0.982</v>
+        <v>0.839</v>
       </c>
       <c r="E180" s="15" t="n">
-        <v>0.847</v>
-      </c>
-      <c r="F180" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.273</v>
+      </c>
+      <c r="F180" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5765,14 +5798,14 @@
       </c>
       <c r="C181" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPQRST</t>
+          <t>ABCDEEGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D181" s="19" t="n">
-        <v>0.969</v>
+        <v>0.858</v>
       </c>
       <c r="E181" s="19" t="n">
-        <v>0.637</v>
+        <v>0.497</v>
       </c>
       <c r="F181" s="16" t="inlineStr">
         <is>
@@ -5780,8 +5813,528 @@
         </is>
       </c>
     </row>
+    <row r="182" ht="20" customHeight="1">
+      <c r="A182" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B182" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C182" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D182" s="15" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="E182" s="15" t="n">
+        <v>0.532</v>
+      </c>
+      <c r="F182" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="20" customHeight="1">
+      <c r="A183" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B183" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C183" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D183" s="19" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E183" s="19" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="F183" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="20" customHeight="1">
+      <c r="A184" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B184" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C184" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-ROX-WITF-TEA</t>
+        </is>
+      </c>
+      <c r="D184" s="15" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="E184" s="15" t="n">
+        <v>0.458</v>
+      </c>
+      <c r="F184" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="20" customHeight="1">
+      <c r="A185" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B185" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C185" s="18" t="inlineStr">
+        <is>
+          <t>FIVEZDOZEN-IIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D185" s="19" t="n">
+        <v>0.885</v>
+      </c>
+      <c r="E185" s="19" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="F185" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="20" customHeight="1">
+      <c r="A186" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B186" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C186" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-RLAOK-GFM-</t>
+        </is>
+      </c>
+      <c r="D186" s="15" t="n">
+        <v>0.883</v>
+      </c>
+      <c r="E186" s="15" t="n">
+        <v>0.459</v>
+      </c>
+      <c r="F186" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="20" customHeight="1">
+      <c r="A187" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B187" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C187" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-GUICKLY</t>
+        </is>
+      </c>
+      <c r="D187" s="19" t="n">
+        <v>0.884</v>
+      </c>
+      <c r="E187" s="19" t="n">
+        <v>0.403</v>
+      </c>
+      <c r="F187" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="20" customHeight="1">
+      <c r="A188" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B188" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C188" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D188" s="15" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E188" s="15" t="n">
+        <v>0.541</v>
+      </c>
+      <c r="F188" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="20" customHeight="1">
+      <c r="A189" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B189" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C189" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-IEST</t>
+        </is>
+      </c>
+      <c r="D189" s="19" t="n">
+        <v>0.844</v>
+      </c>
+      <c r="E189" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F189" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="20" customHeight="1">
+      <c r="A190" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B190" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C190" s="14" t="inlineStr">
+        <is>
+          <t>MAOHINE-LFARNING-AL-</t>
+        </is>
+      </c>
+      <c r="D190" s="15" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="E190" s="15" t="n">
+        <v>0.426</v>
+      </c>
+      <c r="F190" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="20" customHeight="1">
+      <c r="A191" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B191" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C191" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKS</t>
+        </is>
+      </c>
+      <c r="D191" s="19" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E191" s="19" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="F191" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B192" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C192" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-DFTEOT-OK</t>
+        </is>
+      </c>
+      <c r="D192" s="15" t="n">
+        <v>0.836</v>
+      </c>
+      <c r="E192" s="15" t="n">
+        <v>0.398</v>
+      </c>
+      <c r="F192" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="20" customHeight="1">
+      <c r="A193" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B193" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C193" s="18" t="inlineStr">
+        <is>
+          <t>PYIHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D193" s="19" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="E193" s="19" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="F193" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="20" customHeight="1">
+      <c r="A194" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B194" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C194" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D194" s="15" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="E194" s="15" t="n">
+        <v>0.429</v>
+      </c>
+      <c r="F194" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="20" customHeight="1">
+      <c r="A195" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B195" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C195" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDKCTIDN-</t>
+        </is>
+      </c>
+      <c r="D195" s="19" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="E195" s="19" t="n">
+        <v>0.293</v>
+      </c>
+      <c r="F195" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="20" customHeight="1">
+      <c r="A196" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B196" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C196" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-RFEDICTIO</t>
+        </is>
+      </c>
+      <c r="D196" s="15" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="E196" s="15" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F196" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="20" customHeight="1">
+      <c r="A197" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B197" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C197" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WFLCOME-</t>
+        </is>
+      </c>
+      <c r="D197" s="19" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="E197" s="19" t="n">
+        <v>0.538</v>
+      </c>
+      <c r="F197" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="20" customHeight="1">
+      <c r="A198" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B198" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C198" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEPGE-IS-POWFR--</t>
+        </is>
+      </c>
+      <c r="D198" s="15" t="n">
+        <v>0.901</v>
+      </c>
+      <c r="E198" s="15" t="n">
+        <v>0.464</v>
+      </c>
+      <c r="F198" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="20" customHeight="1">
+      <c r="A199" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B199" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C199" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FLNE-GOID</t>
+        </is>
+      </c>
+      <c r="D199" s="19" t="n">
+        <v>0.824</v>
+      </c>
+      <c r="E199" s="19" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="F199" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="20" customHeight="1">
+      <c r="A200" s="13" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B200" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C200" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-OLX-TEN</t>
+        </is>
+      </c>
+      <c r="D200" s="15" t="n">
+        <v>0.878</v>
+      </c>
+      <c r="E200" s="15" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="F200" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="20" customHeight="1">
+      <c r="A201" s="17" t="inlineStr">
+        <is>
+          <t>test10.jpg</t>
+        </is>
+      </c>
+      <c r="B201" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C201" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIGKLMNOEGRST</t>
+        </is>
+      </c>
+      <c r="D201" s="19" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="E201" s="19" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="F201" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F181"/>
+  <autoFilter ref="A1:F201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: reach all-time peak 96.43% benchmark (3857/4000) with Early Stopping fine-tuned CNN
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-25 20:33:42 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 10 แผ่น | รวม 200 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-25 21:28:47 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 10 แผ่น | รวม 200 ข้อ</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>94.70%</t>
+          <t>96.43%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>190 ข้อ</t>
+          <t>197 ข้อ</t>
         </is>
       </c>
     </row>
@@ -760,17 +760,17 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>98.75%</t>
+          <t>99.25%</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.920</t>
+          <t>0.924</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>19 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>86.50%</t>
+          <t>90.50%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.815</t>
+          <t>0.824</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>95.25%</t>
+          <t>97.50%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.899</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>19 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>97.75%</t>
+          <t>98.50%</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.905</t>
+          <t>0.913</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>19 ข้อ</t>
+          <t>18 ข้อ</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -892,12 +892,12 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>94.25%</t>
+          <t>95.50%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>0.891</t>
+          <t>0.897</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -925,17 +925,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>96.50%</t>
+          <t>97.50%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>0.899</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>18 ข้อ</t>
+          <t>19 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>97.25%</t>
+          <t>98.50%</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>0.924</t>
+          <t>0.923</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>18 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -991,17 +991,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>97.50%</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>0.898</t>
+          <t>0.889</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>17 ข้อ</t>
+          <t>20 ข้อ</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1024,12 +1024,12 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>93.75%</t>
+          <t>95.00%</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>0.872</t>
+          <t>0.871</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>91.00%</t>
+          <t>94.50%</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>0.859</t>
+          <t>0.855</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -1148,10 +1148,10 @@
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.916</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.579</v>
+        <v>0.587</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         <v>0.917</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.362</v>
+        <v>0.318</v>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
@@ -1200,10 +1200,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.926</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.589</v>
+        <v>0.603</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -1226,10 +1226,10 @@
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.919</v>
+        <v>0.915</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.751</v>
+        <v>0.721</v>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
@@ -1252,10 +1252,10 @@
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.791</v>
+        <v>0.721</v>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
@@ -1278,10 +1278,10 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.915</v>
+        <v>0.924</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.644</v>
+        <v>0.666</v>
       </c>
       <c r="F7" s="16" t="inlineStr">
         <is>
@@ -1304,10 +1304,10 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.951</v>
+        <v>0.955</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.764</v>
+        <v>0.723</v>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
@@ -1330,10 +1330,10 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>0.895</v>
+        <v>0.909</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.552</v>
+        <v>0.666</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
@@ -1356,10 +1356,10 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.638</v>
+        <v>0.594</v>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
@@ -1382,10 +1382,10 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.911</v>
+        <v>0.912</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.518</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -1404,14 +1404,14 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DEIECT-OK</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.88</v>
+        <v>0.873</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.48</v>
+        <v>0.536</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
@@ -1434,10 +1434,10 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.944</v>
+        <v>0.945</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.762</v>
+        <v>0.794</v>
       </c>
       <c r="F13" s="16" t="inlineStr">
         <is>
@@ -1460,10 +1460,10 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>0.924</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>0.719</v>
+        <v>0.733</v>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
@@ -1486,10 +1486,10 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.909</v>
+        <v>0.924</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.739</v>
+        <v>0.753</v>
       </c>
       <c r="F15" s="16" t="inlineStr">
         <is>
@@ -1512,10 +1512,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.882</v>
+        <v>0.894</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.61</v>
+        <v>0.598</v>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
@@ -1534,18 +1534,18 @@
       </c>
       <c r="C17" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELOOME-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.8080000000000001</v>
-      </c>
-      <c r="F17" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.76</v>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -1564,10 +1564,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.954</v>
+        <v>0.948</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.791</v>
+        <v>0.74</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
@@ -1590,10 +1590,10 @@
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.895</v>
+        <v>0.886</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.651</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
@@ -1616,10 +1616,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.911</v>
+        <v>0.891</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.614</v>
+        <v>0.413</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
@@ -1642,10 +1642,10 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.924</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.668</v>
+        <v>0.746</v>
       </c>
       <c r="F21" s="16" t="inlineStr">
         <is>
@@ -1664,14 +1664,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>TIL-QUICK-RROWN-FQX-</t>
+          <t>TIL-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.878</v>
+        <v>0.872</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.491</v>
+        <v>0.467</v>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
@@ -1690,14 +1690,14 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-IOG-</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.884</v>
+        <v>0.901</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.307</v>
+        <v>0.288</v>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
@@ -1716,14 +1716,14 @@
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-ROX-WITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.924</v>
+        <v>0.926</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.478</v>
+        <v>0.598</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
@@ -1746,10 +1746,10 @@
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.847</v>
+        <v>0.875</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.403</v>
+        <v>0.487</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -1768,14 +1768,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHUNX-OF-BLACK-GEM-</t>
+          <t>SPHINX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
         <v>0.858</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.372</v>
+        <v>0.42</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -1794,14 +1794,14 @@
       </c>
       <c r="C27" s="18" t="inlineStr">
         <is>
-          <t>JUDSE-MY-VOW-QVICKLY</t>
+          <t>JUDGE-MY-VOW-QVICKLY</t>
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.844</v>
+        <v>0.859</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.59</v>
+        <v>0.583</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -1827,7 +1827,7 @@
         <v>0.8159999999999999</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.312</v>
+        <v>0.308</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
@@ -1846,14 +1846,14 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUIER-VISION-TESE</t>
+          <t>COMPUIER-VISION-TEST</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.863</v>
+        <v>0.862</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.331</v>
+        <v>0.404</v>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
@@ -1872,14 +1872,14 @@
       </c>
       <c r="C30" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AJ-</t>
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.881</v>
+        <v>0.894</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.482</v>
+        <v>0.45</v>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
@@ -1898,14 +1898,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NFTWORWS</t>
+          <t>DEEP-NEURAL-NFTWORKS</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.775</v>
+        <v>0.773</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.402</v>
+        <v>0.34</v>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
@@ -1924,14 +1924,14 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MASE-DATA-DEUFOT-CK</t>
+          <t>-MAGE-PATA-DETFCT-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.744</v>
+        <v>0.766</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.309</v>
+        <v>0.43</v>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
@@ -1954,10 +1954,10 @@
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.758</v>
+        <v>0.755</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.37</v>
+        <v>0.368</v>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
@@ -1980,10 +1980,10 @@
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.788</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.475</v>
+        <v>0.343</v>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
@@ -2002,14 +2002,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>AOCURATF--REDIOTJEQ-</t>
+          <t>AOCURATF--REDQCTJON-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.679</v>
+        <v>0.716</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.314</v>
+        <v>0.301</v>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
@@ -2028,14 +2028,14 @@
       </c>
       <c r="C36" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSTEM-CK</t>
+          <t>ARTIFICJAL-SYSTEM-CK</t>
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.786</v>
+        <v>0.792</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.426</v>
+        <v>0.427</v>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
@@ -2058,10 +2058,10 @@
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.773</v>
+        <v>0.786</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.314</v>
+        <v>0.299</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
@@ -2080,14 +2080,14 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KNOWL-OCFCIS-PQWER--</t>
+          <t>KNOWL-OGF-IS-POWER--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.79</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.477</v>
+        <v>0.417</v>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
@@ -2106,14 +2106,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>FIND-FXTRA-EIND-GDLD</t>
+          <t>FIND-FXTRA-FINE-GOLD</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.819</v>
+        <v>0.844</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.388</v>
+        <v>0.452</v>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
@@ -2136,10 +2136,10 @@
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.825</v>
+        <v>0.831</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.385</v>
+        <v>0.494</v>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
@@ -2158,14 +2158,14 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKL-NCPQRST</t>
+          <t>ABCDEFGHIJKL-NOPGRST</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.723</v>
+        <v>0.771</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.255</v>
+        <v>0.491</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
@@ -2188,10 +2188,10 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.915</v>
+        <v>0.911</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.617</v>
+        <v>0.577</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -2214,10 +2214,10 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.584</v>
+        <v>0.585</v>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
@@ -2236,14 +2236,14 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>EACK-MY-ROX-WITH-TEA</t>
+          <t>PACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.912</v>
+        <v>0.887</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.413</v>
+        <v>0.366</v>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
@@ -2266,10 +2266,10 @@
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.929</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.731</v>
+        <v>0.737</v>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
@@ -2292,10 +2292,10 @@
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.918</v>
+        <v>0.928</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.493</v>
+        <v>0.667</v>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
@@ -2318,10 +2318,10 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.915</v>
+        <v>0.919</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.596</v>
+        <v>0.608</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>0.931</v>
+        <v>0.925</v>
       </c>
       <c r="E48" s="15" t="n">
         <v>0.596</v>
@@ -2366,14 +2366,14 @@
       </c>
       <c r="C49" s="18" t="inlineStr">
         <is>
-          <t>DOMPUTER-VISION-TEST</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.901</v>
+        <v>0.893</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.527</v>
+        <v>0.553</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2396,10 +2396,10 @@
         </is>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.962</v>
+        <v>0.96</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.734</v>
+        <v>0.797</v>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
@@ -2422,10 +2422,10 @@
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.738</v>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
@@ -2444,14 +2444,14 @@
       </c>
       <c r="C52" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETEDT-OK</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>0.91</v>
+        <v>0.915</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>0.763</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
@@ -2470,14 +2470,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>PYTHONRDPENUVNROBOT-</t>
+          <t>PYTHON-DPENOV-ROBOT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.771</v>
+        <v>0.783</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.29</v>
+        <v>0.338</v>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
@@ -2500,10 +2500,10 @@
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>0.927</v>
+        <v>0.9</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.676</v>
+        <v>0.574</v>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
@@ -2522,14 +2522,14 @@
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>ADCURATE-PREDIDTION-</t>
+          <t>ACCURATE-PREDIDTION-</t>
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.859</v>
+        <v>0.853</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.577</v>
+        <v>0.583</v>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
@@ -2548,14 +2548,14 @@
       </c>
       <c r="C56" s="14" t="inlineStr">
         <is>
-          <t>ARTIFIDIAL-SYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.856</v>
+        <v>0.863</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.413</v>
+        <v>0.474</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
@@ -2578,10 +2578,10 @@
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.881</v>
+        <v>0.877</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.452</v>
+        <v>0.438</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
@@ -2600,14 +2600,14 @@
       </c>
       <c r="C58" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-FOWER--</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.878</v>
+        <v>0.886</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.417</v>
+        <v>0.522</v>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
@@ -2626,14 +2626,14 @@
       </c>
       <c r="C59" s="18" t="inlineStr">
         <is>
-          <t>FINP-EXTRA-FIND-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>0.877</v>
+        <v>0.888</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.36</v>
+        <v>0.541</v>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
@@ -2656,10 +2656,10 @@
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.898</v>
+        <v>0.887</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.519</v>
+        <v>0.509</v>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
@@ -2682,14 +2682,14 @@
         </is>
       </c>
       <c r="D61" s="19" t="n">
-        <v>0.926</v>
+        <v>0.927</v>
       </c>
       <c r="E61" s="19" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="F61" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.718</v>
+      </c>
+      <c r="F61" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -2708,10 +2708,10 @@
         </is>
       </c>
       <c r="D62" s="15" t="n">
-        <v>0.916</v>
+        <v>0.91</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>0.503</v>
+        <v>0.664</v>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
@@ -2734,10 +2734,10 @@
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.911</v>
+        <v>0.918</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.609</v>
+        <v>0.59</v>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
@@ -2756,14 +2756,14 @@
       </c>
       <c r="C64" s="14" t="inlineStr">
         <is>
-          <t>PAOK-MY-BOX-WITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D64" s="15" t="n">
         <v>0.896</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.475</v>
+        <v>0.512</v>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
@@ -2786,10 +2786,10 @@
         </is>
       </c>
       <c r="D65" s="19" t="n">
-        <v>0.916</v>
+        <v>0.931</v>
       </c>
       <c r="E65" s="19" t="n">
-        <v>0.722</v>
+        <v>0.636</v>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
@@ -2808,18 +2808,18 @@
       </c>
       <c r="C66" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLAOK-GEM-</t>
+          <t>SPHINX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>0.95</v>
+        <v>0.963</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.799</v>
-      </c>
-      <c r="F66" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.826</v>
+      </c>
+      <c r="F66" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2838,10 +2838,10 @@
         </is>
       </c>
       <c r="D67" s="19" t="n">
-        <v>0.873</v>
+        <v>0.896</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>0.602</v>
+        <v>0.592</v>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
@@ -2864,10 +2864,10 @@
         </is>
       </c>
       <c r="D68" s="15" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>0.696</v>
+        <v>0.646</v>
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
@@ -2890,10 +2890,10 @@
         </is>
       </c>
       <c r="D69" s="19" t="n">
-        <v>0.895</v>
+        <v>0.892</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>0.655</v>
+        <v>0.632</v>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
@@ -2916,10 +2916,10 @@
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.967</v>
+        <v>0.973</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>0.85</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
@@ -2938,14 +2938,14 @@
       </c>
       <c r="C71" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEEP-NEURAL-NETNORKS</t>
         </is>
       </c>
       <c r="D71" s="19" t="n">
-        <v>0.906</v>
+        <v>0.912</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>0.596</v>
+        <v>0.487</v>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
@@ -2968,10 +2968,10 @@
         </is>
       </c>
       <c r="D72" s="15" t="n">
-        <v>0.909</v>
+        <v>0.915</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>0.718</v>
+        <v>0.717</v>
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
@@ -2994,10 +2994,10 @@
         </is>
       </c>
       <c r="D73" s="19" t="n">
-        <v>0.878</v>
+        <v>0.872</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.589</v>
+        <v>0.578</v>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
@@ -3020,10 +3020,10 @@
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>0.895</v>
+        <v>0.911</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>0.528</v>
+        <v>0.662</v>
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
@@ -3042,14 +3042,14 @@
       </c>
       <c r="C75" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDIDTION-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>0.851</v>
+        <v>0.869</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>0.506</v>
+        <v>0.6</v>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
@@ -3072,10 +3072,10 @@
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.891</v>
+        <v>0.916</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>0.473</v>
+        <v>0.663</v>
       </c>
       <c r="F76" s="16" t="inlineStr">
         <is>
@@ -3094,14 +3094,14 @@
       </c>
       <c r="C77" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELOOME-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>0.914</v>
+        <v>0.918</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>0.609</v>
+        <v>0.626</v>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
@@ -3124,10 +3124,10 @@
         </is>
       </c>
       <c r="D78" s="15" t="n">
-        <v>0.898</v>
+        <v>0.899</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>0.267</v>
+        <v>0.266</v>
       </c>
       <c r="F78" s="16" t="inlineStr">
         <is>
@@ -3150,10 +3150,10 @@
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>0.892</v>
+        <v>0.887</v>
       </c>
       <c r="E79" s="19" t="n">
-        <v>0.661</v>
+        <v>0.543</v>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
@@ -3176,10 +3176,10 @@
         </is>
       </c>
       <c r="D80" s="15" t="n">
-        <v>0.928</v>
+        <v>0.926</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>0.677</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="F80" s="16" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         </is>
       </c>
       <c r="D81" s="19" t="n">
-        <v>0.875</v>
+        <v>0.904</v>
       </c>
       <c r="E81" s="19" t="n">
-        <v>0.521</v>
+        <v>0.606</v>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
@@ -3228,10 +3228,10 @@
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>0.919</v>
+        <v>0.921</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.44</v>
+        <v>0.413</v>
       </c>
       <c r="F82" s="16" t="inlineStr">
         <is>
@@ -3254,10 +3254,10 @@
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E83" s="19" t="n">
-        <v>0.538</v>
+        <v>0.513</v>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
@@ -3280,10 +3280,10 @@
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>0.913</v>
+        <v>0.927</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.602</v>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
@@ -3306,10 +3306,10 @@
         </is>
       </c>
       <c r="D85" s="19" t="n">
-        <v>0.913</v>
+        <v>0.924</v>
       </c>
       <c r="E85" s="19" t="n">
-        <v>0.544</v>
+        <v>0.622</v>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
@@ -3332,10 +3332,10 @@
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>0.892</v>
+        <v>0.894</v>
       </c>
       <c r="E86" s="15" t="n">
-        <v>0.504</v>
+        <v>0.59</v>
       </c>
       <c r="F86" s="16" t="inlineStr">
         <is>
@@ -3358,10 +3358,10 @@
         </is>
       </c>
       <c r="D87" s="19" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.954</v>
       </c>
       <c r="E87" s="19" t="n">
-        <v>0.735</v>
+        <v>0.765</v>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
@@ -3384,10 +3384,10 @@
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.887</v>
+        <v>0.895</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.296</v>
+        <v>0.472</v>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
@@ -3410,10 +3410,10 @@
         </is>
       </c>
       <c r="D89" s="19" t="n">
-        <v>0.847</v>
+        <v>0.856</v>
       </c>
       <c r="E89" s="19" t="n">
-        <v>0.475</v>
+        <v>0.539</v>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
@@ -3432,14 +3432,14 @@
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>MACHTNE-LFARNJNG-AI-</t>
+          <t>MACHINE-LEARNJNG-AI-</t>
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>0.835</v>
+        <v>0.868</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>0.38</v>
+        <v>0.406</v>
       </c>
       <c r="F90" s="16" t="inlineStr">
         <is>
@@ -3462,10 +3462,10 @@
         </is>
       </c>
       <c r="D91" s="19" t="n">
-        <v>0.914</v>
+        <v>0.917</v>
       </c>
       <c r="E91" s="19" t="n">
-        <v>0.626</v>
+        <v>0.647</v>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
@@ -3488,10 +3488,10 @@
         </is>
       </c>
       <c r="D92" s="15" t="n">
-        <v>0.879</v>
+        <v>0.888</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.525</v>
       </c>
       <c r="F92" s="16" t="inlineStr">
         <is>
@@ -3514,10 +3514,10 @@
         </is>
       </c>
       <c r="D93" s="19" t="n">
-        <v>0.905</v>
+        <v>0.889</v>
       </c>
       <c r="E93" s="19" t="n">
-        <v>0.578</v>
+        <v>0.545</v>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
@@ -3540,10 +3540,10 @@
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>0.926</v>
+        <v>0.922</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>0.792</v>
+        <v>0.703</v>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
@@ -3562,14 +3562,14 @@
       </c>
       <c r="C95" s="18" t="inlineStr">
         <is>
-          <t>ACCURATF-PREPICTION-</t>
+          <t>ACCURATF-PREDICTION-</t>
         </is>
       </c>
       <c r="D95" s="19" t="n">
-        <v>0.851</v>
+        <v>0.897</v>
       </c>
       <c r="E95" s="19" t="n">
-        <v>0.485</v>
+        <v>0.554</v>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
@@ -3592,10 +3592,10 @@
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>0.854</v>
+        <v>0.868</v>
       </c>
       <c r="E96" s="15" t="n">
-        <v>0.368</v>
+        <v>0.513</v>
       </c>
       <c r="F96" s="16" t="inlineStr">
         <is>
@@ -3614,14 +3614,14 @@
       </c>
       <c r="C97" s="18" t="inlineStr">
         <is>
-          <t>HELIO-WORLO-WELCOMF-</t>
+          <t>HELLO-WORLO-WELCOMF-</t>
         </is>
       </c>
       <c r="D97" s="19" t="n">
-        <v>0.891</v>
+        <v>0.861</v>
       </c>
       <c r="E97" s="19" t="n">
-        <v>0.53</v>
+        <v>0.507</v>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
@@ -3640,14 +3640,14 @@
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEOGE-IS-PONEF--</t>
+          <t>KNOWLEOGE-IS-PONER--</t>
         </is>
       </c>
       <c r="D98" s="15" t="n">
-        <v>0.898</v>
+        <v>0.887</v>
       </c>
       <c r="E98" s="15" t="n">
-        <v>0.424</v>
+        <v>0.547</v>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
@@ -3666,14 +3666,14 @@
       </c>
       <c r="C99" s="18" t="inlineStr">
         <is>
-          <t>F-ND-EXTRA-FIND-GOLD</t>
+          <t>F-ND-EETRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.832</v>
+        <v>0.839</v>
       </c>
       <c r="E99" s="19" t="n">
-        <v>0.415</v>
+        <v>0.396</v>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
@@ -3696,10 +3696,10 @@
         </is>
       </c>
       <c r="D100" s="15" t="n">
-        <v>0.911</v>
+        <v>0.897</v>
       </c>
       <c r="E100" s="15" t="n">
-        <v>0.449</v>
+        <v>0.384</v>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
@@ -3718,14 +3718,14 @@
       </c>
       <c r="C101" s="18" t="inlineStr">
         <is>
-          <t>ABNDEFGHIJKLMNOPQRST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D101" s="19" t="n">
-        <v>0.873</v>
+        <v>0.893</v>
       </c>
       <c r="E101" s="19" t="n">
-        <v>0.268</v>
+        <v>0.535</v>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
@@ -3748,10 +3748,10 @@
         </is>
       </c>
       <c r="D102" s="15" t="n">
-        <v>0.862</v>
+        <v>0.875</v>
       </c>
       <c r="E102" s="15" t="n">
-        <v>0.497</v>
+        <v>0.506</v>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
@@ -3774,10 +3774,10 @@
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.901</v>
+        <v>0.9</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.615</v>
+        <v>0.511</v>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
@@ -3800,10 +3800,10 @@
         </is>
       </c>
       <c r="D104" s="15" t="n">
-        <v>0.931</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>0.592</v>
+        <v>0.589</v>
       </c>
       <c r="F104" s="16" t="inlineStr">
         <is>
@@ -3826,10 +3826,10 @@
         </is>
       </c>
       <c r="D105" s="19" t="n">
-        <v>0.893</v>
+        <v>0.892</v>
       </c>
       <c r="E105" s="19" t="n">
-        <v>0.578</v>
+        <v>0.486</v>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
@@ -3852,10 +3852,10 @@
         </is>
       </c>
       <c r="D106" s="15" t="n">
-        <v>0.918</v>
+        <v>0.917</v>
       </c>
       <c r="E106" s="15" t="n">
-        <v>0.669</v>
+        <v>0.679</v>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
@@ -3878,10 +3878,10 @@
         </is>
       </c>
       <c r="D107" s="19" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.946</v>
       </c>
       <c r="E107" s="19" t="n">
-        <v>0.549</v>
+        <v>0.656</v>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
@@ -3904,14 +3904,14 @@
         </is>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.945</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.8120000000000001</v>
-      </c>
-      <c r="F108" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.656</v>
+      </c>
+      <c r="F108" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -3930,10 +3930,10 @@
         </is>
       </c>
       <c r="D109" s="19" t="n">
-        <v>0.918</v>
+        <v>0.911</v>
       </c>
       <c r="E109" s="19" t="n">
-        <v>0.662</v>
+        <v>0.61</v>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
@@ -3956,10 +3956,10 @@
         </is>
       </c>
       <c r="D110" s="15" t="n">
-        <v>0.972</v>
+        <v>0.977</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.834</v>
+        <v>0.881</v>
       </c>
       <c r="F110" s="20" t="inlineStr">
         <is>
@@ -3982,10 +3982,10 @@
         </is>
       </c>
       <c r="D111" s="19" t="n">
-        <v>0.949</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E111" s="19" t="n">
-        <v>0.72</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
@@ -4008,10 +4008,10 @@
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.884</v>
+        <v>0.868</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.55</v>
+        <v>0.501</v>
       </c>
       <c r="F112" s="16" t="inlineStr">
         <is>
@@ -4030,14 +4030,14 @@
       </c>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENDV-ROBOT-</t>
+          <t>PPTHON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D113" s="19" t="n">
-        <v>0.896</v>
+        <v>0.885</v>
       </c>
       <c r="E113" s="19" t="n">
-        <v>0.516</v>
+        <v>0.303</v>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
@@ -4063,7 +4063,7 @@
         <v>0.884</v>
       </c>
       <c r="E114" s="15" t="n">
-        <v>0.672</v>
+        <v>0.613</v>
       </c>
       <c r="F114" s="16" t="inlineStr">
         <is>
@@ -4082,14 +4082,14 @@
       </c>
       <c r="C115" s="18" t="inlineStr">
         <is>
-          <t>AOCURATE-PREDICTION-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D115" s="19" t="n">
-        <v>0.847</v>
+        <v>0.854</v>
       </c>
       <c r="E115" s="19" t="n">
-        <v>0.454</v>
+        <v>0.487</v>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
@@ -4108,14 +4108,14 @@
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>ADTIFTCTAL-SYSTEM-OK</t>
+          <t>ARTIFICTAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.805</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.377</v>
+        <v>0.448</v>
       </c>
       <c r="F116" s="16" t="inlineStr">
         <is>
@@ -4138,10 +4138,10 @@
         </is>
       </c>
       <c r="D117" s="19" t="n">
-        <v>0.885</v>
+        <v>0.876</v>
       </c>
       <c r="E117" s="19" t="n">
-        <v>0.576</v>
+        <v>0.583</v>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
@@ -4164,10 +4164,10 @@
         </is>
       </c>
       <c r="D118" s="15" t="n">
-        <v>0.911</v>
+        <v>0.916</v>
       </c>
       <c r="E118" s="15" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="F118" s="16" t="inlineStr">
         <is>
@@ -4190,10 +4190,10 @@
         </is>
       </c>
       <c r="D119" s="19" t="n">
-        <v>0.886</v>
+        <v>0.9</v>
       </c>
       <c r="E119" s="19" t="n">
-        <v>0.632</v>
+        <v>0.696</v>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
@@ -4216,10 +4216,10 @@
         </is>
       </c>
       <c r="D120" s="15" t="n">
-        <v>0.923</v>
+        <v>0.92</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>0.627</v>
+        <v>0.591</v>
       </c>
       <c r="F120" s="16" t="inlineStr">
         <is>
@@ -4238,14 +4238,14 @@
       </c>
       <c r="C121" s="18" t="inlineStr">
         <is>
-          <t>ABDDEFGHIJKTMNOPORST</t>
+          <t>ABDDEFGHIJKLMNOPORST</t>
         </is>
       </c>
       <c r="D121" s="19" t="n">
-        <v>0.832</v>
+        <v>0.845</v>
       </c>
       <c r="E121" s="19" t="n">
-        <v>0.347</v>
+        <v>0.375</v>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
@@ -4268,10 +4268,10 @@
         </is>
       </c>
       <c r="D122" s="15" t="n">
-        <v>0.927</v>
+        <v>0.917</v>
       </c>
       <c r="E122" s="15" t="n">
-        <v>0.637</v>
+        <v>0.642</v>
       </c>
       <c r="F122" s="16" t="inlineStr">
         <is>
@@ -4297,7 +4297,7 @@
         <v>0.9389999999999999</v>
       </c>
       <c r="E123" s="19" t="n">
-        <v>0.548</v>
+        <v>0.556</v>
       </c>
       <c r="F123" s="16" t="inlineStr">
         <is>
@@ -4316,14 +4316,14 @@
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>PAOK-MY-BOXNWITH-TEA</t>
+          <t>PACK-MY-BOX-WITH-TEA</t>
         </is>
       </c>
       <c r="D124" s="15" t="n">
-        <v>0.919</v>
+        <v>0.926</v>
       </c>
       <c r="E124" s="15" t="n">
-        <v>0.233</v>
+        <v>0.597</v>
       </c>
       <c r="F124" s="16" t="inlineStr">
         <is>
@@ -4346,10 +4346,10 @@
         </is>
       </c>
       <c r="D125" s="19" t="n">
-        <v>0.926</v>
+        <v>0.93</v>
       </c>
       <c r="E125" s="19" t="n">
-        <v>0.592</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="F125" s="16" t="inlineStr">
         <is>
@@ -4372,10 +4372,10 @@
         </is>
       </c>
       <c r="D126" s="15" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E126" s="15" t="n">
-        <v>0.651</v>
+        <v>0.748</v>
       </c>
       <c r="F126" s="16" t="inlineStr">
         <is>
@@ -4394,14 +4394,14 @@
       </c>
       <c r="C127" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MYUVOW-QUICKLY</t>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
         </is>
       </c>
       <c r="D127" s="19" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.926</v>
       </c>
       <c r="E127" s="19" t="n">
-        <v>0.74</v>
+        <v>0.627</v>
       </c>
       <c r="F127" s="16" t="inlineStr">
         <is>
@@ -4424,14 +4424,14 @@
         </is>
       </c>
       <c r="D128" s="15" t="n">
-        <v>0.968</v>
+        <v>0.972</v>
       </c>
       <c r="E128" s="15" t="n">
-        <v>0.8179999999999999</v>
-      </c>
-      <c r="F128" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.712</v>
+      </c>
+      <c r="F128" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4450,10 +4450,10 @@
         </is>
       </c>
       <c r="D129" s="19" t="n">
-        <v>0.907</v>
+        <v>0.909</v>
       </c>
       <c r="E129" s="19" t="n">
-        <v>0.674</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F129" s="16" t="inlineStr">
         <is>
@@ -4472,18 +4472,18 @@
       </c>
       <c r="C130" s="14" t="inlineStr">
         <is>
-          <t>MAOHINE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D130" s="15" t="n">
-        <v>0.96</v>
+        <v>0.956</v>
       </c>
       <c r="E130" s="15" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F130" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.747</v>
+      </c>
+      <c r="F130" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -4502,10 +4502,10 @@
         </is>
       </c>
       <c r="D131" s="19" t="n">
-        <v>0.885</v>
+        <v>0.879</v>
       </c>
       <c r="E131" s="19" t="n">
-        <v>0.361</v>
+        <v>0.302</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -4528,10 +4528,10 @@
         </is>
       </c>
       <c r="D132" s="15" t="n">
-        <v>0.893</v>
+        <v>0.888</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>0.607</v>
+        <v>0.576</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -4554,10 +4554,10 @@
         </is>
       </c>
       <c r="D133" s="19" t="n">
-        <v>0.912</v>
+        <v>0.895</v>
       </c>
       <c r="E133" s="19" t="n">
-        <v>0.696</v>
+        <v>0.622</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         </is>
       </c>
       <c r="D134" s="15" t="n">
-        <v>0.946</v>
+        <v>0.944</v>
       </c>
       <c r="E134" s="15" t="n">
-        <v>0.6830000000000001</v>
+        <v>0.679</v>
       </c>
       <c r="F134" s="16" t="inlineStr">
         <is>
@@ -4606,10 +4606,10 @@
         </is>
       </c>
       <c r="D135" s="19" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.916</v>
       </c>
       <c r="E135" s="19" t="n">
-        <v>0.71</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F135" s="16" t="inlineStr">
         <is>
@@ -4632,10 +4632,10 @@
         </is>
       </c>
       <c r="D136" s="15" t="n">
-        <v>0.889</v>
+        <v>0.896</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>0.484</v>
+        <v>0.439</v>
       </c>
       <c r="F136" s="16" t="inlineStr">
         <is>
@@ -4661,7 +4661,7 @@
         <v>0.9429999999999999</v>
       </c>
       <c r="E137" s="19" t="n">
-        <v>0.748</v>
+        <v>0.708</v>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
@@ -4684,10 +4684,10 @@
         </is>
       </c>
       <c r="D138" s="15" t="n">
-        <v>0.921</v>
+        <v>0.931</v>
       </c>
       <c r="E138" s="15" t="n">
-        <v>0.414</v>
+        <v>0.421</v>
       </c>
       <c r="F138" s="16" t="inlineStr">
         <is>
@@ -4706,14 +4706,14 @@
       </c>
       <c r="C139" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FINP-GOLD</t>
+          <t>FIND-EXTRA-FINE-GOLD</t>
         </is>
       </c>
       <c r="D139" s="19" t="n">
-        <v>0.892</v>
+        <v>0.898</v>
       </c>
       <c r="E139" s="19" t="n">
-        <v>0.374</v>
+        <v>0.39</v>
       </c>
       <c r="F139" s="16" t="inlineStr">
         <is>
@@ -4736,10 +4736,10 @@
         </is>
       </c>
       <c r="D140" s="15" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.925</v>
       </c>
       <c r="E140" s="15" t="n">
-        <v>0.712</v>
+        <v>0.67</v>
       </c>
       <c r="F140" s="16" t="inlineStr">
         <is>
@@ -4762,10 +4762,10 @@
         </is>
       </c>
       <c r="D141" s="19" t="n">
-        <v>0.913</v>
+        <v>0.922</v>
       </c>
       <c r="E141" s="19" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="F141" s="16" t="inlineStr">
         <is>
@@ -4784,14 +4784,14 @@
       </c>
       <c r="C142" s="14" t="inlineStr">
         <is>
-          <t>TPE-QUICK-BRAWN-FOX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D142" s="15" t="n">
-        <v>0.844</v>
+        <v>0.846</v>
       </c>
       <c r="E142" s="15" t="n">
-        <v>0.236</v>
+        <v>0.34</v>
       </c>
       <c r="F142" s="16" t="inlineStr">
         <is>
@@ -4814,10 +4814,10 @@
         </is>
       </c>
       <c r="D143" s="19" t="n">
-        <v>0.886</v>
+        <v>0.885</v>
       </c>
       <c r="E143" s="19" t="n">
-        <v>0.413</v>
+        <v>0.466</v>
       </c>
       <c r="F143" s="16" t="inlineStr">
         <is>
@@ -4840,10 +4840,10 @@
         </is>
       </c>
       <c r="D144" s="15" t="n">
-        <v>0.863</v>
+        <v>0.844</v>
       </c>
       <c r="E144" s="15" t="n">
-        <v>0.431</v>
+        <v>0.341</v>
       </c>
       <c r="F144" s="16" t="inlineStr">
         <is>
@@ -4866,10 +4866,10 @@
         </is>
       </c>
       <c r="D145" s="19" t="n">
-        <v>0.893</v>
+        <v>0.872</v>
       </c>
       <c r="E145" s="19" t="n">
-        <v>0.497</v>
+        <v>0.52</v>
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
@@ -4888,14 +4888,14 @@
       </c>
       <c r="C146" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OR-BLAOK-GES-</t>
+          <t>SPHINX-OR-BLAOK-GEM-</t>
         </is>
       </c>
       <c r="D146" s="15" t="n">
-        <v>0.87</v>
+        <v>0.864</v>
       </c>
       <c r="E146" s="15" t="n">
-        <v>0.287</v>
+        <v>0.381</v>
       </c>
       <c r="F146" s="16" t="inlineStr">
         <is>
@@ -4918,10 +4918,10 @@
         </is>
       </c>
       <c r="D147" s="19" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="E147" s="19" t="n">
-        <v>0.792</v>
+        <v>0.739</v>
       </c>
       <c r="F147" s="16" t="inlineStr">
         <is>
@@ -4944,10 +4944,10 @@
         </is>
       </c>
       <c r="D148" s="15" t="n">
-        <v>0.931</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="E148" s="15" t="n">
-        <v>0.605</v>
+        <v>0.592</v>
       </c>
       <c r="F148" s="16" t="inlineStr">
         <is>
@@ -4970,10 +4970,10 @@
         </is>
       </c>
       <c r="D149" s="19" t="n">
-        <v>0.91</v>
+        <v>0.887</v>
       </c>
       <c r="E149" s="19" t="n">
-        <v>0.663</v>
+        <v>0.573</v>
       </c>
       <c r="F149" s="16" t="inlineStr">
         <is>
@@ -4996,14 +4996,14 @@
         </is>
       </c>
       <c r="D150" s="15" t="n">
-        <v>0.948</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E150" s="15" t="n">
-        <v>0.8120000000000001</v>
-      </c>
-      <c r="F150" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.706</v>
+      </c>
+      <c r="F150" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5018,14 +5018,14 @@
       </c>
       <c r="C151" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEEP-NEURAL-NETMORKS</t>
         </is>
       </c>
       <c r="D151" s="19" t="n">
         <v>0.882</v>
       </c>
       <c r="E151" s="19" t="n">
-        <v>0.592</v>
+        <v>0.509</v>
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
@@ -5048,10 +5048,10 @@
         </is>
       </c>
       <c r="D152" s="15" t="n">
-        <v>0.875</v>
+        <v>0.853</v>
       </c>
       <c r="E152" s="15" t="n">
-        <v>0.61</v>
+        <v>0.506</v>
       </c>
       <c r="F152" s="16" t="inlineStr">
         <is>
@@ -5074,10 +5074,10 @@
         </is>
       </c>
       <c r="D153" s="19" t="n">
-        <v>0.911</v>
+        <v>0.898</v>
       </c>
       <c r="E153" s="19" t="n">
-        <v>0.539</v>
+        <v>0.642</v>
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
@@ -5096,18 +5096,18 @@
       </c>
       <c r="C154" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-REOOGNIZE-</t>
+          <t>SMART-OCR-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D154" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.916</v>
       </c>
       <c r="E154" s="15" t="n">
-        <v>0.821</v>
-      </c>
-      <c r="F154" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.697</v>
+      </c>
+      <c r="F154" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5122,14 +5122,14 @@
       </c>
       <c r="C155" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDIOTJON-</t>
+          <t>ACCURATE-PREDIOTION-</t>
         </is>
       </c>
       <c r="D155" s="19" t="n">
-        <v>0.854</v>
+        <v>0.86</v>
       </c>
       <c r="E155" s="19" t="n">
-        <v>0.368</v>
+        <v>0.333</v>
       </c>
       <c r="F155" s="16" t="inlineStr">
         <is>
@@ -5148,14 +5148,14 @@
       </c>
       <c r="C156" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIALESYSTEM-OK</t>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D156" s="15" t="n">
-        <v>0.912</v>
+        <v>0.921</v>
       </c>
       <c r="E156" s="15" t="n">
-        <v>0.46</v>
+        <v>0.535</v>
       </c>
       <c r="F156" s="16" t="inlineStr">
         <is>
@@ -5178,10 +5178,10 @@
         </is>
       </c>
       <c r="D157" s="19" t="n">
-        <v>0.905</v>
+        <v>0.888</v>
       </c>
       <c r="E157" s="19" t="n">
-        <v>0.595</v>
+        <v>0.626</v>
       </c>
       <c r="F157" s="16" t="inlineStr">
         <is>
@@ -5204,10 +5204,10 @@
         </is>
       </c>
       <c r="D158" s="15" t="n">
-        <v>0.923</v>
+        <v>0.912</v>
       </c>
       <c r="E158" s="15" t="n">
-        <v>0.704</v>
+        <v>0.676</v>
       </c>
       <c r="F158" s="16" t="inlineStr">
         <is>
@@ -5230,10 +5230,10 @@
         </is>
       </c>
       <c r="D159" s="19" t="n">
-        <v>0.867</v>
+        <v>0.861</v>
       </c>
       <c r="E159" s="19" t="n">
-        <v>0.5</v>
+        <v>0.515</v>
       </c>
       <c r="F159" s="16" t="inlineStr">
         <is>
@@ -5256,14 +5256,14 @@
         </is>
       </c>
       <c r="D160" s="15" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.921</v>
       </c>
       <c r="E160" s="15" t="n">
-        <v>0.837</v>
-      </c>
-      <c r="F160" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.705</v>
+      </c>
+      <c r="F160" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -5278,14 +5278,14 @@
       </c>
       <c r="C161" s="18" t="inlineStr">
         <is>
-          <t>ABODEFQHIJKLMNOPQRST</t>
+          <t>ABODEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D161" s="19" t="n">
-        <v>0.853</v>
+        <v>0.871</v>
       </c>
       <c r="E161" s="19" t="n">
-        <v>0.425</v>
+        <v>0.588</v>
       </c>
       <c r="F161" s="16" t="inlineStr">
         <is>
@@ -5308,10 +5308,10 @@
         </is>
       </c>
       <c r="D162" s="15" t="n">
-        <v>0.898</v>
+        <v>0.907</v>
       </c>
       <c r="E162" s="15" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.586</v>
       </c>
       <c r="F162" s="16" t="inlineStr">
         <is>
@@ -5330,14 +5330,14 @@
       </c>
       <c r="C163" s="18" t="inlineStr">
         <is>
-          <t>IUMPS-OVER-LAZY-OOG-</t>
+          <t>IVMPS-OVER-LAZY-OOG-</t>
         </is>
       </c>
       <c r="D163" s="19" t="n">
-        <v>0.911</v>
+        <v>0.897</v>
       </c>
       <c r="E163" s="19" t="n">
-        <v>0.486</v>
+        <v>0.538</v>
       </c>
       <c r="F163" s="16" t="inlineStr">
         <is>
@@ -5360,10 +5360,10 @@
         </is>
       </c>
       <c r="D164" s="15" t="n">
-        <v>0.926</v>
+        <v>0.92</v>
       </c>
       <c r="E164" s="15" t="n">
-        <v>0.661</v>
+        <v>0.658</v>
       </c>
       <c r="F164" s="16" t="inlineStr">
         <is>
@@ -5382,14 +5382,14 @@
       </c>
       <c r="C165" s="18" t="inlineStr">
         <is>
-          <t>FJVE-DOZEN-LIQUOR-IU</t>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
         </is>
       </c>
       <c r="D165" s="19" t="n">
-        <v>0.871</v>
+        <v>0.845</v>
       </c>
       <c r="E165" s="19" t="n">
-        <v>0.536</v>
+        <v>0.497</v>
       </c>
       <c r="F165" s="16" t="inlineStr">
         <is>
@@ -5408,14 +5408,14 @@
       </c>
       <c r="C166" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OT-RLACK-GEM-</t>
+          <t>SPHINX-OF-RLACK-GEM-</t>
         </is>
       </c>
       <c r="D166" s="15" t="n">
-        <v>0.88</v>
+        <v>0.903</v>
       </c>
       <c r="E166" s="15" t="n">
-        <v>0.351</v>
+        <v>0.413</v>
       </c>
       <c r="F166" s="16" t="inlineStr">
         <is>
@@ -5438,10 +5438,10 @@
         </is>
       </c>
       <c r="D167" s="19" t="n">
-        <v>0.853</v>
+        <v>0.889</v>
       </c>
       <c r="E167" s="19" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.681</v>
       </c>
       <c r="F167" s="16" t="inlineStr">
         <is>
@@ -5460,14 +5460,14 @@
       </c>
       <c r="C168" s="14" t="inlineStr">
         <is>
-          <t>BRZGHT-ZFPHYRS-RLOW-</t>
+          <t>BRZGHT-ZFPMYRS-RLOW-</t>
         </is>
       </c>
       <c r="D168" s="15" t="n">
-        <v>0.839</v>
+        <v>0.849</v>
       </c>
       <c r="E168" s="15" t="n">
-        <v>0.43</v>
+        <v>0.506</v>
       </c>
       <c r="F168" s="16" t="inlineStr">
         <is>
@@ -5490,10 +5490,10 @@
         </is>
       </c>
       <c r="D169" s="19" t="n">
-        <v>0.868</v>
+        <v>0.843</v>
       </c>
       <c r="E169" s="19" t="n">
-        <v>0.599</v>
+        <v>0.495</v>
       </c>
       <c r="F169" s="16" t="inlineStr">
         <is>
@@ -5516,10 +5516,10 @@
         </is>
       </c>
       <c r="D170" s="15" t="n">
-        <v>0.924</v>
+        <v>0.923</v>
       </c>
       <c r="E170" s="15" t="n">
-        <v>0.601</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="F170" s="16" t="inlineStr">
         <is>
@@ -5538,11 +5538,11 @@
       </c>
       <c r="C171" s="18" t="inlineStr">
         <is>
-          <t>DEER-NQURAL-NETWORXS</t>
+          <t>DEEP-NQURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D171" s="19" t="n">
-        <v>0.851</v>
+        <v>0.847</v>
       </c>
       <c r="E171" s="19" t="n">
         <v>0.278</v>
@@ -5568,10 +5568,10 @@
         </is>
       </c>
       <c r="D172" s="15" t="n">
-        <v>0.838</v>
+        <v>0.853</v>
       </c>
       <c r="E172" s="15" t="n">
-        <v>0.463</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="F172" s="16" t="inlineStr">
         <is>
@@ -5594,10 +5594,10 @@
         </is>
       </c>
       <c r="D173" s="19" t="n">
-        <v>0.884</v>
+        <v>0.887</v>
       </c>
       <c r="E173" s="19" t="n">
-        <v>0.385</v>
+        <v>0.597</v>
       </c>
       <c r="F173" s="16" t="inlineStr">
         <is>
@@ -5620,10 +5620,10 @@
         </is>
       </c>
       <c r="D174" s="15" t="n">
-        <v>0.831</v>
+        <v>0.8129999999999999</v>
       </c>
       <c r="E174" s="15" t="n">
-        <v>0.401</v>
+        <v>0.415</v>
       </c>
       <c r="F174" s="16" t="inlineStr">
         <is>
@@ -5646,10 +5646,10 @@
         </is>
       </c>
       <c r="D175" s="19" t="n">
-        <v>0.886</v>
+        <v>0.881</v>
       </c>
       <c r="E175" s="19" t="n">
-        <v>0.637</v>
+        <v>0.601</v>
       </c>
       <c r="F175" s="16" t="inlineStr">
         <is>
@@ -5668,14 +5668,14 @@
       </c>
       <c r="C176" s="14" t="inlineStr">
         <is>
-          <t>ARTIEICJAL-SYSTEM-OK</t>
+          <t>ARTIEZCJAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D176" s="15" t="n">
-        <v>0.84</v>
+        <v>0.835</v>
       </c>
       <c r="E176" s="15" t="n">
-        <v>0.539</v>
+        <v>0.516</v>
       </c>
       <c r="F176" s="16" t="inlineStr">
         <is>
@@ -5694,14 +5694,14 @@
       </c>
       <c r="C177" s="18" t="inlineStr">
         <is>
-          <t>HEDLO-WORLD-WELCOME-</t>
+          <t>HELLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D177" s="19" t="n">
-        <v>0.852</v>
+        <v>0.863</v>
       </c>
       <c r="E177" s="19" t="n">
-        <v>0.306</v>
+        <v>0.386</v>
       </c>
       <c r="F177" s="16" t="inlineStr">
         <is>
@@ -5720,14 +5720,14 @@
       </c>
       <c r="C178" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEPGE-IS-POWER--</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D178" s="15" t="n">
-        <v>0.918</v>
+        <v>0.909</v>
       </c>
       <c r="E178" s="15" t="n">
-        <v>0.418</v>
+        <v>0.412</v>
       </c>
       <c r="F178" s="16" t="inlineStr">
         <is>
@@ -5746,14 +5746,14 @@
       </c>
       <c r="C179" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-OOLD</t>
+          <t>EIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D179" s="19" t="n">
-        <v>0.868</v>
+        <v>0.855</v>
       </c>
       <c r="E179" s="19" t="n">
-        <v>0.454</v>
+        <v>0.405</v>
       </c>
       <c r="F179" s="16" t="inlineStr">
         <is>
@@ -5772,14 +5772,14 @@
       </c>
       <c r="C180" s="14" t="inlineStr">
         <is>
-          <t>ZERGNONE-TWO-SIX-TEN</t>
+          <t>ZERG-ONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D180" s="15" t="n">
-        <v>0.839</v>
+        <v>0.852</v>
       </c>
       <c r="E180" s="15" t="n">
-        <v>0.273</v>
+        <v>0.475</v>
       </c>
       <c r="F180" s="16" t="inlineStr">
         <is>
@@ -5798,14 +5798,14 @@
       </c>
       <c r="C181" s="18" t="inlineStr">
         <is>
-          <t>ABCDEEGHIJKLMNOPQRST</t>
+          <t>ABCDEEGVIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D181" s="19" t="n">
         <v>0.858</v>
       </c>
       <c r="E181" s="19" t="n">
-        <v>0.497</v>
+        <v>0.477</v>
       </c>
       <c r="F181" s="16" t="inlineStr">
         <is>
@@ -5828,10 +5828,10 @@
         </is>
       </c>
       <c r="D182" s="15" t="n">
-        <v>0.883</v>
+        <v>0.903</v>
       </c>
       <c r="E182" s="15" t="n">
-        <v>0.532</v>
+        <v>0.543</v>
       </c>
       <c r="F182" s="16" t="inlineStr">
         <is>
@@ -5854,10 +5854,10 @@
         </is>
       </c>
       <c r="D183" s="19" t="n">
-        <v>0.88</v>
+        <v>0.895</v>
       </c>
       <c r="E183" s="19" t="n">
-        <v>0.478</v>
+        <v>0.605</v>
       </c>
       <c r="F183" s="16" t="inlineStr">
         <is>
@@ -5880,10 +5880,10 @@
         </is>
       </c>
       <c r="D184" s="15" t="n">
-        <v>0.878</v>
+        <v>0.885</v>
       </c>
       <c r="E184" s="15" t="n">
-        <v>0.458</v>
+        <v>0.505</v>
       </c>
       <c r="F184" s="16" t="inlineStr">
         <is>
@@ -5906,10 +5906,10 @@
         </is>
       </c>
       <c r="D185" s="19" t="n">
-        <v>0.885</v>
+        <v>0.882</v>
       </c>
       <c r="E185" s="19" t="n">
-        <v>0.364</v>
+        <v>0.353</v>
       </c>
       <c r="F185" s="16" t="inlineStr">
         <is>
@@ -5932,10 +5932,10 @@
         </is>
       </c>
       <c r="D186" s="15" t="n">
-        <v>0.883</v>
+        <v>0.88</v>
       </c>
       <c r="E186" s="15" t="n">
-        <v>0.459</v>
+        <v>0.537</v>
       </c>
       <c r="F186" s="16" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         </is>
       </c>
       <c r="D187" s="19" t="n">
-        <v>0.884</v>
+        <v>0.891</v>
       </c>
       <c r="E187" s="19" t="n">
-        <v>0.403</v>
+        <v>0.485</v>
       </c>
       <c r="F187" s="16" t="inlineStr">
         <is>
@@ -5984,10 +5984,10 @@
         </is>
       </c>
       <c r="D188" s="15" t="n">
-        <v>0.88</v>
+        <v>0.869</v>
       </c>
       <c r="E188" s="15" t="n">
-        <v>0.541</v>
+        <v>0.518</v>
       </c>
       <c r="F188" s="16" t="inlineStr">
         <is>
@@ -6006,14 +6006,14 @@
       </c>
       <c r="C189" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-IEST</t>
+          <t>COMPUTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D189" s="19" t="n">
-        <v>0.844</v>
+        <v>0.821</v>
       </c>
       <c r="E189" s="19" t="n">
-        <v>0.5</v>
+        <v>0.485</v>
       </c>
       <c r="F189" s="16" t="inlineStr">
         <is>
@@ -6032,14 +6032,14 @@
       </c>
       <c r="C190" s="14" t="inlineStr">
         <is>
-          <t>MAOHINE-LFARNING-AL-</t>
+          <t>MACHINE-LFARNING-AI-</t>
         </is>
       </c>
       <c r="D190" s="15" t="n">
-        <v>0.872</v>
+        <v>0.844</v>
       </c>
       <c r="E190" s="15" t="n">
-        <v>0.426</v>
+        <v>0.456</v>
       </c>
       <c r="F190" s="16" t="inlineStr">
         <is>
@@ -6062,10 +6062,10 @@
         </is>
       </c>
       <c r="D191" s="19" t="n">
-        <v>0.882</v>
+        <v>0.887</v>
       </c>
       <c r="E191" s="19" t="n">
-        <v>0.474</v>
+        <v>0.54</v>
       </c>
       <c r="F191" s="16" t="inlineStr">
         <is>
@@ -6084,14 +6084,14 @@
       </c>
       <c r="C192" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DFTEOT-OK</t>
+          <t>IMAGE-DATA-DFTECT-OK</t>
         </is>
       </c>
       <c r="D192" s="15" t="n">
-        <v>0.836</v>
+        <v>0.832</v>
       </c>
       <c r="E192" s="15" t="n">
-        <v>0.398</v>
+        <v>0.322</v>
       </c>
       <c r="F192" s="16" t="inlineStr">
         <is>
@@ -6114,10 +6114,10 @@
         </is>
       </c>
       <c r="D193" s="19" t="n">
-        <v>0.872</v>
+        <v>0.852</v>
       </c>
       <c r="E193" s="19" t="n">
-        <v>0.477</v>
+        <v>0.483</v>
       </c>
       <c r="F193" s="16" t="inlineStr">
         <is>
@@ -6140,10 +6140,10 @@
         </is>
       </c>
       <c r="D194" s="15" t="n">
-        <v>0.862</v>
+        <v>0.837</v>
       </c>
       <c r="E194" s="15" t="n">
-        <v>0.429</v>
+        <v>0.315</v>
       </c>
       <c r="F194" s="16" t="inlineStr">
         <is>
@@ -6162,14 +6162,14 @@
       </c>
       <c r="C195" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDKCTIDN-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D195" s="19" t="n">
-        <v>0.82</v>
+        <v>0.827</v>
       </c>
       <c r="E195" s="19" t="n">
-        <v>0.293</v>
+        <v>0.405</v>
       </c>
       <c r="F195" s="16" t="inlineStr">
         <is>
@@ -6188,14 +6188,14 @@
       </c>
       <c r="C196" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-RFEDICTIO</t>
+          <t>ARTIFICIAL-SYSIIMTIO</t>
         </is>
       </c>
       <c r="D196" s="15" t="n">
-        <v>0.715</v>
+        <v>0.729</v>
       </c>
       <c r="E196" s="15" t="n">
-        <v>0.37</v>
+        <v>0.452</v>
       </c>
       <c r="F196" s="16" t="inlineStr">
         <is>
@@ -6218,10 +6218,10 @@
         </is>
       </c>
       <c r="D197" s="19" t="n">
-        <v>0.895</v>
+        <v>0.88</v>
       </c>
       <c r="E197" s="19" t="n">
-        <v>0.538</v>
+        <v>0.503</v>
       </c>
       <c r="F197" s="16" t="inlineStr">
         <is>
@@ -6240,14 +6240,14 @@
       </c>
       <c r="C198" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEPGE-IS-POWFR--</t>
+          <t>KNOWLEDGE-IS-POWFR--</t>
         </is>
       </c>
       <c r="D198" s="15" t="n">
-        <v>0.901</v>
+        <v>0.9</v>
       </c>
       <c r="E198" s="15" t="n">
-        <v>0.464</v>
+        <v>0.541</v>
       </c>
       <c r="F198" s="16" t="inlineStr">
         <is>
@@ -6266,14 +6266,14 @@
       </c>
       <c r="C199" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FLNE-GOID</t>
+          <t>FIND-EXTRA-FINE-GOID</t>
         </is>
       </c>
       <c r="D199" s="19" t="n">
-        <v>0.824</v>
+        <v>0.827</v>
       </c>
       <c r="E199" s="19" t="n">
-        <v>0.402</v>
+        <v>0.362</v>
       </c>
       <c r="F199" s="16" t="inlineStr">
         <is>
@@ -6292,14 +6292,14 @@
       </c>
       <c r="C200" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-OLX-TEN</t>
+          <t>ZERO-ONE-TWO-CIX-TEN</t>
         </is>
       </c>
       <c r="D200" s="15" t="n">
-        <v>0.878</v>
+        <v>0.839</v>
       </c>
       <c r="E200" s="15" t="n">
-        <v>0.454</v>
+        <v>0.489</v>
       </c>
       <c r="F200" s="16" t="inlineStr">
         <is>
@@ -6318,14 +6318,14 @@
       </c>
       <c r="C201" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIGKLMNOEGRST</t>
+          <t>ABCDEFGHIJKLMNOPGPST</t>
         </is>
       </c>
       <c r="D201" s="19" t="n">
-        <v>0.8139999999999999</v>
+        <v>0.823</v>
       </c>
       <c r="E201" s="19" t="n">
-        <v>0.432</v>
+        <v>0.342</v>
       </c>
       <c r="F201" s="16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: expand benchmark to 12 sheets (95.12% Super-Ensemble) and organize project files
- Update char_classifier.pkl to 17MB Dual-Ensemble model (93.04%)
- Fix Excel export and auto-route reports for all 3 models:
  * all_results.xlsx (Super-Ensemble 95.12%)
  * all_results_ensemble.xlsx (Dual-Ensemble MLP 93.04%)
  * all_results_cnn.xlsx (Custom 2D CNN 95.04%)
- Complete 12-sheet test benchmark (including test11 and test12)
- Add create_guided_templates.py and printable templates in templete/
- Organize project documentation and move pdf_text.txt to docs/
- Clean up redundant temporary visual artifacts
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard_ภาพรวม" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$241</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -618,10 +618,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="133" customWidth="1" min="1" max="1"/>
+    <col width="113" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-25 21:28:47 | โมเดลที่ใช้ตรวจ: Super-Ensemble (MLP + CNN: 94.19%) | ตรวจทั้งหมด: 10 แผ่น | รวม 200 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-26 14:44:14 | โมเดลที่ใช้ตรวจ: Super-Ensemble | ตรวจทั้งหมด: 12 แผ่น | รวม 240 ข้อ</t>
         </is>
       </c>
     </row>
@@ -676,27 +676,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>10 แผ่น</t>
+          <t>12 แผ่น</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>200 ข้อ</t>
+          <t>240 ข้อ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>4,000 ตัว</t>
+          <t>4,800 ตัว</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>96.43%</t>
+          <t>95.12%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>197 ข้อ</t>
+          <t>176 ข้อ</t>
         </is>
       </c>
     </row>
@@ -765,12 +765,12 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>0.924</t>
+          <t>0.963</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>11 ข้อ</t>
         </is>
       </c>
       <c r="G11" s="11" t="inlineStr">
@@ -793,12 +793,12 @@
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>90.50%</t>
+          <t>83.75%</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.862</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -826,17 +826,17 @@
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>97.50%</t>
+          <t>96.25%</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>0.899</t>
+          <t>0.942</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>17 ข้อ</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -859,17 +859,17 @@
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>98.50%</t>
+          <t>99.50%</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>0.913</t>
+          <t>0.971</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>18 ข้อ</t>
+          <t>8 ข้อ</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -892,17 +892,17 @@
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>95.50%</t>
+          <t>93.75%</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>0.897</t>
+          <t>0.938</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>19 ข้อ</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -925,17 +925,17 @@
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>97.50%</t>
+          <t>97.00%</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.955</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>19 ข้อ</t>
+          <t>13 ข้อ</t>
         </is>
       </c>
       <c r="G16" s="11" t="inlineStr">
@@ -958,17 +958,17 @@
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>98.50%</t>
+          <t>97.50%</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>0.923</t>
+          <t>0.963</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>11 ข้อ</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -991,17 +991,17 @@
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>97.50%</t>
+          <t>95.25%</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.917</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>18 ข้อ</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -1024,17 +1024,17 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>95.00%</t>
+          <t>94.00%</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>0.871</t>
+          <t>0.919</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>20 ข้อ</t>
+          <t>18 ข้อ</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>94.50%</t>
+          <t>88.25%</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>0.855</t>
+          <t>0.884</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -1071,6 +1071,72 @@
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>97.75%</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>0.956</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>14 ข้อ</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>99.25%</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>7 ข้อ</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
         <is>
           <t>English &amp; Tech (ชุดที่ 1)</t>
         </is>
@@ -1090,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
+  <dimension ref="A1:F241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1148,10 +1214,10 @@
         </is>
       </c>
       <c r="D2" s="15" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.965</v>
       </c>
       <c r="E2" s="15" t="n">
-        <v>0.587</v>
+        <v>0.79</v>
       </c>
       <c r="F2" s="16" t="inlineStr">
         <is>
@@ -1170,14 +1236,14 @@
       </c>
       <c r="C3" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>JUMPS-OVER-LAZY-COG-</t>
         </is>
       </c>
       <c r="D3" s="19" t="n">
-        <v>0.917</v>
+        <v>0.949</v>
       </c>
       <c r="E3" s="19" t="n">
-        <v>0.318</v>
+        <v>0.355</v>
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
@@ -1200,10 +1266,10 @@
         </is>
       </c>
       <c r="D4" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.965</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>0.603</v>
+        <v>0.775</v>
       </c>
       <c r="F4" s="16" t="inlineStr">
         <is>
@@ -1226,14 +1292,14 @@
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.915</v>
+        <v>0.969</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.721</v>
-      </c>
-      <c r="F5" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1248,18 +1314,18 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OE-BLACK-GEM-</t>
+          <t>SPHINX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D6" s="15" t="n">
-        <v>0.96</v>
+        <v>0.978</v>
       </c>
       <c r="E6" s="15" t="n">
-        <v>0.721</v>
-      </c>
-      <c r="F6" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.884</v>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1278,14 +1344,14 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>0.924</v>
+        <v>0.967</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>0.666</v>
-      </c>
-      <c r="F7" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.851</v>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1304,14 +1370,14 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.955</v>
+        <v>0.988</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>0.723</v>
-      </c>
-      <c r="F8" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.963</v>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1330,10 +1396,10 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>0.909</v>
+        <v>0.966</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>0.666</v>
+        <v>0.783</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
@@ -1356,10 +1422,10 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.953</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>0.594</v>
+        <v>0.538</v>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
@@ -1382,10 +1448,10 @@
         </is>
       </c>
       <c r="D11" s="19" t="n">
-        <v>0.912</v>
+        <v>0.956</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.638</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -1408,10 +1474,10 @@
         </is>
       </c>
       <c r="D12" s="15" t="n">
-        <v>0.873</v>
+        <v>0.93</v>
       </c>
       <c r="E12" s="15" t="n">
-        <v>0.536</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
@@ -1434,14 +1500,14 @@
         </is>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.945</v>
+        <v>0.989</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.794</v>
-      </c>
-      <c r="F13" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.946</v>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1460,14 +1526,14 @@
         </is>
       </c>
       <c r="D14" s="15" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.981</v>
       </c>
       <c r="E14" s="15" t="n">
-        <v>0.733</v>
-      </c>
-      <c r="F14" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.874</v>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1486,14 +1552,14 @@
         </is>
       </c>
       <c r="D15" s="19" t="n">
-        <v>0.924</v>
+        <v>0.966</v>
       </c>
       <c r="E15" s="19" t="n">
-        <v>0.753</v>
-      </c>
-      <c r="F15" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1512,10 +1578,10 @@
         </is>
       </c>
       <c r="D16" s="15" t="n">
-        <v>0.894</v>
+        <v>0.922</v>
       </c>
       <c r="E16" s="15" t="n">
-        <v>0.598</v>
+        <v>0.467</v>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
@@ -1538,14 +1604,14 @@
         </is>
       </c>
       <c r="D17" s="19" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.975</v>
       </c>
       <c r="E17" s="19" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.878</v>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1564,10 +1630,10 @@
         </is>
       </c>
       <c r="D18" s="15" t="n">
-        <v>0.948</v>
+        <v>0.968</v>
       </c>
       <c r="E18" s="15" t="n">
-        <v>0.74</v>
+        <v>0.671</v>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
@@ -1590,10 +1656,10 @@
         </is>
       </c>
       <c r="D19" s="19" t="n">
-        <v>0.886</v>
+        <v>0.948</v>
       </c>
       <c r="E19" s="19" t="n">
-        <v>0.651</v>
+        <v>0.622</v>
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
@@ -1616,10 +1682,10 @@
         </is>
       </c>
       <c r="D20" s="15" t="n">
-        <v>0.891</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="E20" s="15" t="n">
-        <v>0.413</v>
+        <v>0.548</v>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
@@ -1642,14 +1708,14 @@
         </is>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.977</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.746</v>
-      </c>
-      <c r="F21" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.88</v>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -1664,14 +1730,14 @@
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>TIL-QUICK-BROWN-FOX-</t>
+          <t>TIL-QUICK-BROWN-FCX-</t>
         </is>
       </c>
       <c r="D22" s="15" t="n">
-        <v>0.872</v>
+        <v>0.88</v>
       </c>
       <c r="E22" s="15" t="n">
-        <v>0.467</v>
+        <v>0.474</v>
       </c>
       <c r="F22" s="16" t="inlineStr">
         <is>
@@ -1690,14 +1756,14 @@
       </c>
       <c r="C23" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>JUMMS-OVER-LAZY-CQG-</t>
         </is>
       </c>
       <c r="D23" s="19" t="n">
-        <v>0.901</v>
+        <v>0.887</v>
       </c>
       <c r="E23" s="19" t="n">
-        <v>0.288</v>
+        <v>0.524</v>
       </c>
       <c r="F23" s="16" t="inlineStr">
         <is>
@@ -1720,10 +1786,10 @@
         </is>
       </c>
       <c r="D24" s="15" t="n">
-        <v>0.926</v>
+        <v>0.948</v>
       </c>
       <c r="E24" s="15" t="n">
-        <v>0.598</v>
+        <v>0.715</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
@@ -1742,14 +1808,14 @@
       </c>
       <c r="C25" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOR-JU</t>
+          <t>FIVE-DOZEN-LIQUQR-JU</t>
         </is>
       </c>
       <c r="D25" s="19" t="n">
-        <v>0.875</v>
+        <v>0.845</v>
       </c>
       <c r="E25" s="19" t="n">
-        <v>0.487</v>
+        <v>0.433</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -1768,14 +1834,14 @@
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLACK-GEM-</t>
+          <t>SPHUNX-OF-BLACK-GFM-</t>
         </is>
       </c>
       <c r="D26" s="15" t="n">
-        <v>0.858</v>
+        <v>0.895</v>
       </c>
       <c r="E26" s="15" t="n">
-        <v>0.42</v>
+        <v>0.456</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -1798,10 +1864,10 @@
         </is>
       </c>
       <c r="D27" s="19" t="n">
-        <v>0.859</v>
+        <v>0.899</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>0.583</v>
+        <v>0.532</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -1820,14 +1886,14 @@
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>RR-GHI-ZEPHYRS-ILOW-</t>
+          <t>BR-GHI-LEPHYRS-ELOW-</t>
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.844</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.308</v>
+        <v>0.189</v>
       </c>
       <c r="F28" s="16" t="inlineStr">
         <is>
@@ -1846,14 +1912,14 @@
       </c>
       <c r="C29" s="18" t="inlineStr">
         <is>
-          <t>COMPUIER-VISION-TEST</t>
+          <t>COMPUIER-VISION-TESE</t>
         </is>
       </c>
       <c r="D29" s="19" t="n">
-        <v>0.862</v>
+        <v>0.88</v>
       </c>
       <c r="E29" s="19" t="n">
-        <v>0.404</v>
+        <v>0.152</v>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
@@ -1876,10 +1942,10 @@
         </is>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.894</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.45</v>
+        <v>0.649</v>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
@@ -1898,14 +1964,14 @@
       </c>
       <c r="C31" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NFTWORKS</t>
+          <t>DEEP-NEURAU-NFTWORKS</t>
         </is>
       </c>
       <c r="D31" s="19" t="n">
-        <v>0.773</v>
+        <v>0.78</v>
       </c>
       <c r="E31" s="19" t="n">
-        <v>0.34</v>
+        <v>0.367</v>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
@@ -1924,14 +1990,14 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>-MAGE-PATA-DETFCT-CK</t>
+          <t>-MAGE-DATA-DELFCT-CK</t>
         </is>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.766</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.43</v>
+        <v>0.36</v>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
@@ -1950,14 +2016,14 @@
       </c>
       <c r="C33" s="18" t="inlineStr">
         <is>
-          <t>DYIHON-OPENCV-BORCT-</t>
+          <t>DYIHON-OPFNCV-BOBCT-</t>
         </is>
       </c>
       <c r="D33" s="19" t="n">
-        <v>0.755</v>
+        <v>0.9</v>
       </c>
       <c r="E33" s="19" t="n">
-        <v>0.368</v>
+        <v>0.613</v>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
@@ -1976,14 +2042,14 @@
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-RECOGNIZE-</t>
+          <t>SMART-CCR-BECCGWIZE-</t>
         </is>
       </c>
       <c r="D34" s="15" t="n">
-        <v>0.788</v>
+        <v>0.844</v>
       </c>
       <c r="E34" s="15" t="n">
-        <v>0.343</v>
+        <v>0.383</v>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
@@ -2002,14 +2068,14 @@
       </c>
       <c r="C35" s="18" t="inlineStr">
         <is>
-          <t>AOCURATF--REDQCTJON-</t>
+          <t>ACCUKATF--BEDICTJBA-</t>
         </is>
       </c>
       <c r="D35" s="19" t="n">
-        <v>0.716</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="E35" s="19" t="n">
-        <v>0.301</v>
+        <v>0.296</v>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
@@ -2032,10 +2098,10 @@
         </is>
       </c>
       <c r="D36" s="15" t="n">
-        <v>0.792</v>
+        <v>0.858</v>
       </c>
       <c r="E36" s="15" t="n">
-        <v>0.427</v>
+        <v>0.499</v>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
@@ -2054,14 +2120,14 @@
       </c>
       <c r="C37" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-ZELOOME-</t>
+          <t>HELLC-WOFLD-VELOCME-</t>
         </is>
       </c>
       <c r="D37" s="19" t="n">
-        <v>0.786</v>
+        <v>0.834</v>
       </c>
       <c r="E37" s="19" t="n">
-        <v>0.299</v>
+        <v>0.201</v>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
@@ -2080,14 +2146,14 @@
       </c>
       <c r="C38" s="14" t="inlineStr">
         <is>
-          <t>KNOWL-OGF-IS-POWER--</t>
+          <t>KNOWL-CCFCIS-PQWEB--</t>
         </is>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.79</v>
+        <v>0.875</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.417</v>
+        <v>0.368</v>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
@@ -2106,14 +2172,14 @@
       </c>
       <c r="C39" s="18" t="inlineStr">
         <is>
-          <t>FIND-FXTRA-FINE-GOLD</t>
+          <t>FIND-FXTRA-EINF-GDLD</t>
         </is>
       </c>
       <c r="D39" s="19" t="n">
-        <v>0.844</v>
+        <v>0.835</v>
       </c>
       <c r="E39" s="19" t="n">
-        <v>0.452</v>
+        <v>0.266</v>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
@@ -2132,14 +2198,14 @@
       </c>
       <c r="C40" s="14" t="inlineStr">
         <is>
-          <t>ZFRO-ONF--WG-SIX-TEN</t>
+          <t>ZERQ-ONF--WG-SIX-TEN</t>
         </is>
       </c>
       <c r="D40" s="15" t="n">
-        <v>0.831</v>
+        <v>0.829</v>
       </c>
       <c r="E40" s="15" t="n">
-        <v>0.494</v>
+        <v>0.415</v>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
@@ -2158,14 +2224,14 @@
       </c>
       <c r="C41" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKL-NOPGRST</t>
+          <t>ABCDEFGHIJKL-NCHGRST</t>
         </is>
       </c>
       <c r="D41" s="19" t="n">
-        <v>0.771</v>
+        <v>0.837</v>
       </c>
       <c r="E41" s="19" t="n">
-        <v>0.491</v>
+        <v>0.189</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
@@ -2188,10 +2254,10 @@
         </is>
       </c>
       <c r="D42" s="15" t="n">
-        <v>0.911</v>
+        <v>0.963</v>
       </c>
       <c r="E42" s="15" t="n">
-        <v>0.577</v>
+        <v>0.77</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -2214,10 +2280,10 @@
         </is>
       </c>
       <c r="D43" s="19" t="n">
-        <v>0.91</v>
+        <v>0.955</v>
       </c>
       <c r="E43" s="19" t="n">
-        <v>0.585</v>
+        <v>0.63</v>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
@@ -2236,14 +2302,14 @@
       </c>
       <c r="C44" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-ROX-WITH-TEA</t>
+          <t>DACK-MY-ROX-WITH-TEA</t>
         </is>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.887</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.366</v>
+        <v>0.347</v>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
@@ -2266,14 +2332,14 @@
         </is>
       </c>
       <c r="D45" s="19" t="n">
-        <v>0.929</v>
+        <v>0.96</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.737</v>
-      </c>
-      <c r="F45" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.824</v>
+      </c>
+      <c r="F45" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2288,18 +2354,18 @@
       </c>
       <c r="C46" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLADK-GEM-</t>
+          <t>SPHINX-OF-BLHCK-GEM-</t>
         </is>
       </c>
       <c r="D46" s="15" t="n">
-        <v>0.928</v>
+        <v>0.946</v>
       </c>
       <c r="E46" s="15" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="F46" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="F46" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2318,10 +2384,10 @@
         </is>
       </c>
       <c r="D47" s="19" t="n">
-        <v>0.919</v>
+        <v>0.958</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>0.608</v>
+        <v>0.67</v>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
@@ -2344,10 +2410,10 @@
         </is>
       </c>
       <c r="D48" s="15" t="n">
-        <v>0.925</v>
+        <v>0.948</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.596</v>
+        <v>0.708</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
@@ -2370,10 +2436,10 @@
         </is>
       </c>
       <c r="D49" s="19" t="n">
-        <v>0.893</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E49" s="19" t="n">
-        <v>0.553</v>
+        <v>0.579</v>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
@@ -2392,14 +2458,14 @@
       </c>
       <c r="C50" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNING-AI-</t>
+          <t>MACHTNE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D50" s="15" t="n">
         <v>0.96</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.797</v>
+        <v>0.506</v>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
@@ -2422,10 +2488,10 @@
         </is>
       </c>
       <c r="D51" s="19" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.964</v>
       </c>
       <c r="E51" s="19" t="n">
-        <v>0.738</v>
+        <v>0.789</v>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
@@ -2448,10 +2514,10 @@
         </is>
       </c>
       <c r="D52" s="15" t="n">
-        <v>0.915</v>
+        <v>0.97</v>
       </c>
       <c r="E52" s="15" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
@@ -2470,14 +2536,14 @@
       </c>
       <c r="C53" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-DPENOV-ROBOT-</t>
+          <t>SYTHONPDPENUVRROBDT-</t>
         </is>
       </c>
       <c r="D53" s="19" t="n">
-        <v>0.783</v>
+        <v>0.848</v>
       </c>
       <c r="E53" s="19" t="n">
-        <v>0.338</v>
+        <v>0.313</v>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
@@ -2496,14 +2562,14 @@
       </c>
       <c r="C54" s="14" t="inlineStr">
         <is>
-          <t>SMART-ORD-RECOGNIZE-</t>
+          <t>SMART-ORC-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D54" s="15" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E54" s="15" t="n">
-        <v>0.574</v>
+        <v>0.731</v>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
@@ -2522,14 +2588,14 @@
       </c>
       <c r="C55" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDIDTION-</t>
+          <t>ACCURATE-PREDICTION-</t>
         </is>
       </c>
       <c r="D55" s="19" t="n">
-        <v>0.853</v>
+        <v>0.918</v>
       </c>
       <c r="E55" s="19" t="n">
-        <v>0.583</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
@@ -2552,10 +2618,10 @@
         </is>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.863</v>
+        <v>0.9</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.474</v>
+        <v>0.462</v>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
@@ -2578,10 +2644,10 @@
         </is>
       </c>
       <c r="D57" s="19" t="n">
-        <v>0.877</v>
+        <v>0.923</v>
       </c>
       <c r="E57" s="19" t="n">
-        <v>0.438</v>
+        <v>0.404</v>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
@@ -2604,10 +2670,10 @@
         </is>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.886</v>
+        <v>0.93</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.522</v>
+        <v>0.575</v>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
@@ -2630,10 +2696,10 @@
         </is>
       </c>
       <c r="D59" s="19" t="n">
-        <v>0.888</v>
+        <v>0.955</v>
       </c>
       <c r="E59" s="19" t="n">
-        <v>0.541</v>
+        <v>0.589</v>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
@@ -2656,10 +2722,10 @@
         </is>
       </c>
       <c r="D60" s="15" t="n">
-        <v>0.887</v>
+        <v>0.945</v>
       </c>
       <c r="E60" s="15" t="n">
-        <v>0.509</v>
+        <v>0.298</v>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
@@ -2682,14 +2748,14 @@
         </is>
       </c>
       <c r="D61" s="19" t="n">
-        <v>0.927</v>
+        <v>0.978</v>
       </c>
       <c r="E61" s="19" t="n">
-        <v>0.718</v>
-      </c>
-      <c r="F61" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.907</v>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2708,14 +2774,14 @@
         </is>
       </c>
       <c r="D62" s="15" t="n">
-        <v>0.91</v>
+        <v>0.97</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>0.664</v>
-      </c>
-      <c r="F62" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.861</v>
+      </c>
+      <c r="F62" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2734,10 +2800,10 @@
         </is>
       </c>
       <c r="D63" s="19" t="n">
-        <v>0.918</v>
+        <v>0.967</v>
       </c>
       <c r="E63" s="19" t="n">
-        <v>0.59</v>
+        <v>0.629</v>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
@@ -2760,10 +2826,10 @@
         </is>
       </c>
       <c r="D64" s="15" t="n">
-        <v>0.896</v>
+        <v>0.966</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.512</v>
+        <v>0.766</v>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
@@ -2786,14 +2852,14 @@
         </is>
       </c>
       <c r="D65" s="19" t="n">
-        <v>0.931</v>
+        <v>0.979</v>
       </c>
       <c r="E65" s="19" t="n">
-        <v>0.636</v>
-      </c>
-      <c r="F65" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.909</v>
+      </c>
+      <c r="F65" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2812,10 +2878,10 @@
         </is>
       </c>
       <c r="D66" s="15" t="n">
-        <v>0.963</v>
+        <v>0.984</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.826</v>
+        <v>0.884</v>
       </c>
       <c r="F66" s="20" t="inlineStr">
         <is>
@@ -2838,10 +2904,10 @@
         </is>
       </c>
       <c r="D67" s="19" t="n">
-        <v>0.896</v>
+        <v>0.954</v>
       </c>
       <c r="E67" s="19" t="n">
-        <v>0.592</v>
+        <v>0.495</v>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
@@ -2864,14 +2930,14 @@
         </is>
       </c>
       <c r="D68" s="15" t="n">
-        <v>0.95</v>
+        <v>0.986</v>
       </c>
       <c r="E68" s="15" t="n">
-        <v>0.646</v>
-      </c>
-      <c r="F68" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.918</v>
+      </c>
+      <c r="F68" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2890,14 +2956,14 @@
         </is>
       </c>
       <c r="D69" s="19" t="n">
-        <v>0.892</v>
+        <v>0.976</v>
       </c>
       <c r="E69" s="19" t="n">
-        <v>0.632</v>
-      </c>
-      <c r="F69" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.849</v>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2912,14 +2978,14 @@
       </c>
       <c r="C70" s="14" t="inlineStr">
         <is>
-          <t>MAOHINE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.973</v>
+        <v>0.981</v>
       </c>
       <c r="E70" s="15" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.885</v>
       </c>
       <c r="F70" s="20" t="inlineStr">
         <is>
@@ -2942,10 +3008,10 @@
         </is>
       </c>
       <c r="D71" s="19" t="n">
-        <v>0.912</v>
+        <v>0.949</v>
       </c>
       <c r="E71" s="19" t="n">
-        <v>0.487</v>
+        <v>0.481</v>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
@@ -2964,18 +3030,18 @@
       </c>
       <c r="C72" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETEOT-OK</t>
+          <t>IMAGE-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D72" s="15" t="n">
-        <v>0.915</v>
+        <v>0.975</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>0.717</v>
-      </c>
-      <c r="F72" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.885</v>
+      </c>
+      <c r="F72" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -2994,14 +3060,14 @@
         </is>
       </c>
       <c r="D73" s="19" t="n">
-        <v>0.872</v>
+        <v>0.977</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="F73" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.834</v>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3016,18 +3082,18 @@
       </c>
       <c r="C74" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-REOOGNIZE-</t>
+          <t>SMART-OCR-RECOGNIZE-</t>
         </is>
       </c>
       <c r="D74" s="15" t="n">
-        <v>0.911</v>
+        <v>0.98</v>
       </c>
       <c r="E74" s="15" t="n">
-        <v>0.662</v>
-      </c>
-      <c r="F74" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.918</v>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3046,10 +3112,10 @@
         </is>
       </c>
       <c r="D75" s="19" t="n">
-        <v>0.869</v>
+        <v>0.958</v>
       </c>
       <c r="E75" s="19" t="n">
-        <v>0.6</v>
+        <v>0.793</v>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
@@ -3072,14 +3138,14 @@
         </is>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.916</v>
+        <v>0.978</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>0.663</v>
-      </c>
-      <c r="F76" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.84</v>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3098,10 +3164,10 @@
         </is>
       </c>
       <c r="D77" s="19" t="n">
-        <v>0.918</v>
+        <v>0.969</v>
       </c>
       <c r="E77" s="19" t="n">
-        <v>0.626</v>
+        <v>0.627</v>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
@@ -3120,18 +3186,18 @@
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>KNOWKEDGE-IS-POWER--</t>
+          <t>KNOWLEDGE-IS-POWER--</t>
         </is>
       </c>
       <c r="D78" s="15" t="n">
-        <v>0.899</v>
+        <v>0.981</v>
       </c>
       <c r="E78" s="15" t="n">
-        <v>0.266</v>
-      </c>
-      <c r="F78" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.805</v>
+      </c>
+      <c r="F78" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3150,10 +3216,10 @@
         </is>
       </c>
       <c r="D79" s="19" t="n">
-        <v>0.887</v>
+        <v>0.949</v>
       </c>
       <c r="E79" s="19" t="n">
-        <v>0.543</v>
+        <v>0.57</v>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
@@ -3176,14 +3242,14 @@
         </is>
       </c>
       <c r="D80" s="15" t="n">
-        <v>0.926</v>
+        <v>0.979</v>
       </c>
       <c r="E80" s="15" t="n">
-        <v>0.6870000000000001</v>
-      </c>
-      <c r="F80" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.89</v>
+      </c>
+      <c r="F80" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3202,10 +3268,10 @@
         </is>
       </c>
       <c r="D81" s="19" t="n">
-        <v>0.904</v>
+        <v>0.956</v>
       </c>
       <c r="E81" s="19" t="n">
-        <v>0.606</v>
+        <v>0.512</v>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
@@ -3224,14 +3290,14 @@
       </c>
       <c r="C82" s="14" t="inlineStr">
         <is>
-          <t>THE-QUTDK-BROWN-FOX-</t>
+          <t>THE-QUTCK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D82" s="15" t="n">
-        <v>0.921</v>
+        <v>0.961</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.413</v>
+        <v>0.762</v>
       </c>
       <c r="F82" s="16" t="inlineStr">
         <is>
@@ -3250,14 +3316,14 @@
       </c>
       <c r="C83" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-LAZY-DOG-</t>
+          <t>JUMPS-OVFR-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D83" s="19" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.969</v>
       </c>
       <c r="E83" s="19" t="n">
-        <v>0.513</v>
+        <v>0.583</v>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
@@ -3280,10 +3346,10 @@
         </is>
       </c>
       <c r="D84" s="15" t="n">
-        <v>0.927</v>
+        <v>0.963</v>
       </c>
       <c r="E84" s="15" t="n">
-        <v>0.602</v>
+        <v>0.766</v>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
@@ -3306,10 +3372,10 @@
         </is>
       </c>
       <c r="D85" s="19" t="n">
-        <v>0.924</v>
+        <v>0.963</v>
       </c>
       <c r="E85" s="19" t="n">
-        <v>0.622</v>
+        <v>0.771</v>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
@@ -3328,14 +3394,14 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>SPHJNX-OF-RLACK-GEM-</t>
+          <t>SPHJNX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D86" s="15" t="n">
-        <v>0.894</v>
+        <v>0.963</v>
       </c>
       <c r="E86" s="15" t="n">
-        <v>0.59</v>
+        <v>0.725</v>
       </c>
       <c r="F86" s="16" t="inlineStr">
         <is>
@@ -3358,14 +3424,14 @@
         </is>
       </c>
       <c r="D87" s="19" t="n">
-        <v>0.954</v>
+        <v>0.978</v>
       </c>
       <c r="E87" s="19" t="n">
-        <v>0.765</v>
-      </c>
-      <c r="F87" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.887</v>
+      </c>
+      <c r="F87" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3380,14 +3446,14 @@
       </c>
       <c r="C88" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+          <t>BRIGHT-ZFPHYRS-BLOW-</t>
         </is>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.895</v>
+        <v>0.949</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.472</v>
+        <v>0.511</v>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
@@ -3406,14 +3472,14 @@
       </c>
       <c r="C89" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISTON-TEST</t>
+          <t>COMPUTER-VIJTON-TEST</t>
         </is>
       </c>
       <c r="D89" s="19" t="n">
-        <v>0.856</v>
+        <v>0.889</v>
       </c>
       <c r="E89" s="19" t="n">
-        <v>0.539</v>
+        <v>0.405</v>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
@@ -3432,14 +3498,14 @@
       </c>
       <c r="C90" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LEARNJNG-AI-</t>
+          <t>MACHTNE-LFARNJNW-AI-</t>
         </is>
       </c>
       <c r="D90" s="15" t="n">
-        <v>0.868</v>
+        <v>0.909</v>
       </c>
       <c r="E90" s="15" t="n">
-        <v>0.406</v>
+        <v>0.555</v>
       </c>
       <c r="F90" s="16" t="inlineStr">
         <is>
@@ -3458,14 +3524,14 @@
       </c>
       <c r="C91" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEED-NEURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D91" s="19" t="n">
-        <v>0.917</v>
+        <v>0.925</v>
       </c>
       <c r="E91" s="19" t="n">
-        <v>0.647</v>
+        <v>0.528</v>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
@@ -3488,10 +3554,10 @@
         </is>
       </c>
       <c r="D92" s="15" t="n">
-        <v>0.888</v>
+        <v>0.955</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.525</v>
+        <v>0.788</v>
       </c>
       <c r="F92" s="16" t="inlineStr">
         <is>
@@ -3514,10 +3580,10 @@
         </is>
       </c>
       <c r="D93" s="19" t="n">
-        <v>0.889</v>
+        <v>0.969</v>
       </c>
       <c r="E93" s="19" t="n">
-        <v>0.545</v>
+        <v>0.769</v>
       </c>
       <c r="F93" s="16" t="inlineStr">
         <is>
@@ -3540,10 +3606,10 @@
         </is>
       </c>
       <c r="D94" s="15" t="n">
-        <v>0.922</v>
+        <v>0.924</v>
       </c>
       <c r="E94" s="15" t="n">
-        <v>0.703</v>
+        <v>0.7</v>
       </c>
       <c r="F94" s="16" t="inlineStr">
         <is>
@@ -3562,14 +3628,14 @@
       </c>
       <c r="C95" s="18" t="inlineStr">
         <is>
-          <t>ACCURATF-PREDICTION-</t>
+          <t>ACCURATF-PREPICTION-</t>
         </is>
       </c>
       <c r="D95" s="19" t="n">
-        <v>0.897</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E95" s="19" t="n">
-        <v>0.554</v>
+        <v>0.516</v>
       </c>
       <c r="F95" s="16" t="inlineStr">
         <is>
@@ -3592,10 +3658,10 @@
         </is>
       </c>
       <c r="D96" s="15" t="n">
-        <v>0.868</v>
+        <v>0.905</v>
       </c>
       <c r="E96" s="15" t="n">
-        <v>0.513</v>
+        <v>0.533</v>
       </c>
       <c r="F96" s="16" t="inlineStr">
         <is>
@@ -3618,10 +3684,10 @@
         </is>
       </c>
       <c r="D97" s="19" t="n">
-        <v>0.861</v>
+        <v>0.925</v>
       </c>
       <c r="E97" s="19" t="n">
-        <v>0.507</v>
+        <v>0.473</v>
       </c>
       <c r="F97" s="16" t="inlineStr">
         <is>
@@ -3640,14 +3706,14 @@
       </c>
       <c r="C98" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEOGE-IS-PONER--</t>
+          <t>KNOWLEOGE-IS-POWEF--</t>
         </is>
       </c>
       <c r="D98" s="15" t="n">
-        <v>0.887</v>
+        <v>0.927</v>
       </c>
       <c r="E98" s="15" t="n">
-        <v>0.547</v>
+        <v>0.391</v>
       </c>
       <c r="F98" s="16" t="inlineStr">
         <is>
@@ -3666,14 +3732,14 @@
       </c>
       <c r="C99" s="18" t="inlineStr">
         <is>
-          <t>F-ND-EETRA-FIND-GOLD</t>
+          <t>F-ND-FXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D99" s="19" t="n">
-        <v>0.839</v>
+        <v>0.878</v>
       </c>
       <c r="E99" s="19" t="n">
-        <v>0.396</v>
+        <v>0.464</v>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
@@ -3692,14 +3758,14 @@
       </c>
       <c r="C100" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-SIX-TEN</t>
+          <t>ZERO-ONE-TWO-SIX-TRN</t>
         </is>
       </c>
       <c r="D100" s="15" t="n">
-        <v>0.897</v>
+        <v>0.931</v>
       </c>
       <c r="E100" s="15" t="n">
-        <v>0.384</v>
+        <v>0.369</v>
       </c>
       <c r="F100" s="16" t="inlineStr">
         <is>
@@ -3722,10 +3788,10 @@
         </is>
       </c>
       <c r="D101" s="19" t="n">
-        <v>0.893</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E101" s="19" t="n">
-        <v>0.535</v>
+        <v>0.649</v>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
@@ -3744,14 +3810,14 @@
       </c>
       <c r="C102" s="14" t="inlineStr">
         <is>
-          <t>THE-QUTCK-BROWN-FOX-</t>
+          <t>THF-QUTCK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D102" s="15" t="n">
-        <v>0.875</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E102" s="15" t="n">
-        <v>0.506</v>
+        <v>0.595</v>
       </c>
       <c r="F102" s="16" t="inlineStr">
         <is>
@@ -3774,10 +3840,10 @@
         </is>
       </c>
       <c r="D103" s="19" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="E103" s="19" t="n">
-        <v>0.511</v>
+        <v>0.51</v>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
@@ -3800,10 +3866,10 @@
         </is>
       </c>
       <c r="D104" s="15" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.967</v>
       </c>
       <c r="E104" s="15" t="n">
-        <v>0.589</v>
+        <v>0.677</v>
       </c>
       <c r="F104" s="16" t="inlineStr">
         <is>
@@ -3826,14 +3892,14 @@
         </is>
       </c>
       <c r="D105" s="19" t="n">
-        <v>0.892</v>
+        <v>0.959</v>
       </c>
       <c r="E105" s="19" t="n">
-        <v>0.486</v>
-      </c>
-      <c r="F105" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.806</v>
+      </c>
+      <c r="F105" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3852,10 +3918,10 @@
         </is>
       </c>
       <c r="D106" s="15" t="n">
-        <v>0.917</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="E106" s="15" t="n">
-        <v>0.679</v>
+        <v>0.415</v>
       </c>
       <c r="F106" s="16" t="inlineStr">
         <is>
@@ -3878,14 +3944,14 @@
         </is>
       </c>
       <c r="D107" s="19" t="n">
-        <v>0.946</v>
+        <v>0.969</v>
       </c>
       <c r="E107" s="19" t="n">
-        <v>0.656</v>
-      </c>
-      <c r="F107" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.829</v>
+      </c>
+      <c r="F107" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -3904,10 +3970,10 @@
         </is>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.945</v>
+        <v>0.929</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.656</v>
+        <v>0.57</v>
       </c>
       <c r="F108" s="16" t="inlineStr">
         <is>
@@ -3930,10 +3996,10 @@
         </is>
       </c>
       <c r="D109" s="19" t="n">
-        <v>0.911</v>
+        <v>0.955</v>
       </c>
       <c r="E109" s="19" t="n">
-        <v>0.61</v>
+        <v>0.771</v>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
@@ -3956,10 +4022,10 @@
         </is>
       </c>
       <c r="D110" s="15" t="n">
-        <v>0.977</v>
+        <v>0.984</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.881</v>
+        <v>0.893</v>
       </c>
       <c r="F110" s="20" t="inlineStr">
         <is>
@@ -3982,14 +4048,14 @@
         </is>
       </c>
       <c r="D111" s="19" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.982</v>
       </c>
       <c r="E111" s="19" t="n">
-        <v>0.6929999999999999</v>
-      </c>
-      <c r="F111" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.847</v>
+      </c>
+      <c r="F111" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4008,14 +4074,14 @@
         </is>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.868</v>
+        <v>0.973</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.501</v>
-      </c>
-      <c r="F112" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.82</v>
+      </c>
+      <c r="F112" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4030,14 +4096,14 @@
       </c>
       <c r="C113" s="18" t="inlineStr">
         <is>
-          <t>PPTHON-OPENCV-ROBOT-</t>
+          <t>PVTHON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D113" s="19" t="n">
-        <v>0.885</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="E113" s="19" t="n">
-        <v>0.303</v>
+        <v>0.484</v>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
@@ -4060,10 +4126,10 @@
         </is>
       </c>
       <c r="D114" s="15" t="n">
-        <v>0.884</v>
+        <v>0.967</v>
       </c>
       <c r="E114" s="15" t="n">
-        <v>0.613</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="F114" s="16" t="inlineStr">
         <is>
@@ -4086,10 +4152,10 @@
         </is>
       </c>
       <c r="D115" s="19" t="n">
-        <v>0.854</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="E115" s="19" t="n">
-        <v>0.487</v>
+        <v>0.517</v>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
@@ -4108,14 +4174,14 @@
       </c>
       <c r="C116" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICTAL-SYSTEM-OK</t>
+          <t>ADTIFTCTAL-SYSTEM-OK</t>
         </is>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.915</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.448</v>
+        <v>0.504</v>
       </c>
       <c r="F116" s="16" t="inlineStr">
         <is>
@@ -4138,10 +4204,10 @@
         </is>
       </c>
       <c r="D117" s="19" t="n">
-        <v>0.876</v>
+        <v>0.947</v>
       </c>
       <c r="E117" s="19" t="n">
-        <v>0.583</v>
+        <v>0.521</v>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
@@ -4164,14 +4230,14 @@
         </is>
       </c>
       <c r="D118" s="15" t="n">
-        <v>0.916</v>
+        <v>0.988</v>
       </c>
       <c r="E118" s="15" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="F118" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.946</v>
+      </c>
+      <c r="F118" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4190,10 +4256,10 @@
         </is>
       </c>
       <c r="D119" s="19" t="n">
-        <v>0.9</v>
+        <v>0.962</v>
       </c>
       <c r="E119" s="19" t="n">
-        <v>0.696</v>
+        <v>0.781</v>
       </c>
       <c r="F119" s="16" t="inlineStr">
         <is>
@@ -4216,14 +4282,14 @@
         </is>
       </c>
       <c r="D120" s="15" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="E120" s="15" t="n">
-        <v>0.591</v>
-      </c>
-      <c r="F120" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.871</v>
+      </c>
+      <c r="F120" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4238,14 +4304,14 @@
       </c>
       <c r="C121" s="18" t="inlineStr">
         <is>
-          <t>ABDDEFGHIJKLMNOPORST</t>
+          <t>ABCDEFGHIJKLMNOPORST</t>
         </is>
       </c>
       <c r="D121" s="19" t="n">
-        <v>0.845</v>
+        <v>0.912</v>
       </c>
       <c r="E121" s="19" t="n">
-        <v>0.375</v>
+        <v>0.433</v>
       </c>
       <c r="F121" s="16" t="inlineStr">
         <is>
@@ -4264,18 +4330,18 @@
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>THE-QUIOK-BROWN-FOX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D122" s="15" t="n">
-        <v>0.917</v>
+        <v>0.974</v>
       </c>
       <c r="E122" s="15" t="n">
-        <v>0.642</v>
-      </c>
-      <c r="F122" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.836</v>
+      </c>
+      <c r="F122" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4294,14 +4360,14 @@
         </is>
       </c>
       <c r="D123" s="19" t="n">
-        <v>0.9389999999999999</v>
+        <v>0.98</v>
       </c>
       <c r="E123" s="19" t="n">
-        <v>0.556</v>
-      </c>
-      <c r="F123" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.889</v>
+      </c>
+      <c r="F123" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4316,14 +4382,14 @@
       </c>
       <c r="C124" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOX-WITH-TEA</t>
+          <t>PACK-MY-BOXCWITH-TEA</t>
         </is>
       </c>
       <c r="D124" s="15" t="n">
-        <v>0.926</v>
+        <v>0.9370000000000001</v>
       </c>
       <c r="E124" s="15" t="n">
-        <v>0.597</v>
+        <v>0.151</v>
       </c>
       <c r="F124" s="16" t="inlineStr">
         <is>
@@ -4346,14 +4412,14 @@
         </is>
       </c>
       <c r="D125" s="19" t="n">
-        <v>0.93</v>
+        <v>0.971</v>
       </c>
       <c r="E125" s="19" t="n">
-        <v>0.6830000000000001</v>
-      </c>
-      <c r="F125" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.829</v>
+      </c>
+      <c r="F125" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4368,14 +4434,14 @@
       </c>
       <c r="C126" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-BLACK-OEM-</t>
+          <t>SPHINX-OF-BLACK-CEM-</t>
         </is>
       </c>
       <c r="D126" s="15" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.967</v>
       </c>
       <c r="E126" s="15" t="n">
-        <v>0.748</v>
+        <v>0.584</v>
       </c>
       <c r="F126" s="16" t="inlineStr">
         <is>
@@ -4394,18 +4460,18 @@
       </c>
       <c r="C127" s="18" t="inlineStr">
         <is>
-          <t>JUDGE-MY-VOW-QUICKLY</t>
+          <t>JUDGE-MYUVOW-QUICKLY</t>
         </is>
       </c>
       <c r="D127" s="19" t="n">
-        <v>0.926</v>
+        <v>0.97</v>
       </c>
       <c r="E127" s="19" t="n">
-        <v>0.627</v>
-      </c>
-      <c r="F127" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.851</v>
+      </c>
+      <c r="F127" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4424,14 +4490,14 @@
         </is>
       </c>
       <c r="D128" s="15" t="n">
-        <v>0.972</v>
+        <v>0.985</v>
       </c>
       <c r="E128" s="15" t="n">
-        <v>0.712</v>
-      </c>
-      <c r="F128" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.853</v>
+      </c>
+      <c r="F128" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4516,7 @@
         </is>
       </c>
       <c r="D129" s="19" t="n">
-        <v>0.909</v>
+        <v>0.946</v>
       </c>
       <c r="E129" s="19" t="n">
         <v>0.6850000000000001</v>
@@ -4476,10 +4542,10 @@
         </is>
       </c>
       <c r="D130" s="15" t="n">
-        <v>0.956</v>
+        <v>0.954</v>
       </c>
       <c r="E130" s="15" t="n">
-        <v>0.747</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="F130" s="16" t="inlineStr">
         <is>
@@ -4498,14 +4564,14 @@
       </c>
       <c r="C131" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEEP-NEURAC-NETWORKO</t>
         </is>
       </c>
       <c r="D131" s="19" t="n">
-        <v>0.879</v>
+        <v>0.916</v>
       </c>
       <c r="E131" s="19" t="n">
-        <v>0.302</v>
+        <v>0.351</v>
       </c>
       <c r="F131" s="16" t="inlineStr">
         <is>
@@ -4528,10 +4594,10 @@
         </is>
       </c>
       <c r="D132" s="15" t="n">
-        <v>0.888</v>
+        <v>0.951</v>
       </c>
       <c r="E132" s="15" t="n">
-        <v>0.576</v>
+        <v>0.6850000000000001</v>
       </c>
       <c r="F132" s="16" t="inlineStr">
         <is>
@@ -4554,10 +4620,10 @@
         </is>
       </c>
       <c r="D133" s="19" t="n">
-        <v>0.895</v>
+        <v>0.968</v>
       </c>
       <c r="E133" s="19" t="n">
-        <v>0.622</v>
+        <v>0.799</v>
       </c>
       <c r="F133" s="16" t="inlineStr">
         <is>
@@ -4580,14 +4646,14 @@
         </is>
       </c>
       <c r="D134" s="15" t="n">
-        <v>0.944</v>
+        <v>0.979</v>
       </c>
       <c r="E134" s="15" t="n">
-        <v>0.679</v>
-      </c>
-      <c r="F134" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.866</v>
+      </c>
+      <c r="F134" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4606,14 +4672,14 @@
         </is>
       </c>
       <c r="D135" s="19" t="n">
-        <v>0.916</v>
+        <v>0.987</v>
       </c>
       <c r="E135" s="19" t="n">
-        <v>0.6899999999999999</v>
-      </c>
-      <c r="F135" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.921</v>
+      </c>
+      <c r="F135" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4632,14 +4698,14 @@
         </is>
       </c>
       <c r="D136" s="15" t="n">
-        <v>0.896</v>
+        <v>0.965</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>0.439</v>
-      </c>
-      <c r="F136" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.825</v>
+      </c>
+      <c r="F136" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4658,10 +4724,10 @@
         </is>
       </c>
       <c r="D137" s="19" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.959</v>
       </c>
       <c r="E137" s="19" t="n">
-        <v>0.708</v>
+        <v>0.705</v>
       </c>
       <c r="F137" s="16" t="inlineStr">
         <is>
@@ -4684,10 +4750,10 @@
         </is>
       </c>
       <c r="D138" s="15" t="n">
-        <v>0.931</v>
+        <v>0.969</v>
       </c>
       <c r="E138" s="15" t="n">
-        <v>0.421</v>
+        <v>0.699</v>
       </c>
       <c r="F138" s="16" t="inlineStr">
         <is>
@@ -4706,14 +4772,14 @@
       </c>
       <c r="C139" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FINE-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D139" s="19" t="n">
-        <v>0.898</v>
+        <v>0.953</v>
       </c>
       <c r="E139" s="19" t="n">
-        <v>0.39</v>
+        <v>0.659</v>
       </c>
       <c r="F139" s="16" t="inlineStr">
         <is>
@@ -4736,14 +4802,14 @@
         </is>
       </c>
       <c r="D140" s="15" t="n">
-        <v>0.925</v>
+        <v>0.98</v>
       </c>
       <c r="E140" s="15" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="F140" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.842</v>
+      </c>
+      <c r="F140" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4762,10 +4828,10 @@
         </is>
       </c>
       <c r="D141" s="19" t="n">
-        <v>0.922</v>
+        <v>0.953</v>
       </c>
       <c r="E141" s="19" t="n">
-        <v>0.707</v>
+        <v>0.739</v>
       </c>
       <c r="F141" s="16" t="inlineStr">
         <is>
@@ -4784,14 +4850,14 @@
       </c>
       <c r="C142" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOX-</t>
+          <t>IHE-QUICK-BRAWN-FOX-</t>
         </is>
       </c>
       <c r="D142" s="15" t="n">
         <v>0.846</v>
       </c>
       <c r="E142" s="15" t="n">
-        <v>0.34</v>
+        <v>0.307</v>
       </c>
       <c r="F142" s="16" t="inlineStr">
         <is>
@@ -4810,14 +4876,14 @@
       </c>
       <c r="C143" s="18" t="inlineStr">
         <is>
-          <t>JUMPS-OVER-IAZY-DOG-</t>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
         </is>
       </c>
       <c r="D143" s="19" t="n">
-        <v>0.885</v>
+        <v>0.928</v>
       </c>
       <c r="E143" s="19" t="n">
-        <v>0.466</v>
+        <v>0.531</v>
       </c>
       <c r="F143" s="16" t="inlineStr">
         <is>
@@ -4836,14 +4902,14 @@
       </c>
       <c r="C144" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-BOX-WITH-TEA</t>
+          <t>YACK-MY-BCX-WITH-TEA</t>
         </is>
       </c>
       <c r="D144" s="15" t="n">
-        <v>0.844</v>
+        <v>0.891</v>
       </c>
       <c r="E144" s="15" t="n">
-        <v>0.341</v>
+        <v>0.224</v>
       </c>
       <c r="F144" s="16" t="inlineStr">
         <is>
@@ -4866,10 +4932,10 @@
         </is>
       </c>
       <c r="D145" s="19" t="n">
-        <v>0.872</v>
+        <v>0.898</v>
       </c>
       <c r="E145" s="19" t="n">
-        <v>0.52</v>
+        <v>0.443</v>
       </c>
       <c r="F145" s="16" t="inlineStr">
         <is>
@@ -4888,14 +4954,14 @@
       </c>
       <c r="C146" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OR-BLAOK-GEM-</t>
+          <t>SPHINX-OR-BLACK-QEM-</t>
         </is>
       </c>
       <c r="D146" s="15" t="n">
-        <v>0.864</v>
+        <v>0.917</v>
       </c>
       <c r="E146" s="15" t="n">
-        <v>0.381</v>
+        <v>0.236</v>
       </c>
       <c r="F146" s="16" t="inlineStr">
         <is>
@@ -4918,14 +4984,14 @@
         </is>
       </c>
       <c r="D147" s="19" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.968</v>
       </c>
       <c r="E147" s="19" t="n">
-        <v>0.739</v>
-      </c>
-      <c r="F147" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.852</v>
+      </c>
+      <c r="F147" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -4944,10 +5010,10 @@
         </is>
       </c>
       <c r="D148" s="15" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.909</v>
       </c>
       <c r="E148" s="15" t="n">
-        <v>0.592</v>
+        <v>0.396</v>
       </c>
       <c r="F148" s="16" t="inlineStr">
         <is>
@@ -4970,10 +5036,10 @@
         </is>
       </c>
       <c r="D149" s="19" t="n">
-        <v>0.887</v>
+        <v>0.948</v>
       </c>
       <c r="E149" s="19" t="n">
-        <v>0.573</v>
+        <v>0.416</v>
       </c>
       <c r="F149" s="16" t="inlineStr">
         <is>
@@ -4992,14 +5058,14 @@
       </c>
       <c r="C150" s="14" t="inlineStr">
         <is>
-          <t>MAOHINE-LEARNING-AI-</t>
+          <t>MACHINE-LEARNING-AI-</t>
         </is>
       </c>
       <c r="D150" s="15" t="n">
         <v>0.9370000000000001</v>
       </c>
       <c r="E150" s="15" t="n">
-        <v>0.706</v>
+        <v>0.612</v>
       </c>
       <c r="F150" s="16" t="inlineStr">
         <is>
@@ -5018,14 +5084,14 @@
       </c>
       <c r="C151" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETMORKS</t>
+          <t>DEEP-NEURAI-NITMORKS</t>
         </is>
       </c>
       <c r="D151" s="19" t="n">
-        <v>0.882</v>
+        <v>0.894</v>
       </c>
       <c r="E151" s="19" t="n">
-        <v>0.509</v>
+        <v>0.516</v>
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
@@ -5044,14 +5110,14 @@
       </c>
       <c r="C152" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGF-DATA-DETECT-OK</t>
         </is>
       </c>
       <c r="D152" s="15" t="n">
-        <v>0.853</v>
+        <v>0.918</v>
       </c>
       <c r="E152" s="15" t="n">
-        <v>0.506</v>
+        <v>0.492</v>
       </c>
       <c r="F152" s="16" t="inlineStr">
         <is>
@@ -5070,14 +5136,14 @@
       </c>
       <c r="C153" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENDV-ROBOT-</t>
+          <t>PYTHON-OPENCV-ROBOT-</t>
         </is>
       </c>
       <c r="D153" s="19" t="n">
-        <v>0.898</v>
+        <v>0.946</v>
       </c>
       <c r="E153" s="19" t="n">
-        <v>0.642</v>
+        <v>0.726</v>
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
@@ -5100,14 +5166,14 @@
         </is>
       </c>
       <c r="D154" s="15" t="n">
-        <v>0.916</v>
+        <v>0.963</v>
       </c>
       <c r="E154" s="15" t="n">
-        <v>0.697</v>
-      </c>
-      <c r="F154" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.867</v>
+      </c>
+      <c r="F154" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -5122,14 +5188,14 @@
       </c>
       <c r="C155" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDIOTION-</t>
+          <t>ACCURATE-PREIICTJOD-</t>
         </is>
       </c>
       <c r="D155" s="19" t="n">
-        <v>0.86</v>
+        <v>0.882</v>
       </c>
       <c r="E155" s="19" t="n">
-        <v>0.333</v>
+        <v>0.243</v>
       </c>
       <c r="F155" s="16" t="inlineStr">
         <is>
@@ -5148,14 +5214,14 @@
       </c>
       <c r="C156" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSTEM-OK</t>
+          <t>ARTIFICIALESYSTEM-OK</t>
         </is>
       </c>
       <c r="D156" s="15" t="n">
-        <v>0.921</v>
+        <v>0.909</v>
       </c>
       <c r="E156" s="15" t="n">
-        <v>0.535</v>
+        <v>0.271</v>
       </c>
       <c r="F156" s="16" t="inlineStr">
         <is>
@@ -5178,10 +5244,10 @@
         </is>
       </c>
       <c r="D157" s="19" t="n">
-        <v>0.888</v>
+        <v>0.921</v>
       </c>
       <c r="E157" s="19" t="n">
-        <v>0.626</v>
+        <v>0.473</v>
       </c>
       <c r="F157" s="16" t="inlineStr">
         <is>
@@ -5200,14 +5266,14 @@
       </c>
       <c r="C158" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWER--</t>
+          <t>KNOWLEDGE-IS-POWBR--</t>
         </is>
       </c>
       <c r="D158" s="15" t="n">
-        <v>0.912</v>
+        <v>0.916</v>
       </c>
       <c r="E158" s="15" t="n">
-        <v>0.676</v>
+        <v>0.375</v>
       </c>
       <c r="F158" s="16" t="inlineStr">
         <is>
@@ -5226,14 +5292,14 @@
       </c>
       <c r="C159" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FIND-GOLD</t>
+          <t>FIND-EXTRA-FIND-AOID</t>
         </is>
       </c>
       <c r="D159" s="19" t="n">
-        <v>0.861</v>
+        <v>0.901</v>
       </c>
       <c r="E159" s="19" t="n">
-        <v>0.515</v>
+        <v>0.298</v>
       </c>
       <c r="F159" s="16" t="inlineStr">
         <is>
@@ -5256,10 +5322,10 @@
         </is>
       </c>
       <c r="D160" s="15" t="n">
-        <v>0.921</v>
+        <v>0.961</v>
       </c>
       <c r="E160" s="15" t="n">
-        <v>0.705</v>
+        <v>0.67</v>
       </c>
       <c r="F160" s="16" t="inlineStr">
         <is>
@@ -5278,14 +5344,14 @@
       </c>
       <c r="C161" s="18" t="inlineStr">
         <is>
-          <t>ABODEFGHIJKLMNOPQRST</t>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D161" s="19" t="n">
-        <v>0.871</v>
+        <v>0.88</v>
       </c>
       <c r="E161" s="19" t="n">
-        <v>0.588</v>
+        <v>0.471</v>
       </c>
       <c r="F161" s="16" t="inlineStr">
         <is>
@@ -5304,14 +5370,14 @@
       </c>
       <c r="C162" s="14" t="inlineStr">
         <is>
-          <t>IHE-QUICK-BROWN-FOX-</t>
+          <t>THE-QUICK-BROWN-FOX-</t>
         </is>
       </c>
       <c r="D162" s="15" t="n">
-        <v>0.907</v>
+        <v>0.963</v>
       </c>
       <c r="E162" s="15" t="n">
-        <v>0.586</v>
+        <v>0.787</v>
       </c>
       <c r="F162" s="16" t="inlineStr">
         <is>
@@ -5334,10 +5400,10 @@
         </is>
       </c>
       <c r="D163" s="19" t="n">
-        <v>0.897</v>
+        <v>0.955</v>
       </c>
       <c r="E163" s="19" t="n">
-        <v>0.538</v>
+        <v>0.548</v>
       </c>
       <c r="F163" s="16" t="inlineStr">
         <is>
@@ -5360,14 +5426,14 @@
         </is>
       </c>
       <c r="D164" s="15" t="n">
-        <v>0.92</v>
+        <v>0.961</v>
       </c>
       <c r="E164" s="15" t="n">
-        <v>0.658</v>
-      </c>
-      <c r="F164" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.83</v>
+      </c>
+      <c r="F164" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -5382,14 +5448,14 @@
       </c>
       <c r="C165" s="18" t="inlineStr">
         <is>
-          <t>FIVE-DOZEN-LIQUOR-JU</t>
+          <t>FJVE-DOZEN-LIQUOR-IU</t>
         </is>
       </c>
       <c r="D165" s="19" t="n">
-        <v>0.845</v>
+        <v>0.947</v>
       </c>
       <c r="E165" s="19" t="n">
-        <v>0.497</v>
+        <v>0.676</v>
       </c>
       <c r="F165" s="16" t="inlineStr">
         <is>
@@ -5408,14 +5474,14 @@
       </c>
       <c r="C166" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-RLACK-GEM-</t>
+          <t>SPHINX-OF-BLACK-GEM-</t>
         </is>
       </c>
       <c r="D166" s="15" t="n">
-        <v>0.903</v>
+        <v>0.926</v>
       </c>
       <c r="E166" s="15" t="n">
-        <v>0.413</v>
+        <v>0.276</v>
       </c>
       <c r="F166" s="16" t="inlineStr">
         <is>
@@ -5438,10 +5504,10 @@
         </is>
       </c>
       <c r="D167" s="19" t="n">
-        <v>0.889</v>
+        <v>0.931</v>
       </c>
       <c r="E167" s="19" t="n">
-        <v>0.681</v>
+        <v>0.55</v>
       </c>
       <c r="F167" s="16" t="inlineStr">
         <is>
@@ -5460,14 +5526,14 @@
       </c>
       <c r="C168" s="14" t="inlineStr">
         <is>
-          <t>BRZGHT-ZFPMYRS-RLOW-</t>
+          <t>BRZGHT-ZFPHYRS-BLOW-</t>
         </is>
       </c>
       <c r="D168" s="15" t="n">
-        <v>0.849</v>
+        <v>0.846</v>
       </c>
       <c r="E168" s="15" t="n">
-        <v>0.506</v>
+        <v>0.382</v>
       </c>
       <c r="F168" s="16" t="inlineStr">
         <is>
@@ -5486,14 +5552,14 @@
       </c>
       <c r="C169" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TEST</t>
+          <t>COMPVTER-VISION-TEST</t>
         </is>
       </c>
       <c r="D169" s="19" t="n">
-        <v>0.843</v>
+        <v>0.893</v>
       </c>
       <c r="E169" s="19" t="n">
-        <v>0.495</v>
+        <v>0.538</v>
       </c>
       <c r="F169" s="16" t="inlineStr">
         <is>
@@ -5516,10 +5582,10 @@
         </is>
       </c>
       <c r="D170" s="15" t="n">
-        <v>0.923</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E170" s="15" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.594</v>
       </c>
       <c r="F170" s="16" t="inlineStr">
         <is>
@@ -5538,14 +5604,14 @@
       </c>
       <c r="C171" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NQURAL-NETWORKS</t>
+          <t>DEER-NFURAL-NETWORKS</t>
         </is>
       </c>
       <c r="D171" s="19" t="n">
-        <v>0.847</v>
+        <v>0.926</v>
       </c>
       <c r="E171" s="19" t="n">
-        <v>0.278</v>
+        <v>0.238</v>
       </c>
       <c r="F171" s="16" t="inlineStr">
         <is>
@@ -5564,14 +5630,14 @@
       </c>
       <c r="C172" s="14" t="inlineStr">
         <is>
-          <t>IMAGE-DATA-DETECT-OK</t>
+          <t>IMAGE-DATA-DETECT-CK</t>
         </is>
       </c>
       <c r="D172" s="15" t="n">
-        <v>0.853</v>
+        <v>0.9</v>
       </c>
       <c r="E172" s="15" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.447</v>
       </c>
       <c r="F172" s="16" t="inlineStr">
         <is>
@@ -5590,14 +5656,14 @@
       </c>
       <c r="C173" s="18" t="inlineStr">
         <is>
-          <t>PYTHON-OPENCV-ROROT-</t>
+          <t>PYTHON-OPENCV-ROOOT-</t>
         </is>
       </c>
       <c r="D173" s="19" t="n">
-        <v>0.887</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E173" s="19" t="n">
-        <v>0.597</v>
+        <v>0.413</v>
       </c>
       <c r="F173" s="16" t="inlineStr">
         <is>
@@ -5620,10 +5686,10 @@
         </is>
       </c>
       <c r="D174" s="15" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.927</v>
       </c>
       <c r="E174" s="15" t="n">
-        <v>0.415</v>
+        <v>0.397</v>
       </c>
       <c r="F174" s="16" t="inlineStr">
         <is>
@@ -5642,14 +5708,14 @@
       </c>
       <c r="C175" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTION-</t>
+          <t>ACCURATE-PRFDICTION-</t>
         </is>
       </c>
       <c r="D175" s="19" t="n">
-        <v>0.881</v>
+        <v>0.906</v>
       </c>
       <c r="E175" s="19" t="n">
-        <v>0.601</v>
+        <v>0.506</v>
       </c>
       <c r="F175" s="16" t="inlineStr">
         <is>
@@ -5672,14 +5738,14 @@
         </is>
       </c>
       <c r="D176" s="15" t="n">
-        <v>0.835</v>
+        <v>0.948</v>
       </c>
       <c r="E176" s="15" t="n">
-        <v>0.516</v>
-      </c>
-      <c r="F176" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.822</v>
+      </c>
+      <c r="F176" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -5694,14 +5760,14 @@
       </c>
       <c r="C177" s="18" t="inlineStr">
         <is>
-          <t>HELLO-WORLD-WELCOME-</t>
+          <t>HEWLO-WORLD-WELCOME-</t>
         </is>
       </c>
       <c r="D177" s="19" t="n">
-        <v>0.863</v>
+        <v>0.915</v>
       </c>
       <c r="E177" s="19" t="n">
-        <v>0.386</v>
+        <v>0.223</v>
       </c>
       <c r="F177" s="16" t="inlineStr">
         <is>
@@ -5724,10 +5790,10 @@
         </is>
       </c>
       <c r="D178" s="15" t="n">
-        <v>0.909</v>
+        <v>0.912</v>
       </c>
       <c r="E178" s="15" t="n">
-        <v>0.412</v>
+        <v>0.539</v>
       </c>
       <c r="F178" s="16" t="inlineStr">
         <is>
@@ -5746,14 +5812,14 @@
       </c>
       <c r="C179" s="18" t="inlineStr">
         <is>
-          <t>EIND-EXTRA-FIND-GOLD</t>
+          <t>HIND-EXTRA-FIND-GGLD</t>
         </is>
       </c>
       <c r="D179" s="19" t="n">
-        <v>0.855</v>
+        <v>0.868</v>
       </c>
       <c r="E179" s="19" t="n">
-        <v>0.405</v>
+        <v>0.38</v>
       </c>
       <c r="F179" s="16" t="inlineStr">
         <is>
@@ -5772,14 +5838,14 @@
       </c>
       <c r="C180" s="14" t="inlineStr">
         <is>
-          <t>ZERG-ONE-TWO-SIX-TEN</t>
+          <t>ZERGHONE-TWO-SIX-TEN</t>
         </is>
       </c>
       <c r="D180" s="15" t="n">
-        <v>0.852</v>
+        <v>0.839</v>
       </c>
       <c r="E180" s="15" t="n">
-        <v>0.475</v>
+        <v>0.145</v>
       </c>
       <c r="F180" s="16" t="inlineStr">
         <is>
@@ -5798,14 +5864,14 @@
       </c>
       <c r="C181" s="18" t="inlineStr">
         <is>
-          <t>ABCDEEGVIJKLMNOPQRST</t>
+          <t>ABCDEEGHIJKLMNOPQRST</t>
         </is>
       </c>
       <c r="D181" s="19" t="n">
-        <v>0.858</v>
+        <v>0.929</v>
       </c>
       <c r="E181" s="19" t="n">
-        <v>0.477</v>
+        <v>0.52</v>
       </c>
       <c r="F181" s="16" t="inlineStr">
         <is>
@@ -5824,14 +5890,14 @@
       </c>
       <c r="C182" s="14" t="inlineStr">
         <is>
-          <t>THE-QUICK-BROWN-FOX-</t>
+          <t>THE-QUICK-BROWN-FQX-</t>
         </is>
       </c>
       <c r="D182" s="15" t="n">
-        <v>0.903</v>
+        <v>0.919</v>
       </c>
       <c r="E182" s="15" t="n">
-        <v>0.543</v>
+        <v>0.547</v>
       </c>
       <c r="F182" s="16" t="inlineStr">
         <is>
@@ -5854,10 +5920,10 @@
         </is>
       </c>
       <c r="D183" s="19" t="n">
-        <v>0.895</v>
+        <v>0.881</v>
       </c>
       <c r="E183" s="19" t="n">
-        <v>0.605</v>
+        <v>0.509</v>
       </c>
       <c r="F183" s="16" t="inlineStr">
         <is>
@@ -5876,14 +5942,14 @@
       </c>
       <c r="C184" s="14" t="inlineStr">
         <is>
-          <t>PACK-MY-ROX-WITF-TEA</t>
+          <t>PACK-MY-BOX-WITE-TEA</t>
         </is>
       </c>
       <c r="D184" s="15" t="n">
-        <v>0.885</v>
+        <v>0.901</v>
       </c>
       <c r="E184" s="15" t="n">
-        <v>0.505</v>
+        <v>0.439</v>
       </c>
       <c r="F184" s="16" t="inlineStr">
         <is>
@@ -5902,14 +5968,14 @@
       </c>
       <c r="C185" s="18" t="inlineStr">
         <is>
-          <t>FIVEZDOZEN-IIQUOR-JU</t>
+          <t>FIVEADOZEN-IIQUOR-JU</t>
         </is>
       </c>
       <c r="D185" s="19" t="n">
-        <v>0.882</v>
+        <v>0.898</v>
       </c>
       <c r="E185" s="19" t="n">
-        <v>0.353</v>
+        <v>0.333</v>
       </c>
       <c r="F185" s="16" t="inlineStr">
         <is>
@@ -5928,14 +5994,14 @@
       </c>
       <c r="C186" s="14" t="inlineStr">
         <is>
-          <t>SPHINX-OF-RLAOK-GFM-</t>
+          <t>SPHLNX-OF-RLACK-GFM-</t>
         </is>
       </c>
       <c r="D186" s="15" t="n">
-        <v>0.88</v>
+        <v>0.915</v>
       </c>
       <c r="E186" s="15" t="n">
-        <v>0.537</v>
+        <v>0.459</v>
       </c>
       <c r="F186" s="16" t="inlineStr">
         <is>
@@ -5958,10 +6024,10 @@
         </is>
       </c>
       <c r="D187" s="19" t="n">
-        <v>0.891</v>
+        <v>0.944</v>
       </c>
       <c r="E187" s="19" t="n">
-        <v>0.485</v>
+        <v>0.368</v>
       </c>
       <c r="F187" s="16" t="inlineStr">
         <is>
@@ -5980,14 +6046,14 @@
       </c>
       <c r="C188" s="14" t="inlineStr">
         <is>
-          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+          <t>BXIGHT-ZEPHYRS-BLCW-</t>
         </is>
       </c>
       <c r="D188" s="15" t="n">
-        <v>0.869</v>
+        <v>0.852</v>
       </c>
       <c r="E188" s="15" t="n">
-        <v>0.518</v>
+        <v>0.379</v>
       </c>
       <c r="F188" s="16" t="inlineStr">
         <is>
@@ -6006,14 +6072,14 @@
       </c>
       <c r="C189" s="18" t="inlineStr">
         <is>
-          <t>COMPUTER-VISION-TEST</t>
+          <t>CQMPUTER-VISIQN-TEST</t>
         </is>
       </c>
       <c r="D189" s="19" t="n">
-        <v>0.821</v>
+        <v>0.839</v>
       </c>
       <c r="E189" s="19" t="n">
-        <v>0.485</v>
+        <v>0.494</v>
       </c>
       <c r="F189" s="16" t="inlineStr">
         <is>
@@ -6032,14 +6098,14 @@
       </c>
       <c r="C190" s="14" t="inlineStr">
         <is>
-          <t>MACHINE-LFARNING-AI-</t>
+          <t>MACHINE-LFARNLNG-AL-</t>
         </is>
       </c>
       <c r="D190" s="15" t="n">
-        <v>0.844</v>
+        <v>0.836</v>
       </c>
       <c r="E190" s="15" t="n">
-        <v>0.456</v>
+        <v>0.379</v>
       </c>
       <c r="F190" s="16" t="inlineStr">
         <is>
@@ -6058,14 +6124,14 @@
       </c>
       <c r="C191" s="18" t="inlineStr">
         <is>
-          <t>DEEP-NEURAL-NETWORKS</t>
+          <t>DEEP-NEURAL-NETWQRKS</t>
         </is>
       </c>
       <c r="D191" s="19" t="n">
-        <v>0.887</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="E191" s="19" t="n">
-        <v>0.54</v>
+        <v>0.597</v>
       </c>
       <c r="F191" s="16" t="inlineStr">
         <is>
@@ -6088,10 +6154,10 @@
         </is>
       </c>
       <c r="D192" s="15" t="n">
-        <v>0.832</v>
+        <v>0.916</v>
       </c>
       <c r="E192" s="15" t="n">
-        <v>0.322</v>
+        <v>0.35</v>
       </c>
       <c r="F192" s="16" t="inlineStr">
         <is>
@@ -6110,14 +6176,14 @@
       </c>
       <c r="C193" s="18" t="inlineStr">
         <is>
-          <t>PYIHON-OPENCV-ROBOT-</t>
+          <t>PYTHON-OPENCV-DOBOT-</t>
         </is>
       </c>
       <c r="D193" s="19" t="n">
-        <v>0.852</v>
+        <v>0.878</v>
       </c>
       <c r="E193" s="19" t="n">
-        <v>0.483</v>
+        <v>0.371</v>
       </c>
       <c r="F193" s="16" t="inlineStr">
         <is>
@@ -6136,14 +6202,14 @@
       </c>
       <c r="C194" s="14" t="inlineStr">
         <is>
-          <t>SMART-OCR-RECOGNIZE-</t>
+          <t>SMART-OCR-RRCOGNIZF-</t>
         </is>
       </c>
       <c r="D194" s="15" t="n">
-        <v>0.837</v>
+        <v>0.884</v>
       </c>
       <c r="E194" s="15" t="n">
-        <v>0.315</v>
+        <v>0.362</v>
       </c>
       <c r="F194" s="16" t="inlineStr">
         <is>
@@ -6162,14 +6228,14 @@
       </c>
       <c r="C195" s="18" t="inlineStr">
         <is>
-          <t>ACCURATE-PREDICTION-</t>
+          <t>ACCURATE-PREDHCTION-</t>
         </is>
       </c>
       <c r="D195" s="19" t="n">
-        <v>0.827</v>
+        <v>0.872</v>
       </c>
       <c r="E195" s="19" t="n">
-        <v>0.405</v>
+        <v>0.179</v>
       </c>
       <c r="F195" s="16" t="inlineStr">
         <is>
@@ -6188,14 +6254,14 @@
       </c>
       <c r="C196" s="14" t="inlineStr">
         <is>
-          <t>ARTIFICIAL-SYSIIMTIO</t>
+          <t>ARTIFICIAL-EEEDLCTIO</t>
         </is>
       </c>
       <c r="D196" s="15" t="n">
-        <v>0.729</v>
+        <v>0.781</v>
       </c>
       <c r="E196" s="15" t="n">
-        <v>0.452</v>
+        <v>0.304</v>
       </c>
       <c r="F196" s="16" t="inlineStr">
         <is>
@@ -6218,10 +6284,10 @@
         </is>
       </c>
       <c r="D197" s="19" t="n">
-        <v>0.88</v>
+        <v>0.931</v>
       </c>
       <c r="E197" s="19" t="n">
-        <v>0.503</v>
+        <v>0.669</v>
       </c>
       <c r="F197" s="16" t="inlineStr">
         <is>
@@ -6240,14 +6306,14 @@
       </c>
       <c r="C198" s="14" t="inlineStr">
         <is>
-          <t>KNOWLEDGE-IS-POWFR--</t>
+          <t>KNOWLEPGE-LS-POWFR--</t>
         </is>
       </c>
       <c r="D198" s="15" t="n">
-        <v>0.9</v>
+        <v>0.882</v>
       </c>
       <c r="E198" s="15" t="n">
-        <v>0.541</v>
+        <v>0.4</v>
       </c>
       <c r="F198" s="16" t="inlineStr">
         <is>
@@ -6266,14 +6332,14 @@
       </c>
       <c r="C199" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FINE-GOID</t>
+          <t>FLND-EXTRA-FLNK-GOID</t>
         </is>
       </c>
       <c r="D199" s="19" t="n">
-        <v>0.827</v>
+        <v>0.841</v>
       </c>
       <c r="E199" s="19" t="n">
-        <v>0.362</v>
+        <v>0.441</v>
       </c>
       <c r="F199" s="16" t="inlineStr">
         <is>
@@ -6292,14 +6358,14 @@
       </c>
       <c r="C200" s="14" t="inlineStr">
         <is>
-          <t>ZERO-ONE-TWO-CIX-TEN</t>
+          <t>ZEBO-ONE-TWU-CLX-TEN</t>
         </is>
       </c>
       <c r="D200" s="15" t="n">
-        <v>0.839</v>
+        <v>0.862</v>
       </c>
       <c r="E200" s="15" t="n">
-        <v>0.489</v>
+        <v>0.456</v>
       </c>
       <c r="F200" s="16" t="inlineStr">
         <is>
@@ -6318,14 +6384,14 @@
       </c>
       <c r="C201" s="18" t="inlineStr">
         <is>
-          <t>ABCDEFGHIJKLMNOPGPST</t>
+          <t>ABCDEFGHIGKLMNCEGPST</t>
         </is>
       </c>
       <c r="D201" s="19" t="n">
-        <v>0.823</v>
+        <v>0.917</v>
       </c>
       <c r="E201" s="19" t="n">
-        <v>0.342</v>
+        <v>0.367</v>
       </c>
       <c r="F201" s="16" t="inlineStr">
         <is>
@@ -6333,8 +6399,1048 @@
         </is>
       </c>
     </row>
+    <row r="202" ht="20" customHeight="1">
+      <c r="A202" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B202" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C202" s="14" t="inlineStr">
+        <is>
+          <t>IHE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D202" s="15" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="E202" s="15" t="n">
+        <v>0.256</v>
+      </c>
+      <c r="F202" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="20" customHeight="1">
+      <c r="A203" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B203" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C203" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D203" s="19" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E203" s="19" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="F203" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="20" customHeight="1">
+      <c r="A204" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B204" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C204" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D204" s="15" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="E204" s="15" t="n">
+        <v>0.664</v>
+      </c>
+      <c r="F204" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="20" customHeight="1">
+      <c r="A205" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B205" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C205" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LTQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D205" s="19" t="n">
+        <v>0.951</v>
+      </c>
+      <c r="E205" s="19" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="F205" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="20" customHeight="1">
+      <c r="A206" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B206" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C206" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-BLACK-GEM-</t>
+        </is>
+      </c>
+      <c r="D206" s="15" t="n">
+        <v>0.968</v>
+      </c>
+      <c r="E206" s="15" t="n">
+        <v>0.6830000000000001</v>
+      </c>
+      <c r="F206" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="20" customHeight="1">
+      <c r="A207" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B207" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C207" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D207" s="19" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="E207" s="19" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="F207" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="20" customHeight="1">
+      <c r="A208" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B208" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C208" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BIOW-</t>
+        </is>
+      </c>
+      <c r="D208" s="15" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="E208" s="15" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="F208" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="20" customHeight="1">
+      <c r="A209" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B209" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C209" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D209" s="19" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="E209" s="19" t="n">
+        <v>0.652</v>
+      </c>
+      <c r="F209" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="20" customHeight="1">
+      <c r="A210" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B210" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C210" s="14" t="inlineStr">
+        <is>
+          <t>MACHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D210" s="15" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="E210" s="15" t="n">
+        <v>0.904</v>
+      </c>
+      <c r="F210" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="20" customHeight="1">
+      <c r="A211" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B211" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C211" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NFTKORKS</t>
+        </is>
+      </c>
+      <c r="D211" s="19" t="n">
+        <v>0.931</v>
+      </c>
+      <c r="E211" s="19" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="F211" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="20" customHeight="1">
+      <c r="A212" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B212" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C212" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-DETECT-OK</t>
+        </is>
+      </c>
+      <c r="D212" s="15" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="E212" s="15" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="F212" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="20" customHeight="1">
+      <c r="A213" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B213" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C213" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D213" s="19" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="E213" s="19" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F213" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="20" customHeight="1">
+      <c r="A214" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B214" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C214" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D214" s="15" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="E214" s="15" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="F214" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="20" customHeight="1">
+      <c r="A215" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B215" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C215" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTIOD-</t>
+        </is>
+      </c>
+      <c r="D215" s="19" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="E215" s="19" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="F215" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="20" customHeight="1">
+      <c r="A216" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B216" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C216" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D216" s="15" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="E216" s="15" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="F216" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="20" customHeight="1">
+      <c r="A217" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B217" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C217" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D217" s="19" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="E217" s="19" t="n">
+        <v>0.6919999999999999</v>
+      </c>
+      <c r="F217" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="20" customHeight="1">
+      <c r="A218" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B218" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C218" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POKER--</t>
+        </is>
+      </c>
+      <c r="D218" s="15" t="n">
+        <v>0.985</v>
+      </c>
+      <c r="E218" s="15" t="n">
+        <v>0.895</v>
+      </c>
+      <c r="F218" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="20" customHeight="1">
+      <c r="A219" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B219" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C219" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FIND-GOLD</t>
+        </is>
+      </c>
+      <c r="D219" s="19" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="E219" s="19" t="n">
+        <v>0.412</v>
+      </c>
+      <c r="F219" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="20" customHeight="1">
+      <c r="A220" s="13" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B220" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C220" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D220" s="15" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="E220" s="15" t="n">
+        <v>0.678</v>
+      </c>
+      <c r="F220" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="20" customHeight="1">
+      <c r="A221" s="17" t="inlineStr">
+        <is>
+          <t>test11.jpg</t>
+        </is>
+      </c>
+      <c r="B221" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C221" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNQPQRST</t>
+        </is>
+      </c>
+      <c r="D221" s="19" t="n">
+        <v>0.952</v>
+      </c>
+      <c r="E221" s="19" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="F221" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="20" customHeight="1">
+      <c r="A222" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B222" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D222" s="15" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="E222" s="15" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="F222" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="20" customHeight="1">
+      <c r="A223" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B223" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C223" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D223" s="19" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="E223" s="19" t="n">
+        <v>0.629</v>
+      </c>
+      <c r="F223" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="20" customHeight="1">
+      <c r="A224" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B224" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C224" s="14" t="inlineStr">
+        <is>
+          <t>PACK-MY-BOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D224" s="15" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="E224" s="15" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="F224" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="20" customHeight="1">
+      <c r="A225" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B225" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C225" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D225" s="19" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="E225" s="19" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="F225" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="20" customHeight="1">
+      <c r="A226" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B226" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C226" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-BLACK-GEM-</t>
+        </is>
+      </c>
+      <c r="D226" s="15" t="n">
+        <v>0.982</v>
+      </c>
+      <c r="E226" s="15" t="n">
+        <v>0.892</v>
+      </c>
+      <c r="F226" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="20" customHeight="1">
+      <c r="A227" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B227" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C227" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D227" s="19" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E227" s="19" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F227" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="20" customHeight="1">
+      <c r="A228" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B228" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C228" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D228" s="15" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="E228" s="15" t="n">
+        <v>0.857</v>
+      </c>
+      <c r="F228" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="20" customHeight="1">
+      <c r="A229" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B229" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C229" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D229" s="19" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="E229" s="19" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="F229" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="20" customHeight="1">
+      <c r="A230" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B230" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C230" s="14" t="inlineStr">
+        <is>
+          <t>MECHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D230" s="15" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="E230" s="15" t="n">
+        <v>0.916</v>
+      </c>
+      <c r="F230" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="20" customHeight="1">
+      <c r="A231" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B231" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C231" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKS</t>
+        </is>
+      </c>
+      <c r="D231" s="19" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E231" s="19" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="F231" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="20" customHeight="1">
+      <c r="A232" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B232" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C232" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-DATA-OETECT-OK</t>
+        </is>
+      </c>
+      <c r="D232" s="15" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="E232" s="15" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F232" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="20" customHeight="1">
+      <c r="A233" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B233" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C233" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D233" s="19" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="E233" s="19" t="n">
+        <v>0.607</v>
+      </c>
+      <c r="F233" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="20" customHeight="1">
+      <c r="A234" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B234" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C234" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D234" s="15" t="n">
+        <v>0.957</v>
+      </c>
+      <c r="E234" s="15" t="n">
+        <v>0.779</v>
+      </c>
+      <c r="F234" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="20" customHeight="1">
+      <c r="A235" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B235" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C235" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTION-</t>
+        </is>
+      </c>
+      <c r="D235" s="19" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="E235" s="19" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="F235" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="20" customHeight="1">
+      <c r="A236" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B236" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C236" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D236" s="15" t="n">
+        <v>0.967</v>
+      </c>
+      <c r="E236" s="15" t="n">
+        <v>0.8070000000000001</v>
+      </c>
+      <c r="F236" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="20" customHeight="1">
+      <c r="A237" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B237" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C237" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D237" s="19" t="n">
+        <v>0.979</v>
+      </c>
+      <c r="E237" s="19" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="F237" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="20" customHeight="1">
+      <c r="A238" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B238" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C238" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POWER--</t>
+        </is>
+      </c>
+      <c r="D238" s="15" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="E238" s="15" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="F238" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="20" customHeight="1">
+      <c r="A239" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B239" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C239" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FINO-GOLD</t>
+        </is>
+      </c>
+      <c r="D239" s="19" t="n">
+        <v>0.954</v>
+      </c>
+      <c r="E239" s="19" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="F239" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="20" customHeight="1">
+      <c r="A240" s="13" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B240" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C240" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D240" s="15" t="n">
+        <v>0.975</v>
+      </c>
+      <c r="E240" s="15" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="F240" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="20" customHeight="1">
+      <c r="A241" s="17" t="inlineStr">
+        <is>
+          <t>test12.jpg</t>
+        </is>
+      </c>
+      <c r="B241" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C241" s="18" t="inlineStr">
+        <is>
+          <t>ABCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D241" s="19" t="n">
+        <v>0.965</v>
+      </c>
+      <c r="E241" s="19" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="F241" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F201"/>
+  <autoFilter ref="A1:F241"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 2D piecewise mesh warp for curved handheld sheets (test12, test13) and update 13-sheet benchmark (95.35%)
</commit_message>
<xml_diff>
--- a/outputs/results/all_results.xlsx
+++ b/outputs/results/all_results.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed_Results" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detailed_Results'!$A$1:$F$261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -618,7 +618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="113" customWidth="1" min="1" max="1"/>
@@ -641,7 +641,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>สร้างรายงานเมื่อ: 2026-10-26 14:44:14 | โมเดลที่ใช้ตรวจ: Super-Ensemble | ตรวจทั้งหมด: 12 แผ่น | รวม 240 ข้อ</t>
+          <t>สร้างรายงานเมื่อ: 2026-10-28 16:36:32 | โมเดลที่ใช้ตรวจ: Super-Ensemble | ตรวจทั้งหมด: 13 แผ่น | รวม 260 ข้อ</t>
         </is>
       </c>
     </row>
@@ -676,27 +676,27 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>12 แผ่น</t>
+          <t>13 แผ่น</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>240 ข้อ</t>
+          <t>260 ข้อ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>4,800 ตัว</t>
+          <t>5,200 ตัว</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>95.12%</t>
+          <t>95.35%</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>176 ข้อ</t>
+          <t>192 ข้อ</t>
         </is>
       </c>
     </row>
@@ -1128,15 +1128,48 @@
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>0.968</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>7 ข้อ</t>
+          <t>8 ข้อ</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>English &amp; Tech (ชุดที่ 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="C23" s="9" t="n">
+        <v>400</v>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>98.00%</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>15 ข้อ</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
         <is>
           <t>English &amp; Tech (ชุดที่ 1)</t>
         </is>
@@ -1156,7 +1189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F241"/>
+  <dimension ref="A1:F261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -2335,7 +2368,7 @@
         <v>0.96</v>
       </c>
       <c r="E45" s="19" t="n">
-        <v>0.824</v>
+        <v>0.825</v>
       </c>
       <c r="F45" s="20" t="inlineStr">
         <is>
@@ -2413,7 +2446,7 @@
         <v>0.948</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.708</v>
+        <v>0.707</v>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
@@ -3063,7 +3096,7 @@
         <v>0.977</v>
       </c>
       <c r="E73" s="19" t="n">
-        <v>0.834</v>
+        <v>0.833</v>
       </c>
       <c r="F73" s="20" t="inlineStr">
         <is>
@@ -3323,7 +3356,7 @@
         <v>0.969</v>
       </c>
       <c r="E83" s="19" t="n">
-        <v>0.583</v>
+        <v>0.582</v>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
@@ -4181,7 +4214,7 @@
         <v>0.915</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.504</v>
+        <v>0.505</v>
       </c>
       <c r="F116" s="16" t="inlineStr">
         <is>
@@ -4701,7 +4734,7 @@
         <v>0.965</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>0.825</v>
+        <v>0.824</v>
       </c>
       <c r="F136" s="20" t="inlineStr">
         <is>
@@ -4831,7 +4864,7 @@
         <v>0.953</v>
       </c>
       <c r="E141" s="19" t="n">
-        <v>0.739</v>
+        <v>0.738</v>
       </c>
       <c r="F141" s="16" t="inlineStr">
         <is>
@@ -6495,7 +6528,7 @@
         <v>0.951</v>
       </c>
       <c r="E205" s="19" t="n">
-        <v>0.617</v>
+        <v>0.618</v>
       </c>
       <c r="F205" s="16" t="inlineStr">
         <is>
@@ -6934,14 +6967,14 @@
         </is>
       </c>
       <c r="D222" s="15" t="n">
-        <v>0.977</v>
+        <v>0.973</v>
       </c>
       <c r="E222" s="15" t="n">
-        <v>0.8070000000000001</v>
-      </c>
-      <c r="F222" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.778</v>
+      </c>
+      <c r="F222" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -6960,14 +6993,14 @@
         </is>
       </c>
       <c r="D223" s="19" t="n">
-        <v>0.957</v>
+        <v>0.978</v>
       </c>
       <c r="E223" s="19" t="n">
-        <v>0.629</v>
-      </c>
-      <c r="F223" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.911</v>
+      </c>
+      <c r="F223" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -6986,14 +7019,14 @@
         </is>
       </c>
       <c r="D224" s="15" t="n">
-        <v>0.949</v>
+        <v>0.971</v>
       </c>
       <c r="E224" s="15" t="n">
-        <v>0.712</v>
-      </c>
-      <c r="F224" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.835</v>
+      </c>
+      <c r="F224" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -7012,10 +7045,10 @@
         </is>
       </c>
       <c r="D225" s="19" t="n">
-        <v>0.965</v>
+        <v>0.974</v>
       </c>
       <c r="E225" s="19" t="n">
-        <v>0.892</v>
+        <v>0.9</v>
       </c>
       <c r="F225" s="20" t="inlineStr">
         <is>
@@ -7038,10 +7071,10 @@
         </is>
       </c>
       <c r="D226" s="15" t="n">
-        <v>0.982</v>
+        <v>0.986</v>
       </c>
       <c r="E226" s="15" t="n">
-        <v>0.892</v>
+        <v>0.914</v>
       </c>
       <c r="F226" s="20" t="inlineStr">
         <is>
@@ -7064,10 +7097,10 @@
         </is>
       </c>
       <c r="D227" s="19" t="n">
-        <v>0.98</v>
+        <v>0.983</v>
       </c>
       <c r="E227" s="19" t="n">
-        <v>0.92</v>
+        <v>0.944</v>
       </c>
       <c r="F227" s="20" t="inlineStr">
         <is>
@@ -7090,10 +7123,10 @@
         </is>
       </c>
       <c r="D228" s="15" t="n">
-        <v>0.976</v>
+        <v>0.986</v>
       </c>
       <c r="E228" s="15" t="n">
-        <v>0.857</v>
+        <v>0.916</v>
       </c>
       <c r="F228" s="20" t="inlineStr">
         <is>
@@ -7116,10 +7149,10 @@
         </is>
       </c>
       <c r="D229" s="19" t="n">
-        <v>0.962</v>
+        <v>0.953</v>
       </c>
       <c r="E229" s="19" t="n">
-        <v>0.784</v>
+        <v>0.753</v>
       </c>
       <c r="F229" s="16" t="inlineStr">
         <is>
@@ -7142,10 +7175,10 @@
         </is>
       </c>
       <c r="D230" s="15" t="n">
-        <v>0.979</v>
+        <v>0.962</v>
       </c>
       <c r="E230" s="15" t="n">
-        <v>0.916</v>
+        <v>0.841</v>
       </c>
       <c r="F230" s="20" t="inlineStr">
         <is>
@@ -7168,14 +7201,14 @@
         </is>
       </c>
       <c r="D231" s="19" t="n">
-        <v>0.97</v>
+        <v>0.974</v>
       </c>
       <c r="E231" s="19" t="n">
-        <v>0.782</v>
-      </c>
-      <c r="F231" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.899</v>
+      </c>
+      <c r="F231" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -7194,10 +7227,10 @@
         </is>
       </c>
       <c r="D232" s="15" t="n">
-        <v>0.905</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="E232" s="15" t="n">
-        <v>0.51</v>
+        <v>0.614</v>
       </c>
       <c r="F232" s="16" t="inlineStr">
         <is>
@@ -7220,10 +7253,10 @@
         </is>
       </c>
       <c r="D233" s="19" t="n">
-        <v>0.949</v>
+        <v>0.963</v>
       </c>
       <c r="E233" s="19" t="n">
-        <v>0.607</v>
+        <v>0.727</v>
       </c>
       <c r="F233" s="16" t="inlineStr">
         <is>
@@ -7246,14 +7279,14 @@
         </is>
       </c>
       <c r="D234" s="15" t="n">
-        <v>0.957</v>
+        <v>0.966</v>
       </c>
       <c r="E234" s="15" t="n">
-        <v>0.779</v>
-      </c>
-      <c r="F234" s="16" t="inlineStr">
-        <is>
-          <t>YES</t>
+        <v>0.82</v>
+      </c>
+      <c r="F234" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
     </row>
@@ -7272,14 +7305,14 @@
         </is>
       </c>
       <c r="D235" s="19" t="n">
-        <v>0.959</v>
+        <v>0.954</v>
       </c>
       <c r="E235" s="19" t="n">
-        <v>0.876</v>
-      </c>
-      <c r="F235" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.668</v>
+      </c>
+      <c r="F235" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -7301,11 +7334,11 @@
         <v>0.967</v>
       </c>
       <c r="E236" s="15" t="n">
-        <v>0.8070000000000001</v>
-      </c>
-      <c r="F236" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.795</v>
+      </c>
+      <c r="F236" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -7327,7 +7360,7 @@
         <v>0.979</v>
       </c>
       <c r="E237" s="19" t="n">
-        <v>0.928</v>
+        <v>0.88</v>
       </c>
       <c r="F237" s="20" t="inlineStr">
         <is>
@@ -7350,10 +7383,10 @@
         </is>
       </c>
       <c r="D238" s="15" t="n">
-        <v>0.977</v>
+        <v>0.983</v>
       </c>
       <c r="E238" s="15" t="n">
-        <v>0.906</v>
+        <v>0.916</v>
       </c>
       <c r="F238" s="20" t="inlineStr">
         <is>
@@ -7372,18 +7405,18 @@
       </c>
       <c r="C239" s="18" t="inlineStr">
         <is>
-          <t>FIND-EXTRA-FINO-GOLD</t>
+          <t>FIND-EXTRA-FIND-GOLD</t>
         </is>
       </c>
       <c r="D239" s="19" t="n">
-        <v>0.954</v>
+        <v>0.9409999999999999</v>
       </c>
       <c r="E239" s="19" t="n">
-        <v>0.826</v>
-      </c>
-      <c r="F239" s="20" t="inlineStr">
-        <is>
-          <t>NO</t>
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="F239" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
         </is>
       </c>
     </row>
@@ -7402,10 +7435,10 @@
         </is>
       </c>
       <c r="D240" s="15" t="n">
-        <v>0.975</v>
+        <v>0.979</v>
       </c>
       <c r="E240" s="15" t="n">
-        <v>0.872</v>
+        <v>0.895</v>
       </c>
       <c r="F240" s="20" t="inlineStr">
         <is>
@@ -7428,19 +7461,539 @@
         </is>
       </c>
       <c r="D241" s="19" t="n">
-        <v>0.965</v>
+        <v>0.955</v>
       </c>
       <c r="E241" s="19" t="n">
-        <v>0.871</v>
-      </c>
-      <c r="F241" s="20" t="inlineStr">
+        <v>0.543</v>
+      </c>
+      <c r="F241" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="20" customHeight="1">
+      <c r="A242" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B242" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C242" s="14" t="inlineStr">
+        <is>
+          <t>THE-QUICK-BROWN-FOX-</t>
+        </is>
+      </c>
+      <c r="D242" s="15" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="E242" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F242" s="20" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
+    <row r="243" ht="20" customHeight="1">
+      <c r="A243" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B243" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C243" s="18" t="inlineStr">
+        <is>
+          <t>JUMPS-OVER-LAZY-DOG-</t>
+        </is>
+      </c>
+      <c r="D243" s="19" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="E243" s="19" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="F243" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="20" customHeight="1">
+      <c r="A244" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B244" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C244" s="14" t="inlineStr">
+        <is>
+          <t>PACU-MY-BOX-WITH-TEA</t>
+        </is>
+      </c>
+      <c r="D244" s="15" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="E244" s="15" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="F244" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="20" customHeight="1">
+      <c r="A245" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B245" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C245" s="18" t="inlineStr">
+        <is>
+          <t>FIVE-DOZEN-LIQUOR-JU</t>
+        </is>
+      </c>
+      <c r="D245" s="19" t="n">
+        <v>0.9379999999999999</v>
+      </c>
+      <c r="E245" s="19" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="F245" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="20" customHeight="1">
+      <c r="A246" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B246" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C246" s="14" t="inlineStr">
+        <is>
+          <t>SPHINX-OF-BLACK-GEM-</t>
+        </is>
+      </c>
+      <c r="D246" s="15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E246" s="15" t="n">
+        <v>0.738</v>
+      </c>
+      <c r="F246" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="20" customHeight="1">
+      <c r="A247" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B247" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C247" s="18" t="inlineStr">
+        <is>
+          <t>JUDGE-MY-VOW-QUICKLY</t>
+        </is>
+      </c>
+      <c r="D247" s="19" t="n">
+        <v>0.972</v>
+      </c>
+      <c r="E247" s="19" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="F247" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="20" customHeight="1">
+      <c r="A248" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B248" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C248" s="14" t="inlineStr">
+        <is>
+          <t>BRIGHT-ZEPHYRS-BLOW-</t>
+        </is>
+      </c>
+      <c r="D248" s="15" t="n">
+        <v>0.902</v>
+      </c>
+      <c r="E248" s="15" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="F248" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="20" customHeight="1">
+      <c r="A249" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B249" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C249" s="18" t="inlineStr">
+        <is>
+          <t>COMPUTER-VISION-TEST</t>
+        </is>
+      </c>
+      <c r="D249" s="19" t="n">
+        <v>0.918</v>
+      </c>
+      <c r="E249" s="19" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="F249" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="20" customHeight="1">
+      <c r="A250" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B250" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="C250" s="14" t="inlineStr">
+        <is>
+          <t>MECHINE-LEARNING-AI-</t>
+        </is>
+      </c>
+      <c r="D250" s="15" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="E250" s="15" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="F250" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="20" customHeight="1">
+      <c r="A251" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B251" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C251" s="18" t="inlineStr">
+        <is>
+          <t>DEEP-NEURAL-NETWORKS</t>
+        </is>
+      </c>
+      <c r="D251" s="19" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="E251" s="19" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="F251" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="20" customHeight="1">
+      <c r="A252" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B252" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="C252" s="14" t="inlineStr">
+        <is>
+          <t>IMAGE-OAIA-OETECT-OK</t>
+        </is>
+      </c>
+      <c r="D252" s="15" t="n">
+        <v>0.913</v>
+      </c>
+      <c r="E252" s="15" t="n">
+        <v>0.522</v>
+      </c>
+      <c r="F252" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="20" customHeight="1">
+      <c r="A253" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B253" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C253" s="18" t="inlineStr">
+        <is>
+          <t>PYTHON-OPENCV-ROBOT-</t>
+        </is>
+      </c>
+      <c r="D253" s="19" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="E253" s="19" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F253" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="20" customHeight="1">
+      <c r="A254" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B254" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="C254" s="14" t="inlineStr">
+        <is>
+          <t>SMART-OCR-RECOGNIZE-</t>
+        </is>
+      </c>
+      <c r="D254" s="15" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="E254" s="15" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="F254" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="20" customHeight="1">
+      <c r="A255" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B255" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="C255" s="18" t="inlineStr">
+        <is>
+          <t>ACCURATE-PREDICTION-</t>
+        </is>
+      </c>
+      <c r="D255" s="19" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="E255" s="19" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="F255" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="20" customHeight="1">
+      <c r="A256" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B256" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="C256" s="14" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL-SYSTEM-OK</t>
+        </is>
+      </c>
+      <c r="D256" s="15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E256" s="15" t="n">
+        <v>0.791</v>
+      </c>
+      <c r="F256" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="20" customHeight="1">
+      <c r="A257" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B257" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C257" s="18" t="inlineStr">
+        <is>
+          <t>HELLO-WORLD-WELCOME-</t>
+        </is>
+      </c>
+      <c r="D257" s="19" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="E257" s="19" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="F257" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="20" customHeight="1">
+      <c r="A258" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B258" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="C258" s="14" t="inlineStr">
+        <is>
+          <t>KNOWLEDGE-IS-POWER--</t>
+        </is>
+      </c>
+      <c r="D258" s="15" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="E258" s="15" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="F258" s="20" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="20" customHeight="1">
+      <c r="A259" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B259" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="C259" s="18" t="inlineStr">
+        <is>
+          <t>FIND-EXTRA-FIND-GOLO</t>
+        </is>
+      </c>
+      <c r="D259" s="19" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E259" s="19" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="F259" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="20" customHeight="1">
+      <c r="A260" s="13" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B260" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C260" s="14" t="inlineStr">
+        <is>
+          <t>ZERO-ONE-TWO-SIX-TEN</t>
+        </is>
+      </c>
+      <c r="D260" s="15" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="E260" s="15" t="n">
+        <v>0.697</v>
+      </c>
+      <c r="F260" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="20" customHeight="1">
+      <c r="A261" s="17" t="inlineStr">
+        <is>
+          <t>test13.jpg</t>
+        </is>
+      </c>
+      <c r="B261" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C261" s="18" t="inlineStr">
+        <is>
+          <t>KBCDEFGHIJKLMNOPQRST</t>
+        </is>
+      </c>
+      <c r="D261" s="19" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="E261" s="19" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="F261" s="16" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F241"/>
+  <autoFilter ref="A1:F261"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>